<commit_message>
Atualiza planilha 28/09/2026 (Jan-Jul refeitos pelas notas fiscais, despesas com NF, vendas do dia)
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -50918,16 +50918,36 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="17" t="n"/>
-      <c r="B207" s="18" t="n"/>
-      <c r="C207" s="18" t="n"/>
-      <c r="D207" s="27" t="n"/>
-      <c r="E207" s="18" t="n"/>
+      <c r="A207" s="17" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B207" s="18" t="inlineStr">
+        <is>
+          <t>Verdes Mares Tintas</t>
+        </is>
+      </c>
+      <c r="C207" s="18" t="inlineStr">
+        <is>
+          <t>Limpeza de Refil</t>
+        </is>
+      </c>
+      <c r="D207" s="27" t="n">
+        <v>40</v>
+      </c>
+      <c r="E207" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F207" s="19" t="n"/>
       <c r="G207" s="19" t="n"/>
       <c r="H207" s="21" t="n"/>
       <c r="I207" s="18" t="n"/>
-      <c r="J207" s="18" t="n"/>
+      <c r="J207" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0303</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="44" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 07/10/2026 15:57
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -54576,12 +54576,30 @@
       <c r="J49" s="18" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="44" t="n"/>
-      <c r="B50" s="45" t="n"/>
-      <c r="C50" s="45" t="n"/>
-      <c r="D50" s="46" t="n"/>
-      <c r="E50" s="45" t="n"/>
-      <c r="F50" s="47" t="n"/>
+      <c r="A50" s="44" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B50" s="45" t="inlineStr">
+        <is>
+          <t>Consumidor Final</t>
+        </is>
+      </c>
+      <c r="C50" s="45" t="inlineStr">
+        <is>
+          <t>Refil E3</t>
+        </is>
+      </c>
+      <c r="D50" s="46" t="n">
+        <v>90</v>
+      </c>
+      <c r="E50" s="45" t="inlineStr">
+        <is>
+          <t>Crédito à Vista</t>
+        </is>
+      </c>
+      <c r="F50" s="47" t="n">
+        <v>3.16</v>
+      </c>
       <c r="G50" s="48" t="n"/>
       <c r="H50" s="49" t="n"/>
       <c r="I50" s="45" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 08/10/2026 08:34
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -54605,27 +54605,78 @@
       <c r="I50" s="45" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="n"/>
-      <c r="B51" s="18" t="n"/>
-      <c r="C51" s="18" t="n"/>
-      <c r="D51" s="27" t="n"/>
-      <c r="E51" s="18" t="n"/>
+      <c r="A51" s="17" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>Leonardo de Carvalho Cruz</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Instalação de Purificador + Refil E3</t>
+        </is>
+      </c>
+      <c r="D51" s="27" t="n">
+        <v>130</v>
+      </c>
+      <c r="E51" s="18" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F51" s="19" t="n"/>
       <c r="G51" s="19" t="n"/>
       <c r="H51" s="21" t="n"/>
-      <c r="I51" s="18" t="n"/>
-      <c r="J51" s="18" t="n"/>
+      <c r="I51" s="18" t="inlineStr">
+        <is>
+          <t>Instalação R$ 40,00 + Refil E3 R$ 90,00.</t>
+        </is>
+      </c>
+      <c r="J51" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0902</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="44" t="n"/>
-      <c r="B52" s="45" t="n"/>
-      <c r="C52" s="45" t="n"/>
-      <c r="D52" s="46" t="n"/>
-      <c r="E52" s="45" t="n"/>
-      <c r="F52" s="47" t="n"/>
+      <c r="A52" s="44" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B52" s="45" t="inlineStr">
+        <is>
+          <t>Eliene</t>
+        </is>
+      </c>
+      <c r="C52" s="45" t="inlineStr">
+        <is>
+          <t>Purificador Everest Baby Branco</t>
+        </is>
+      </c>
+      <c r="D52" s="46" t="n">
+        <v>420</v>
+      </c>
+      <c r="E52" s="45" t="inlineStr">
+        <is>
+          <t>Crédito Parcelado</t>
+        </is>
+      </c>
+      <c r="F52" s="47" t="n">
+        <v>33.52</v>
+      </c>
       <c r="G52" s="48" t="n"/>
       <c r="H52" s="49" t="n"/>
-      <c r="I52" s="45" t="n"/>
+      <c r="I52" s="45" t="inlineStr">
+        <is>
+          <t>Parcelado em 6x.</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>CLI-0903</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 08/10/2026 16:40
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -54679,39 +54679,110 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="17" t="n"/>
-      <c r="B53" s="18" t="n"/>
-      <c r="C53" s="18" t="n"/>
-      <c r="D53" s="27" t="n"/>
-      <c r="E53" s="18" t="n"/>
-      <c r="F53" s="19" t="n"/>
+      <c r="A53" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B53" s="18" t="inlineStr">
+        <is>
+          <t>Guiomar Macedo Freire - Antonio vila</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D53" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E53" s="18" t="inlineStr">
+        <is>
+          <t>Crédito Parcelado</t>
+        </is>
+      </c>
+      <c r="F53" s="19" t="n">
+        <v>9.789999999999999</v>
+      </c>
       <c r="G53" s="19" t="n"/>
       <c r="H53" s="21" t="n"/>
-      <c r="I53" s="18" t="n"/>
-      <c r="J53" s="18" t="n"/>
+      <c r="I53" s="18" t="inlineStr">
+        <is>
+          <t>Parcelado em 2x.</t>
+        </is>
+      </c>
+      <c r="J53" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0041</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="44" t="n"/>
-      <c r="B54" s="45" t="n"/>
-      <c r="C54" s="45" t="n"/>
-      <c r="D54" s="46" t="n"/>
-      <c r="E54" s="45" t="n"/>
+      <c r="A54" s="44" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B54" s="45" t="inlineStr">
+        <is>
+          <t>Geisa Cunha Novais - Marcos</t>
+        </is>
+      </c>
+      <c r="C54" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest + Mangueira</t>
+        </is>
+      </c>
+      <c r="D54" s="46" t="n">
+        <v>150</v>
+      </c>
+      <c r="E54" s="45" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F54" s="47" t="n"/>
       <c r="G54" s="48" t="n"/>
       <c r="H54" s="49" t="n"/>
       <c r="I54" s="45" t="n"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>CLI-0270</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="17" t="n"/>
-      <c r="B55" s="18" t="n"/>
-      <c r="C55" s="18" t="n"/>
-      <c r="D55" s="27" t="n"/>
-      <c r="E55" s="18" t="n"/>
+      <c r="A55" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>Chapada Brindes</t>
+        </is>
+      </c>
+      <c r="C55" s="18" t="inlineStr">
+        <is>
+          <t>Purificador Everest Star Branco</t>
+        </is>
+      </c>
+      <c r="D55" s="27" t="n">
+        <v>1379</v>
+      </c>
+      <c r="E55" s="18" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F55" s="19" t="n"/>
       <c r="G55" s="19" t="n"/>
       <c r="H55" s="21" t="n"/>
-      <c r="I55" s="18" t="n"/>
-      <c r="J55" s="18" t="n"/>
+      <c r="I55" s="18" t="inlineStr">
+        <is>
+          <t>Valor da viagem incluso.</t>
+        </is>
+      </c>
+      <c r="J55" s="18" t="inlineStr">
+        <is>
+          <t>OUT-0102</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="44" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 08/10/2026 17:29
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -54785,15 +54785,42 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="44" t="n"/>
-      <c r="B56" s="45" t="n"/>
-      <c r="C56" s="45" t="n"/>
-      <c r="D56" s="46" t="n"/>
-      <c r="E56" s="45" t="n"/>
-      <c r="F56" s="47" t="n"/>
+      <c r="A56" s="44" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B56" s="45" t="inlineStr">
+        <is>
+          <t>Gabriela Araujo</t>
+        </is>
+      </c>
+      <c r="C56" s="45" t="inlineStr">
+        <is>
+          <t>Purificador Everest Fit Prata</t>
+        </is>
+      </c>
+      <c r="D56" s="46" t="n">
+        <v>1486</v>
+      </c>
+      <c r="E56" s="45" t="inlineStr">
+        <is>
+          <t>Crédito Parcelado</t>
+        </is>
+      </c>
+      <c r="F56" s="47" t="n">
+        <v>207.89</v>
+      </c>
       <c r="G56" s="48" t="n"/>
       <c r="H56" s="49" t="n"/>
-      <c r="I56" s="45" t="n"/>
+      <c r="I56" s="45" t="inlineStr">
+        <is>
+          <t>Parcelado em 10x. Instalação na residência (Rua Miguel Guerrera, 92) em 10/10/2026.</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>CLI-0038</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 08/10/2026 18:07
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -54823,61 +54823,141 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="17" t="n"/>
-      <c r="B57" s="18" t="n"/>
+      <c r="A57" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>Faça Feira Supermercado</t>
+        </is>
+      </c>
       <c r="C57" s="18" t="n"/>
       <c r="D57" s="27" t="n"/>
       <c r="E57" s="18" t="n"/>
       <c r="F57" s="19" t="n"/>
-      <c r="G57" s="19" t="n"/>
-      <c r="H57" s="21" t="n"/>
-      <c r="I57" s="18" t="n"/>
+      <c r="G57" s="19" t="n">
+        <v>7.38</v>
+      </c>
+      <c r="H57" s="21" t="inlineStr">
+        <is>
+          <t>Material de Limpeza e Escritório</t>
+        </is>
+      </c>
+      <c r="I57" s="18" t="inlineStr">
+        <is>
+          <t>Copo descartável (Copo Bom) — pago em dinheiro. DAV 790260205.</t>
+        </is>
+      </c>
       <c r="J57" s="18" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="44" t="n"/>
-      <c r="B58" s="45" t="n"/>
+      <c r="A58" s="44" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B58" s="45" t="inlineStr">
+        <is>
+          <t>Conta de Energia Loja</t>
+        </is>
+      </c>
       <c r="C58" s="45" t="n"/>
       <c r="D58" s="46" t="n"/>
       <c r="E58" s="45" t="n"/>
       <c r="F58" s="47" t="n"/>
-      <c r="G58" s="48" t="n"/>
-      <c r="H58" s="49" t="n"/>
-      <c r="I58" s="45" t="n"/>
+      <c r="G58" s="48" t="n">
+        <v>168.56</v>
+      </c>
+      <c r="H58" s="49" t="inlineStr">
+        <is>
+          <t>Água, Energia e Internet</t>
+        </is>
+      </c>
+      <c r="I58" s="45" t="inlineStr">
+        <is>
+          <t>Neoenergia Coelba — ref. 09/2026, venc. 07/10/2026, pago em 08/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="17" t="n"/>
-      <c r="B59" s="18" t="n"/>
+      <c r="A59" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>Eversoft</t>
+        </is>
+      </c>
       <c r="C59" s="18" t="n"/>
       <c r="D59" s="27" t="n"/>
       <c r="E59" s="18" t="n"/>
       <c r="F59" s="19" t="n"/>
-      <c r="G59" s="19" t="n"/>
-      <c r="H59" s="21" t="n"/>
-      <c r="I59" s="18" t="n"/>
+      <c r="G59" s="19" t="n">
+        <v>878.92</v>
+      </c>
+      <c r="H59" s="21" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I59" s="18" t="inlineStr">
+        <is>
+          <t>Boleto Itaú — NF-e 73636 (emissão 10/06/2026), parcela 4/5, vencimento 08/10/2026, pago em 08/10/2026.</t>
+        </is>
+      </c>
       <c r="J59" s="18" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="44" t="n"/>
-      <c r="B60" s="45" t="n"/>
+      <c r="A60" s="44" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B60" s="45" t="inlineStr">
+        <is>
+          <t>Filtros Planeta Água</t>
+        </is>
+      </c>
       <c r="C60" s="45" t="n"/>
       <c r="D60" s="46" t="n"/>
       <c r="E60" s="45" t="n"/>
       <c r="F60" s="47" t="n"/>
-      <c r="G60" s="48" t="n"/>
-      <c r="H60" s="49" t="n"/>
-      <c r="I60" s="45" t="n"/>
+      <c r="G60" s="48" t="n">
+        <v>500.81</v>
+      </c>
+      <c r="H60" s="49" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I60" s="45" t="inlineStr">
+        <is>
+          <t>NF 133812 parcela 2 — boleto Itaú. Venc. 09/10/2026, pago antecipado em 08/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="17" t="n"/>
-      <c r="B61" s="18" t="n"/>
+      <c r="A61" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>Crédito Celular da Loja</t>
+        </is>
+      </c>
       <c r="C61" s="18" t="n"/>
       <c r="D61" s="27" t="n"/>
       <c r="E61" s="18" t="n"/>
       <c r="F61" s="19" t="n"/>
-      <c r="G61" s="19" t="n"/>
-      <c r="H61" s="21" t="n"/>
-      <c r="I61" s="18" t="n"/>
+      <c r="G61" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="H61" s="21" t="inlineStr">
+        <is>
+          <t>Outras Despesas</t>
+        </is>
+      </c>
+      <c r="I61" s="18" t="inlineStr">
+        <is>
+          <t>Recarga Claro (74) 98858-2298 via RecargaPay na Drogaria Mais Farma — ID 000074730.</t>
+        </is>
+      </c>
       <c r="J61" s="18" t="n"/>
     </row>
     <row r="62">
@@ -66352,7 +66432,7 @@
       </c>
       <c r="E31" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F31" s="112">
@@ -66361,7 +66441,7 @@
       </c>
       <c r="G31" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/24142201-6. Linha digitável 34191.12242 14220.160304 55679.010003 7 15930000087892. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 73636 (emissão 10/06/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.394,61 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260608782043000188550060000736361998873394.</t>
+          <t>Categoria: Fornecedores / Mercadoria. Pago em 08/10/2026 — lançado em Out 2026 como "Eversoft". Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/24142201-6. Linha digitável 34191.12242 14220.160304 55679.010003 7 15930000087892. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 73636 (emissão 10/06/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.394,61 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260608782043000188550060000736361998873394.</t>
         </is>
       </c>
     </row>
@@ -67632,7 +67712,7 @@
       </c>
       <c r="E71" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F71" s="113">
@@ -67641,7 +67721,7 @@
       </c>
       <c r="G71" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/153155. Nosso número 109/00259099-8. Linha digitável 34191.09008 25909.981430 81531.550002 7 15940000050081. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133812 (emissão 28/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.093,55 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora JAMEF TRANSPORTES LIMITADA. Chave da NF-e 43260805097806000163550010001338121014276984.</t>
+          <t>Categoria: Fornecedores / Mercadoria. Pago em 08/10/2026 — lançado em Out 2026 como "Filtros Planeta Água". Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/153155. Nosso número 109/00259099-8. Linha digitável 34191.09008 25909.981430 81531.550002 7 15940000050081. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133812 (emissão 28/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.093,55 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora JAMEF TRANSPORTES LIMITADA. Chave da NF-e 43260805097806000163550010001338121014276984.</t>
         </is>
       </c>
     </row>
@@ -68336,7 +68416,7 @@
       </c>
       <c r="E93" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F93" s="113">
@@ -68345,7 +68425,7 @@
       </c>
       <c r="G93" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Água, Energia e Internet. Fatura em nome de Vitoria Maria de Freitas Santos (Rua Manoel Novaes, 263, SL-3 — a loja), UC 7.908.588.028-80, NF 996962199, consumo 125 kWh (27/08 a 28/09/2026), bandeira amarela. Boleto Itaú 341. Linha digitável (conferida no PDF da fatura): 34191.75215 02379.112937 85832.220009 3 15920000016856. PDF salvo em "boletos planeta agua/Coelba Loja - venc 07-10-2026.pdf". Código para débito automático: 7044847005.</t>
+          <t>Categoria: Água, Energia e Internet. Pago em 08/10/2026 — lançado em Out 2026 como "Conta de Energia Loja". Fatura em nome de Vitoria Maria de Freitas Santos (Rua Manoel Novaes, 263, SL-3 — a loja), UC 7.908.588.028-80, NF 996962199, consumo 125 kWh (27/08 a 28/09/2026), bandeira amarela. Boleto Itaú 341. Linha digitável (conferida no PDF da fatura): 34191.75215 02379.112937 85832.220009 3 15920000016856. PDF salvo em "boletos planeta agua/Coelba Loja - venc 07-10-2026.pdf". Código para débito automático: 7044847005.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao do painel - 09/10/2026 11:57
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -54961,50 +54961,150 @@
       <c r="J61" s="18" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="44" t="n"/>
-      <c r="B62" s="45" t="n"/>
-      <c r="C62" s="45" t="n"/>
-      <c r="D62" s="46" t="n"/>
-      <c r="E62" s="45" t="n"/>
+      <c r="A62" s="44" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B62" s="45" t="inlineStr">
+        <is>
+          <t>Rafael Landin Ribeiro</t>
+        </is>
+      </c>
+      <c r="C62" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D62" s="46" t="n">
+        <v>140</v>
+      </c>
+      <c r="E62" s="45" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F62" s="47" t="n"/>
       <c r="G62" s="48" t="n"/>
       <c r="H62" s="49" t="n"/>
-      <c r="I62" s="45" t="n"/>
+      <c r="I62" s="45" t="inlineStr">
+        <is>
+          <t>Troca do dia 09/10/2026.</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>CLI-0530</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="17" t="n"/>
-      <c r="B63" s="18" t="n"/>
-      <c r="C63" s="18" t="n"/>
-      <c r="D63" s="27" t="n"/>
-      <c r="E63" s="18" t="n"/>
-      <c r="F63" s="19" t="n"/>
+      <c r="A63" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>Refil Pro Life + Refil Universal</t>
+        </is>
+      </c>
+      <c r="D63" s="27" t="n">
+        <v>85</v>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Débito</t>
+        </is>
+      </c>
+      <c r="F63" s="19" t="n">
+        <v>1.23</v>
+      </c>
       <c r="G63" s="19" t="n"/>
       <c r="H63" s="21" t="n"/>
-      <c r="I63" s="18" t="n"/>
-      <c r="J63" s="18" t="n"/>
+      <c r="I63" s="18" t="inlineStr">
+        <is>
+          <t>Venda total R$ 170,00 (Refil Pro Life R$ 140,00 + Refil Universal R$ 30,00) — pagamento dividido: R$ 85,00 no débito em 09/10/2026 + R$ 85,00 via Pix (linha abaixo).</t>
+        </is>
+      </c>
+      <c r="J63" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0258</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="44" t="n"/>
-      <c r="B64" s="45" t="n"/>
-      <c r="C64" s="45" t="n"/>
-      <c r="D64" s="46" t="n"/>
-      <c r="E64" s="45" t="n"/>
+      <c r="A64" s="44" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B64" s="45" t="inlineStr">
+        <is>
+          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
+        </is>
+      </c>
+      <c r="C64" s="45" t="inlineStr">
+        <is>
+          <t>(Mesma venda acima — 2ª forma de pagamento, sem produtos novos)</t>
+        </is>
+      </c>
+      <c r="D64" s="46" t="n">
+        <v>85</v>
+      </c>
+      <c r="E64" s="45" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F64" s="47" t="n"/>
       <c r="G64" s="48" t="n"/>
       <c r="H64" s="49" t="n"/>
-      <c r="I64" s="45" t="n"/>
+      <c r="I64" s="45" t="inlineStr">
+        <is>
+          <t>Restante da venda de R$ 170,00 — Pix previsto para sexta 16/10/2026.</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>EMP-0258</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="17" t="n"/>
-      <c r="B65" s="18" t="n"/>
-      <c r="C65" s="18" t="n"/>
-      <c r="D65" s="27" t="n"/>
-      <c r="E65" s="18" t="n"/>
+      <c r="A65" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t>Tropical Motos LTDA</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>Refil Pro Life</t>
+        </is>
+      </c>
+      <c r="D65" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F65" s="19" t="n"/>
       <c r="G65" s="19" t="n"/>
       <c r="H65" s="21" t="n"/>
-      <c r="I65" s="18" t="n"/>
-      <c r="J65" s="18" t="n"/>
+      <c r="I65" s="18" t="inlineStr">
+        <is>
+          <t>Troca do dia 09/10/2026 — purificador do andar de cima (Pro Life, sem pré-filtro).</t>
+        </is>
+      </c>
+      <c r="J65" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0296</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="44" t="n"/>
@@ -65666,7 +65766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G157"/>
+  <dimension ref="A1:I163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="157" min="1" max="1"/>
@@ -70187,45 +70287,138 @@
       </c>
     </row>
     <row r="154" s="157">
-      <c r="A154" s="86" t="inlineStr">
+      <c r="A154" s="78" t="inlineStr">
+        <is>
+          <t>Rafael Landin Ribeiro</t>
+        </is>
+      </c>
+      <c r="B154" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="C154" s="77" t="n">
+        <v>46304</v>
+      </c>
+      <c r="D154" s="79" t="n">
+        <v>140</v>
+      </c>
+      <c r="E154" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F154" s="112">
+        <f>IF(OR($E154="Recebido",$C154=""),"",MAX(0,TODAY()-$C154))</f>
+        <v/>
+      </c>
+      <c r="G154" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 09/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" s="157">
+      <c r="A155" s="78" t="inlineStr">
+        <is>
+          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
+        </is>
+      </c>
+      <c r="B155" s="78" t="inlineStr">
+        <is>
+          <t>Refil Pro Life + Refil Universal (restante)</t>
+        </is>
+      </c>
+      <c r="C155" s="77" t="n">
+        <v>46304</v>
+      </c>
+      <c r="D155" s="79" t="n">
+        <v>85</v>
+      </c>
+      <c r="E155" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F155" s="112">
+        <f>IF(OR($E155="Recebido",$C155=""),"",MAX(0,TODAY()-$C155))</f>
+        <v/>
+      </c>
+      <c r="G155" s="78" t="inlineStr">
+        <is>
+          <t>Venda de R$ 170,00 — R$ 85,00 pagos no débito em 09/10/2026; restante via Pix previsto para 16/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" s="157">
+      <c r="A156" s="78" t="inlineStr">
+        <is>
+          <t>Tropical Motos LTDA</t>
+        </is>
+      </c>
+      <c r="B156" s="78" t="inlineStr">
+        <is>
+          <t>Refil Pro Life</t>
+        </is>
+      </c>
+      <c r="C156" s="77" t="n">
+        <v>46304</v>
+      </c>
+      <c r="D156" s="79" t="n">
+        <v>140</v>
+      </c>
+      <c r="E156" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F156" s="112">
+        <f>IF(OR($E156="Recebido",$C156=""),"",MAX(0,TODAY()-$C156))</f>
+        <v/>
+      </c>
+      <c r="G156" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 09/10/2026 — purificador do andar de cima.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" s="157">
+      <c r="A157" s="86" t="inlineStr">
         <is>
           <t>TOTAL EM ABERTO A RECEBER (detalhe)</t>
         </is>
       </c>
-      <c r="D154" s="115">
-        <f>SUMIF(E102:E153,"Pendente",D102:D153)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="155" s="157">
-      <c r="A155" s="202" t="inlineStr">
+      <c r="D157" s="115">
+        <f>SUMIF(E102:E156,"Pendente",D102:D156)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158" s="157">
+      <c r="A158" s="202" t="inlineStr">
         <is>
           <t>CONFERÊNCIA COM AS ABAS DOS MESES</t>
         </is>
       </c>
-      <c r="B155" s="159" t="n"/>
-      <c r="C155" s="159" t="n"/>
-      <c r="D155" s="159" t="n"/>
-      <c r="E155" s="159" t="n"/>
-      <c r="F155" s="159" t="n"/>
-      <c r="G155" s="160" t="n"/>
-    </row>
-    <row r="156" s="157">
-      <c r="A156" s="203">
-        <f>IF(ROUND(D154-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D154-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="157" s="157">
-      <c r="A157" s="203" t="inlineStr">
+      <c r="B158" s="159" t="n"/>
+      <c r="C158" s="159" t="n"/>
+      <c r="D158" s="159" t="n"/>
+      <c r="E158" s="159" t="n"/>
+      <c r="F158" s="159" t="n"/>
+      <c r="G158" s="160" t="n"/>
+    </row>
+    <row r="159" s="157">
+      <c r="A159" s="203">
+        <f>IF(ROUND(D157-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D157-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="160" s="157">
+      <c r="A160" s="203" t="inlineStr">
         <is>
           <t>As contas a pagar do DigiSat (pendentes até 27/07/2026) foram todas quitadas — confirmado em 19/08/2026. A única dívida em aberto hoje é o Capital de Giro do Banco do Brasil. Lance aqui novos compromissos conforme surgirem.</t>
         </is>
       </c>
     </row>
-    <row r="158" s="157"/>
-    <row r="159" s="157"/>
-    <row r="160" s="157"/>
     <row r="161" s="157"/>
     <row r="162" s="157"/>
     <row r="163" s="157"/>
@@ -70274,23 +70467,23 @@
   <mergeCells count="13">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="E4:F4"/>
+    <mergeCell ref="A159:G159"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A158:G158"/>
     <mergeCell ref="A100:G100"/>
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="A5:B6"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E5:F6"/>
-    <mergeCell ref="A156:G156"/>
     <mergeCell ref="A99:G99"/>
-    <mergeCell ref="A155:G155"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="E11:E93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Pago,Previsto"</formula1>
     </dataValidation>
-    <dataValidation sqref="E102:E153" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E102:E156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Recebido"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Atualizacao do painel - 09/10/2026 15:00
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -54513,7 +54513,7 @@
     </row>
     <row r="48">
       <c r="A48" s="44" t="n">
-        <v>46301</v>
+        <v>46296</v>
       </c>
       <c r="B48" s="45" t="inlineStr">
         <is>
@@ -54538,7 +54538,7 @@
       <c r="H48" s="49" t="n"/>
       <c r="I48" s="45" t="inlineStr">
         <is>
-          <t>Venda de 30/09/2026 (troca na PC Jacobina / Cartão de Todos, antes em Set 2026) — pagamento recebido via Pix em 06/10/2026.</t>
+          <t>Venda de 30/09/2026 (troca na PC Jacobina / Cartão de Todos, antes em Set 2026) — pagamento recebido via Pix em 01/10/2026 (comprovante enviado em 06/10/2026).</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -54979,7 +54979,7 @@
       </c>
       <c r="E62" s="45" t="inlineStr">
         <is>
-          <t>Aguardando Pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F62" s="47" t="n"/>
@@ -54987,7 +54987,7 @@
       <c r="H62" s="49" t="n"/>
       <c r="I62" s="45" t="inlineStr">
         <is>
-          <t>Troca do dia 09/10/2026.</t>
+          <t>Troca do dia 09/10/2026 — pagamento recebido via Pix em 09/10/2026.</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -55107,15 +55107,31 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="44" t="n"/>
-      <c r="B66" s="45" t="n"/>
+      <c r="A66" s="44" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B66" s="45" t="inlineStr">
+        <is>
+          <t>Estacionamento (Zona Azul)</t>
+        </is>
+      </c>
       <c r="C66" s="45" t="n"/>
       <c r="D66" s="46" t="n"/>
       <c r="E66" s="45" t="n"/>
       <c r="F66" s="47" t="n"/>
-      <c r="G66" s="48" t="n"/>
-      <c r="H66" s="49" t="n"/>
-      <c r="I66" s="45" t="n"/>
+      <c r="G66" s="48" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H66" s="49" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I66" s="45" t="inlineStr">
+        <is>
+          <t>Mob Parking — Zona Azul Digital Jacobina, ticket 210571, 09/10/2026 12:00–13:00, placa PLR9I12. Se aparecer Pix de R$ 2,40 para Pagar.me no extrato deste dia, é este mesmo — não lançar de novo.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="17" t="n"/>
@@ -65766,7 +65782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I163"/>
+  <dimension ref="A1:G160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="157" min="1" max="1"/>
@@ -70154,7 +70170,7 @@
       </c>
       <c r="G149" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 30/09/2026. Recebido via Pix em 06/10/2026 — lançado em "Out 2026".</t>
+          <t>Troca do dia 30/09/2026. Recebido via Pix em 01/10/2026 (comprovante enviado em 06/10/2026) — lançado em "Out 2026".</t>
         </is>
       </c>
     </row>
@@ -70305,7 +70321,7 @@
       </c>
       <c r="E154" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F154" s="112">
@@ -70314,7 +70330,7 @@
       </c>
       <c r="G154" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 09/10/2026.</t>
+          <t>Troca do dia 09/10/2026. Recebido via Pix em 09/10/2026.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao do painel - 10/10/2026 09:33
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -55134,27 +55134,74 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="17" t="n"/>
-      <c r="B67" s="18" t="n"/>
-      <c r="C67" s="18" t="n"/>
-      <c r="D67" s="27" t="n"/>
-      <c r="E67" s="18" t="n"/>
+      <c r="A67" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>Colegio Oasis de Jacobina - Unopar</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="inlineStr">
+        <is>
+          <t>2x Refil Plissado + 2x Carcaça 9"</t>
+        </is>
+      </c>
+      <c r="D67" s="27" t="n">
+        <v>400</v>
+      </c>
+      <c r="E67" s="18" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F67" s="19" t="n"/>
       <c r="G67" s="19" t="n"/>
       <c r="H67" s="21" t="n"/>
-      <c r="I67" s="18" t="n"/>
-      <c r="J67" s="18" t="n"/>
+      <c r="I67" s="18" t="inlineStr">
+        <is>
+          <t>2x Refil Plissado R$ 80,00 cada + 2x Carcaça 9" R$ 120,00 cada. Cláudio assinou para pagar depois. Falta enviar a NF.</t>
+        </is>
+      </c>
+      <c r="J67" s="18" t="inlineStr">
+        <is>
+          <t>ESC-0009</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="44" t="n"/>
-      <c r="B68" s="45" t="n"/>
-      <c r="C68" s="45" t="n"/>
-      <c r="D68" s="46" t="n"/>
-      <c r="E68" s="45" t="n"/>
-      <c r="F68" s="47" t="n"/>
+      <c r="A68" s="44" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B68" s="45" t="inlineStr">
+        <is>
+          <t>Josélia Nascimento da Silva Gomes</t>
+        </is>
+      </c>
+      <c r="C68" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D68" s="46" t="n">
+        <v>140</v>
+      </c>
+      <c r="E68" s="45" t="inlineStr">
+        <is>
+          <t>Crédito à Vista</t>
+        </is>
+      </c>
+      <c r="F68" s="47" t="n">
+        <v>4.91</v>
+      </c>
       <c r="G68" s="48" t="n"/>
       <c r="H68" s="49" t="n"/>
       <c r="I68" s="45" t="n"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>CLI-0313</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 10/10/2026 12:37
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -55204,46 +55204,137 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="17" t="n"/>
-      <c r="B69" s="18" t="n"/>
-      <c r="C69" s="18" t="n"/>
-      <c r="D69" s="27" t="n"/>
-      <c r="E69" s="18" t="n"/>
+      <c r="A69" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B69" s="18" t="inlineStr">
+        <is>
+          <t>Gabriela Araujo</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>Conexão T Everest</t>
+        </is>
+      </c>
+      <c r="D69" s="27" t="n">
+        <v>30</v>
+      </c>
+      <c r="E69" s="18" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F69" s="19" t="n"/>
       <c r="G69" s="19" t="n"/>
       <c r="H69" s="21" t="n"/>
-      <c r="I69" s="18" t="n"/>
-      <c r="J69" s="18" t="n"/>
+      <c r="I69" s="18" t="inlineStr">
+        <is>
+          <t>Peça usada na instalação do Purificador Everest Fit Prata (comprado em 08/10/2026).</t>
+        </is>
+      </c>
+      <c r="J69" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0038</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="44" t="n"/>
-      <c r="B70" s="45" t="n"/>
-      <c r="C70" s="45" t="n"/>
-      <c r="D70" s="46" t="n"/>
-      <c r="E70" s="45" t="n"/>
-      <c r="F70" s="47" t="n"/>
+      <c r="A70" s="44" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B70" s="45" t="inlineStr">
+        <is>
+          <t>Michelle Santos de Almeida Rocha</t>
+        </is>
+      </c>
+      <c r="C70" s="45" t="inlineStr">
+        <is>
+          <t>Purificador Everest Foz Grafite</t>
+        </is>
+      </c>
+      <c r="D70" s="46" t="n">
+        <v>1689</v>
+      </c>
+      <c r="E70" s="45" t="inlineStr">
+        <is>
+          <t>Crédito Parcelado</t>
+        </is>
+      </c>
+      <c r="F70" s="47" t="n">
+        <v>236.29</v>
+      </c>
       <c r="G70" s="48" t="n"/>
       <c r="H70" s="49" t="n"/>
-      <c r="I70" s="45" t="n"/>
+      <c r="I70" s="45" t="inlineStr">
+        <is>
+          <t>Crédito em 10x. Instalação feita em 10/10/2026.</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>CLI-0904</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="17" t="n"/>
-      <c r="B71" s="18" t="n"/>
-      <c r="C71" s="18" t="n"/>
-      <c r="D71" s="27" t="n"/>
-      <c r="E71" s="18" t="n"/>
+      <c r="A71" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>Michelle Santos de Almeida Rocha</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D71" s="27" t="n">
+        <v>60</v>
+      </c>
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F71" s="19" t="n"/>
       <c r="G71" s="19" t="n"/>
       <c r="H71" s="21" t="n"/>
-      <c r="I71" s="18" t="n"/>
-      <c r="J71" s="18" t="n"/>
+      <c r="I71" s="18" t="inlineStr">
+        <is>
+          <t>Oferecido e vendido na hora da instalação do purificador.</t>
+        </is>
+      </c>
+      <c r="J71" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0904</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="44" t="n"/>
-      <c r="B72" s="45" t="n"/>
-      <c r="C72" s="45" t="n"/>
-      <c r="D72" s="46" t="n"/>
-      <c r="E72" s="45" t="n"/>
+      <c r="A72" s="44" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B72" s="45" t="inlineStr">
+        <is>
+          <t>Consumidor Final</t>
+        </is>
+      </c>
+      <c r="C72" s="45" t="inlineStr">
+        <is>
+          <t>Refil Universal</t>
+        </is>
+      </c>
+      <c r="D72" s="46" t="n">
+        <v>30</v>
+      </c>
+      <c r="E72" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F72" s="47" t="n"/>
       <c r="G72" s="48" t="n"/>
       <c r="H72" s="49" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 13/10/2026 14:46
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -55341,27 +55341,70 @@
       <c r="I72" s="45" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="17" t="n"/>
-      <c r="B73" s="18" t="n"/>
-      <c r="C73" s="18" t="n"/>
-      <c r="D73" s="27" t="n"/>
-      <c r="E73" s="18" t="n"/>
+      <c r="A73" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>Leonardo Silva de Brito</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest + Mangueira + Limpeza do Purificador</t>
+        </is>
+      </c>
+      <c r="D73" s="27" t="n">
+        <v>170</v>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F73" s="19" t="n"/>
       <c r="G73" s="19" t="n"/>
       <c r="H73" s="21" t="n"/>
       <c r="I73" s="18" t="n"/>
-      <c r="J73" s="18" t="n"/>
+      <c r="J73" s="18" t="inlineStr">
+        <is>
+          <t>OUT-0103</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="44" t="n"/>
-      <c r="B74" s="45" t="n"/>
-      <c r="C74" s="45" t="n"/>
-      <c r="D74" s="46" t="n"/>
-      <c r="E74" s="45" t="n"/>
-      <c r="F74" s="47" t="n"/>
+      <c r="A74" s="44" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B74" s="45" t="inlineStr">
+        <is>
+          <t>Lorena Coelho</t>
+        </is>
+      </c>
+      <c r="C74" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D74" s="46" t="n">
+        <v>200</v>
+      </c>
+      <c r="E74" s="45" t="inlineStr">
+        <is>
+          <t>Débito</t>
+        </is>
+      </c>
+      <c r="F74" s="47" t="n">
+        <v>5.28</v>
+      </c>
       <c r="G74" s="48" t="n"/>
       <c r="H74" s="49" t="n"/>
       <c r="I74" s="45" t="n"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>CLI-0905</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 13/10/2026 17:24
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -55407,211 +55407,499 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="17" t="n"/>
-      <c r="B75" s="18" t="n"/>
+      <c r="A75" s="17" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>Estacionamento (Pagar.me)</t>
+        </is>
+      </c>
       <c r="C75" s="18" t="n"/>
       <c r="D75" s="27" t="n"/>
       <c r="E75" s="18" t="n"/>
       <c r="F75" s="19" t="n"/>
-      <c r="G75" s="19" t="n"/>
-      <c r="H75" s="21" t="n"/>
-      <c r="I75" s="18" t="n"/>
+      <c r="G75" s="19" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H75" s="21" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I75" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — Pix de 01/10/2026 para Pagar.me Instituição de Pagamento (estacionamento).</t>
+        </is>
+      </c>
       <c r="J75" s="18" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="44" t="n"/>
-      <c r="B76" s="45" t="n"/>
+      <c r="A76" s="44" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B76" s="45" t="inlineStr">
+        <is>
+          <t>Thiago de Jesus Nascimento</t>
+        </is>
+      </c>
       <c r="C76" s="45" t="n"/>
       <c r="D76" s="46" t="n"/>
       <c r="E76" s="45" t="n"/>
       <c r="F76" s="47" t="n"/>
-      <c r="G76" s="48" t="n"/>
-      <c r="H76" s="49" t="n"/>
-      <c r="I76" s="45" t="n"/>
+      <c r="G76" s="48" t="n">
+        <v>35</v>
+      </c>
+      <c r="H76" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I76" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 01/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="17" t="n"/>
-      <c r="B77" s="18" t="n"/>
+      <c r="A77" s="17" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>Maria Eva dos Santos</t>
+        </is>
+      </c>
       <c r="C77" s="18" t="n"/>
       <c r="D77" s="27" t="n"/>
       <c r="E77" s="18" t="n"/>
       <c r="F77" s="19" t="n"/>
-      <c r="G77" s="19" t="n"/>
-      <c r="H77" s="21" t="n"/>
-      <c r="I77" s="18" t="n"/>
+      <c r="G77" s="19" t="n">
+        <v>380</v>
+      </c>
+      <c r="H77" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I77" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 02/10/2026.</t>
+        </is>
+      </c>
       <c r="J77" s="18" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="44" t="n"/>
-      <c r="B78" s="45" t="n"/>
+      <c r="A78" s="44" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B78" s="45" t="inlineStr">
+        <is>
+          <t>Cezar Silva Atacado e Varejo (Iene Quedila Nunes Dourado)</t>
+        </is>
+      </c>
       <c r="C78" s="45" t="n"/>
       <c r="D78" s="46" t="n"/>
       <c r="E78" s="45" t="n"/>
       <c r="F78" s="47" t="n"/>
-      <c r="G78" s="48" t="n"/>
-      <c r="H78" s="49" t="n"/>
-      <c r="I78" s="45" t="n"/>
+      <c r="G78" s="48" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="H78" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I78" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 02/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="17" t="n"/>
-      <c r="B79" s="18" t="n"/>
+      <c r="A79" s="17" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t>Estacionamento (Pagar.me)</t>
+        </is>
+      </c>
       <c r="C79" s="18" t="n"/>
       <c r="D79" s="27" t="n"/>
       <c r="E79" s="18" t="n"/>
       <c r="F79" s="19" t="n"/>
-      <c r="G79" s="19" t="n"/>
-      <c r="H79" s="21" t="n"/>
-      <c r="I79" s="18" t="n"/>
+      <c r="G79" s="19" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H79" s="21" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I79" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — Pix de 02/10/2026 para Pagar.me Instituição de Pagamento (estacionamento).</t>
+        </is>
+      </c>
       <c r="J79" s="18" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="44" t="n"/>
-      <c r="B80" s="45" t="n"/>
+      <c r="A80" s="44" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B80" s="45" t="inlineStr">
+        <is>
+          <t>Japedido Software</t>
+        </is>
+      </c>
       <c r="C80" s="45" t="n"/>
       <c r="D80" s="46" t="n"/>
       <c r="E80" s="45" t="n"/>
       <c r="F80" s="47" t="n"/>
-      <c r="G80" s="48" t="n"/>
-      <c r="H80" s="49" t="n"/>
-      <c r="I80" s="45" t="n"/>
+      <c r="G80" s="48" t="n">
+        <v>48.49</v>
+      </c>
+      <c r="H80" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I80" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 07/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="17" t="n"/>
-      <c r="B81" s="18" t="n"/>
+      <c r="A81" s="17" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t>Thiago de Jesus Nascimento</t>
+        </is>
+      </c>
       <c r="C81" s="18" t="n"/>
       <c r="D81" s="27" t="n"/>
       <c r="E81" s="18" t="n"/>
       <c r="F81" s="19" t="n"/>
-      <c r="G81" s="19" t="n"/>
-      <c r="H81" s="21" t="n"/>
-      <c r="I81" s="18" t="n"/>
+      <c r="G81" s="19" t="n">
+        <v>28</v>
+      </c>
+      <c r="H81" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I81" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 08/10/2026.</t>
+        </is>
+      </c>
       <c r="J81" s="18" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="44" t="n"/>
-      <c r="B82" s="45" t="n"/>
+      <c r="A82" s="44" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B82" s="45" t="inlineStr">
+        <is>
+          <t>Estacionamento (Pagar.me)</t>
+        </is>
+      </c>
       <c r="C82" s="45" t="n"/>
       <c r="D82" s="46" t="n"/>
       <c r="E82" s="45" t="n"/>
       <c r="F82" s="47" t="n"/>
-      <c r="G82" s="48" t="n"/>
-      <c r="H82" s="49" t="n"/>
-      <c r="I82" s="45" t="n"/>
+      <c r="G82" s="48" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H82" s="49" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I82" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — Pix de 08/10/2026 para Pagar.me Instituição de Pagamento (estacionamento). Diferente do Zona Azul de 09/10.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="17" t="n"/>
-      <c r="B83" s="18" t="n"/>
+      <c r="A83" s="17" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t>Marcos Pereira Cirqueira</t>
+        </is>
+      </c>
       <c r="C83" s="18" t="n"/>
       <c r="D83" s="27" t="n"/>
       <c r="E83" s="18" t="n"/>
       <c r="F83" s="19" t="n"/>
-      <c r="G83" s="19" t="n"/>
-      <c r="H83" s="21" t="n"/>
-      <c r="I83" s="18" t="n"/>
+      <c r="G83" s="19" t="n">
+        <v>54</v>
+      </c>
+      <c r="H83" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I83" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 09/10/2026.</t>
+        </is>
+      </c>
       <c r="J83" s="18" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="44" t="n"/>
-      <c r="B84" s="45" t="n"/>
+      <c r="A84" s="44" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B84" s="45" t="inlineStr">
+        <is>
+          <t>Ledson Batista da Silva</t>
+        </is>
+      </c>
       <c r="C84" s="45" t="n"/>
       <c r="D84" s="46" t="n"/>
       <c r="E84" s="45" t="n"/>
       <c r="F84" s="47" t="n"/>
-      <c r="G84" s="48" t="n"/>
-      <c r="H84" s="49" t="n"/>
-      <c r="I84" s="45" t="n"/>
+      <c r="G84" s="48" t="n">
+        <v>120</v>
+      </c>
+      <c r="H84" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I84" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 09/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="17" t="n"/>
-      <c r="B85" s="18" t="n"/>
+      <c r="A85" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t>App 99 — reembolso Wiliam</t>
+        </is>
+      </c>
       <c r="C85" s="18" t="n"/>
       <c r="D85" s="27" t="n"/>
       <c r="E85" s="18" t="n"/>
       <c r="F85" s="19" t="n"/>
-      <c r="G85" s="19" t="n"/>
-      <c r="H85" s="21" t="n"/>
-      <c r="I85" s="18" t="n"/>
+      <c r="G85" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H85" s="21" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I85" s="18" t="inlineStr">
+        <is>
+          <t>Pix para Wiliam Pinto Bispo em 10/10/2026 — reembolso de corridas no 99 para fazer serviços (Extrato Stone).</t>
+        </is>
+      </c>
       <c r="J85" s="18" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="44" t="n"/>
-      <c r="B86" s="45" t="n"/>
+      <c r="A86" s="44" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B86" s="45" t="inlineStr">
+        <is>
+          <t>Dlocal Brasil Instituição de Pagamento</t>
+        </is>
+      </c>
       <c r="C86" s="45" t="n"/>
       <c r="D86" s="46" t="n"/>
       <c r="E86" s="45" t="n"/>
       <c r="F86" s="47" t="n"/>
-      <c r="G86" s="48" t="n"/>
-      <c r="H86" s="49" t="n"/>
-      <c r="I86" s="45" t="n"/>
+      <c r="G86" s="48" t="n">
+        <v>144.61</v>
+      </c>
+      <c r="H86" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I86" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 10/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="17" t="n"/>
-      <c r="B87" s="18" t="n"/>
+      <c r="A87" s="17" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t>Mercado Pago (Pix Marketplace)</t>
+        </is>
+      </c>
       <c r="C87" s="18" t="n"/>
       <c r="D87" s="27" t="n"/>
       <c r="E87" s="18" t="n"/>
       <c r="F87" s="19" t="n"/>
-      <c r="G87" s="19" t="n"/>
-      <c r="H87" s="21" t="n"/>
-      <c r="I87" s="18" t="n"/>
+      <c r="G87" s="19" t="n">
+        <v>69.03</v>
+      </c>
+      <c r="H87" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I87" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 10/10/2026.</t>
+        </is>
+      </c>
       <c r="J87" s="18" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="44" t="n"/>
-      <c r="B88" s="45" t="n"/>
+      <c r="A88" s="44" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B88" s="45" t="inlineStr">
+        <is>
+          <t>Janaina dos Santos</t>
+        </is>
+      </c>
       <c r="C88" s="45" t="n"/>
       <c r="D88" s="46" t="n"/>
       <c r="E88" s="45" t="n"/>
       <c r="F88" s="47" t="n"/>
-      <c r="G88" s="48" t="n"/>
-      <c r="H88" s="49" t="n"/>
-      <c r="I88" s="45" t="n"/>
+      <c r="G88" s="48" t="n">
+        <v>61.89</v>
+      </c>
+      <c r="H88" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I88" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 10/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="17" t="n"/>
-      <c r="B89" s="18" t="n"/>
+      <c r="A89" s="17" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t>Maree Instituição de Pagamento</t>
+        </is>
+      </c>
       <c r="C89" s="18" t="n"/>
       <c r="D89" s="27" t="n"/>
       <c r="E89" s="18" t="n"/>
       <c r="F89" s="19" t="n"/>
-      <c r="G89" s="19" t="n"/>
-      <c r="H89" s="21" t="n"/>
-      <c r="I89" s="18" t="n"/>
+      <c r="G89" s="19" t="n">
+        <v>86.84999999999999</v>
+      </c>
+      <c r="H89" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I89" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 12/10/2026.</t>
+        </is>
+      </c>
       <c r="J89" s="18" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="44" t="n"/>
-      <c r="B90" s="45" t="n"/>
+      <c r="A90" s="44" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B90" s="45" t="inlineStr">
+        <is>
+          <t>Estacionamento (Pagar.me)</t>
+        </is>
+      </c>
       <c r="C90" s="45" t="n"/>
       <c r="D90" s="46" t="n"/>
       <c r="E90" s="45" t="n"/>
       <c r="F90" s="47" t="n"/>
-      <c r="G90" s="48" t="n"/>
-      <c r="H90" s="49" t="n"/>
-      <c r="I90" s="45" t="n"/>
+      <c r="G90" s="48" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H90" s="49" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I90" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — Pix de 13/10/2026 para Pagar.me Instituição de Pagamento (estacionamento).</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="17" t="n"/>
-      <c r="B91" s="18" t="n"/>
+      <c r="A91" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t>N de Souza Oliveira Ltda</t>
+        </is>
+      </c>
       <c r="C91" s="18" t="n"/>
       <c r="D91" s="27" t="n"/>
       <c r="E91" s="18" t="n"/>
       <c r="F91" s="19" t="n"/>
-      <c r="G91" s="19" t="n"/>
-      <c r="H91" s="21" t="n"/>
-      <c r="I91" s="18" t="n"/>
+      <c r="G91" s="19" t="n">
+        <v>21</v>
+      </c>
+      <c r="H91" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I91" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 13/10/2026.</t>
+        </is>
+      </c>
       <c r="J91" s="18" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="44" t="n"/>
-      <c r="B92" s="45" t="n"/>
+      <c r="A92" s="44" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B92" s="45" t="inlineStr">
+        <is>
+          <t>Japedido Software</t>
+        </is>
+      </c>
       <c r="C92" s="45" t="n"/>
       <c r="D92" s="46" t="n"/>
       <c r="E92" s="45" t="n"/>
       <c r="F92" s="47" t="n"/>
-      <c r="G92" s="48" t="n"/>
-      <c r="H92" s="49" t="n"/>
-      <c r="I92" s="45" t="n"/>
+      <c r="G92" s="48" t="n">
+        <v>44.99</v>
+      </c>
+      <c r="H92" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I92" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 13/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 14/10/2026 11:57
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -55902,16 +55902,36 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="17" t="n"/>
-      <c r="B93" s="18" t="n"/>
-      <c r="C93" s="18" t="n"/>
-      <c r="D93" s="27" t="n"/>
-      <c r="E93" s="18" t="n"/>
+      <c r="A93" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t>Olegario Oliveira da Silva</t>
+        </is>
+      </c>
+      <c r="C93" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest + Mangueira</t>
+        </is>
+      </c>
+      <c r="D93" s="27" t="n">
+        <v>150</v>
+      </c>
+      <c r="E93" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F93" s="19" t="n"/>
       <c r="G93" s="19" t="n"/>
       <c r="H93" s="21" t="n"/>
       <c r="I93" s="18" t="n"/>
-      <c r="J93" s="18" t="n"/>
+      <c r="J93" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0523</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="44" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 14/10/2026 15:19
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -51790,7 +51790,7 @@
       </c>
       <c r="E212" s="45" t="inlineStr">
         <is>
-          <t>Aguardando Pagamento</t>
+          <t>Dinheiro</t>
         </is>
       </c>
       <c r="F212" s="47" t="n"/>
@@ -51798,7 +51798,7 @@
       <c r="H212" s="49" t="n"/>
       <c r="I212" s="45" t="inlineStr">
         <is>
-          <t>Preço com desconto de cliente. Pagamento previsto para 30/09/2026.</t>
+          <t>Preço com desconto de cliente. Pagamento previsto para 30/09/2026. Pago em dinheiro em 14/10/2026.</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">

</xml_diff>

<commit_message>
Atualizacao do painel - 14/10/2026 17:39
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -55934,50 +55934,148 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="44" t="n"/>
-      <c r="B94" s="45" t="n"/>
-      <c r="C94" s="45" t="n"/>
-      <c r="D94" s="46" t="n"/>
-      <c r="E94" s="45" t="n"/>
+      <c r="A94" s="44" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B94" s="45" t="inlineStr">
+        <is>
+          <t>Aldaci Freire de Araujo</t>
+        </is>
+      </c>
+      <c r="C94" s="45" t="inlineStr">
+        <is>
+          <t>Refil Pro Life</t>
+        </is>
+      </c>
+      <c r="D94" s="46" t="n">
+        <v>130</v>
+      </c>
+      <c r="E94" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F94" s="47" t="n"/>
       <c r="G94" s="48" t="n"/>
       <c r="H94" s="49" t="n"/>
-      <c r="I94" s="45" t="n"/>
+      <c r="I94" s="45" t="inlineStr">
+        <is>
+          <t>Cliente pediu desconto (Pro Life no lugar do Everest do cadastro). Troca do dia 14/10/2026. Com o suporte (linha abaixo), total R$ 150,00 em dinheiro.</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>CLI-0529</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="17" t="n"/>
-      <c r="B95" s="18" t="n"/>
-      <c r="C95" s="18" t="n"/>
-      <c r="D95" s="27" t="n"/>
-      <c r="E95" s="18" t="n"/>
+      <c r="A95" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B95" s="18" t="inlineStr">
+        <is>
+          <t>Aldaci Freire de Araujo</t>
+        </is>
+      </c>
+      <c r="C95" s="18" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D95" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="E95" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F95" s="19" t="n"/>
       <c r="G95" s="19" t="n"/>
       <c r="H95" s="21" t="n"/>
-      <c r="I95" s="18" t="n"/>
-      <c r="J95" s="18" t="n"/>
+      <c r="I95" s="18" t="inlineStr">
+        <is>
+          <t>Suporte do aparelho estava ruim; trocado só um lado (kit suporte normal R$ 40,00).</t>
+        </is>
+      </c>
+      <c r="J95" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0529</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="44" t="n"/>
-      <c r="B96" s="45" t="n"/>
-      <c r="C96" s="45" t="n"/>
-      <c r="D96" s="46" t="n"/>
-      <c r="E96" s="45" t="n"/>
-      <c r="F96" s="47" t="n"/>
+      <c r="A96" s="44" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B96" s="45" t="inlineStr">
+        <is>
+          <t>Marilia Silva</t>
+        </is>
+      </c>
+      <c r="C96" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro + Termostato</t>
+        </is>
+      </c>
+      <c r="D96" s="46" t="n">
+        <v>370</v>
+      </c>
+      <c r="E96" s="45" t="inlineStr">
+        <is>
+          <t>Crédito à Vista</t>
+        </is>
+      </c>
+      <c r="F96" s="47" t="n">
+        <v>12.99</v>
+      </c>
       <c r="G96" s="48" t="n"/>
       <c r="H96" s="49" t="n"/>
-      <c r="I96" s="45" t="n"/>
+      <c r="I96" s="45" t="inlineStr">
+        <is>
+          <t>Termostato trocado por defeito (não desligava). Ao entregar o aparelho consertado, adiantou a troca do refil (vencia no mês que vem). Crédito 1x.</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>CLI-0590</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="17" t="n"/>
-      <c r="B97" s="18" t="n"/>
-      <c r="C97" s="18" t="n"/>
-      <c r="D97" s="27" t="n"/>
-      <c r="E97" s="18" t="n"/>
-      <c r="F97" s="19" t="n"/>
+      <c r="A97" s="17" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t>Reginaldo Novaes de Oliveira - Barbara Novais</t>
+        </is>
+      </c>
+      <c r="C97" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D97" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E97" s="18" t="inlineStr">
+        <is>
+          <t>Débito</t>
+        </is>
+      </c>
+      <c r="F97" s="19" t="n">
+        <v>2.03</v>
+      </c>
       <c r="G97" s="19" t="n"/>
       <c r="H97" s="21" t="n"/>
       <c r="I97" s="18" t="n"/>
-      <c r="J97" s="18" t="n"/>
+      <c r="J97" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0524</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="44" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 14/10/2026 18:07
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -66420,7 +66420,7 @@
     </row>
     <row r="5">
       <c r="A5" s="189">
-        <f>D96</f>
+        <f>D97</f>
         <v/>
       </c>
       <c r="C5" s="204">
@@ -69133,54 +69133,85 @@
       </c>
     </row>
     <row r="94" s="157">
-      <c r="A94" s="86" t="inlineStr">
+      <c r="A94" s="78" t="inlineStr">
+        <is>
+          <t>Proxxima Telecomunicacoes S.A.</t>
+        </is>
+      </c>
+      <c r="B94" s="78" t="inlineStr">
+        <is>
+          <t>Internet da loja — plano Turbinados 700 MB, contrato 578646</t>
+        </is>
+      </c>
+      <c r="C94" s="77" t="n">
+        <v>46310</v>
+      </c>
+      <c r="D94" s="79" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="E94" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F94" s="112">
+        <f>IF(OR($E94="Pago",$C94=""),"",MAX(0,TODAY()-$C94))</f>
+        <v/>
+      </c>
+      <c r="G94" s="78" t="inlineStr">
+        <is>
+          <t>Categoria quando pagar: Água, Energia e Internet. Fatura FAT26091809010676 (emissão 18/09/2026), NFCom 410732, boleto Bradesco 237. Linha digitável 23790.49303 90000.443094 56025.103005 3 16000000006999. Nosso número 09000044309567. Após o vencimento: multa de 2% + mora de 1,20% a.m. A fatura sai em nome do sócio, mas o serviço é da loja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" s="157">
+      <c r="A95" s="86" t="inlineStr">
         <is>
           <t>TOTAL A PAGAR — COM BOLETO EM MÃOS</t>
         </is>
       </c>
-      <c r="B94" s="86" t="n"/>
-      <c r="C94" s="114" t="n"/>
-      <c r="D94" s="115">
-        <f>SUMIF(E11:E93,"Pendente",D11:D93)</f>
-        <v/>
-      </c>
-      <c r="E94" s="116" t="n"/>
-      <c r="F94" s="116" t="n"/>
-      <c r="G94" s="86" t="n"/>
-    </row>
-    <row r="95" s="157">
-      <c r="A95" s="144" t="inlineStr">
+      <c r="B95" s="86" t="n"/>
+      <c r="C95" s="114" t="n"/>
+      <c r="D95" s="115">
+        <f>SUMIF(E11:E94,"Pendente",D11:D94)</f>
+        <v/>
+      </c>
+      <c r="E95" s="116" t="n"/>
+      <c r="F95" s="116" t="n"/>
+      <c r="G95" s="86" t="n"/>
+    </row>
+    <row r="96" s="157">
+      <c r="A96" s="144" t="inlineStr">
         <is>
           <t>PREVISTO — compromisso certo que ainda não está documentado</t>
         </is>
       </c>
-      <c r="B95" s="144" t="n"/>
-      <c r="C95" s="145" t="n"/>
-      <c r="D95" s="146">
-        <f>SUMIF(E11:E93,"Previsto",D11:D93)</f>
-        <v/>
-      </c>
-      <c r="E95" s="142" t="n"/>
-      <c r="F95" s="142" t="n"/>
-      <c r="G95" s="144" t="n"/>
-    </row>
-    <row r="96" s="157">
-      <c r="A96" s="86" t="inlineStr">
+      <c r="B96" s="144" t="n"/>
+      <c r="C96" s="145" t="n"/>
+      <c r="D96" s="146">
+        <f>SUMIF(E11:E94,"Previsto",D11:D94)</f>
+        <v/>
+      </c>
+      <c r="E96" s="142" t="n"/>
+      <c r="F96" s="142" t="n"/>
+      <c r="G96" s="144" t="n"/>
+    </row>
+    <row r="97" s="157">
+      <c r="A97" s="86" t="inlineStr">
         <is>
           <t>TOTAL GERAL A PAGAR (boletos + previsão)</t>
         </is>
       </c>
-      <c r="B96" s="86" t="n"/>
-      <c r="C96" s="114" t="n"/>
-      <c r="D96" s="115">
-        <f>D94+D95</f>
-        <v/>
-      </c>
-      <c r="E96" s="116" t="n"/>
-      <c r="F96" s="116" t="n"/>
-      <c r="G96" s="86" t="n"/>
-    </row>
-    <row r="97" s="157"/>
+      <c r="B97" s="86" t="n"/>
+      <c r="C97" s="114" t="n"/>
+      <c r="D97" s="115">
+        <f>D95+D96</f>
+        <v/>
+      </c>
+      <c r="E97" s="116" t="n"/>
+      <c r="F97" s="116" t="n"/>
+      <c r="G97" s="86" t="n"/>
+    </row>
     <row r="98" ht="15.75" customHeight="1" s="157"/>
     <row r="99" ht="15.75" customHeight="1" s="157">
       <c r="A99" s="200" t="inlineStr">
@@ -71083,7 +71114,7 @@
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E11:E93" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E11:E94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Pago,Previsto"</formula1>
     </dataValidation>
     <dataValidation sqref="E102:E156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Atualizacao do painel - 15/10/2026 11:27
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -56078,73 +56078,186 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="44" t="n"/>
-      <c r="B98" s="45" t="n"/>
-      <c r="C98" s="45" t="n"/>
-      <c r="D98" s="46" t="n"/>
-      <c r="E98" s="45" t="n"/>
+      <c r="A98" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B98" s="45" t="inlineStr">
+        <is>
+          <t>Consumidor Final</t>
+        </is>
+      </c>
+      <c r="C98" s="45" t="inlineStr">
+        <is>
+          <t>Torneira para Purificador Latina</t>
+        </is>
+      </c>
+      <c r="D98" s="46" t="n">
+        <v>20</v>
+      </c>
+      <c r="E98" s="45" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F98" s="47" t="n"/>
       <c r="G98" s="48" t="n"/>
       <c r="H98" s="49" t="n"/>
       <c r="I98" s="45" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="17" t="n"/>
-      <c r="B99" s="18" t="n"/>
+      <c r="A99" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B99" s="18" t="inlineStr">
+        <is>
+          <t>Combustível</t>
+        </is>
+      </c>
       <c r="C99" s="18" t="n"/>
       <c r="D99" s="27" t="n"/>
       <c r="E99" s="18" t="n"/>
       <c r="F99" s="19" t="n"/>
-      <c r="G99" s="19" t="n"/>
-      <c r="H99" s="21" t="n"/>
-      <c r="I99" s="18" t="n"/>
+      <c r="G99" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="H99" s="21" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I99" s="18" t="inlineStr">
+        <is>
+          <t>Gasolina comum 1,482 L a R$ 6,75/L — Posto Avenida Jacobina (Avenida Posto de Combustíveis LTDA, CNPJ 46.115.794/0001-30, Av. Orlando Oliveira Pires, 1430, Centro, Jacobina), NFC-e nº 000927128 série 002 de 15/10/2026 09:39. Pago R$ 10,00 em dinheiro.</t>
+        </is>
+      </c>
       <c r="J99" s="18" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="44" t="n"/>
-      <c r="B100" s="45" t="n"/>
+      <c r="A100" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B100" s="45" t="inlineStr">
+        <is>
+          <t>Combustível</t>
+        </is>
+      </c>
       <c r="C100" s="45" t="n"/>
       <c r="D100" s="46" t="n"/>
       <c r="E100" s="45" t="n"/>
       <c r="F100" s="47" t="n"/>
-      <c r="G100" s="48" t="n"/>
-      <c r="H100" s="49" t="n"/>
-      <c r="I100" s="45" t="n"/>
+      <c r="G100" s="48" t="n">
+        <v>40</v>
+      </c>
+      <c r="H100" s="49" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I100" s="45" t="inlineStr">
+        <is>
+          <t>Gasolina aditivada (Ipimax) 5,806 L a R$ 6,89/L — Transvale Derivados de Petróleo LTDA (CNPJ 11.271.229/0002-68, Av. Orlando Oliveira Pires, 1164, Centro, Jacobina), NFC-e nº 000285556 série 001 de 15/10/2026 10:21. Pago R$ 40,00 em dinheiro.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" s="17" t="n"/>
-      <c r="B101" s="18" t="n"/>
-      <c r="C101" s="18" t="n"/>
-      <c r="D101" s="27" t="n"/>
-      <c r="E101" s="18" t="n"/>
+      <c r="A101" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B101" s="18" t="inlineStr">
+        <is>
+          <t>Casa das Portas Comercio de Madeiras LTDA</t>
+        </is>
+      </c>
+      <c r="C101" s="18" t="inlineStr">
+        <is>
+          <t>Refil Pro Life</t>
+        </is>
+      </c>
+      <c r="D101" s="27" t="n">
+        <v>130</v>
+      </c>
+      <c r="E101" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F101" s="19" t="n"/>
       <c r="G101" s="19" t="n"/>
       <c r="H101" s="21" t="n"/>
       <c r="I101" s="18" t="n"/>
-      <c r="J101" s="18" t="n"/>
+      <c r="J101" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0046</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="44" t="n"/>
-      <c r="B102" s="45" t="n"/>
-      <c r="C102" s="45" t="n"/>
-      <c r="D102" s="46" t="n"/>
-      <c r="E102" s="45" t="n"/>
+      <c r="A102" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B102" s="45" t="inlineStr">
+        <is>
+          <t>Casa do Construtor</t>
+        </is>
+      </c>
+      <c r="C102" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D102" s="46" t="n">
+        <v>140</v>
+      </c>
+      <c r="E102" s="45" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F102" s="47" t="n"/>
       <c r="G102" s="48" t="n"/>
       <c r="H102" s="49" t="n"/>
       <c r="I102" s="45" t="n"/>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>EMP-0320</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="17" t="n"/>
-      <c r="B103" s="18" t="n"/>
-      <c r="C103" s="18" t="n"/>
-      <c r="D103" s="27" t="n"/>
-      <c r="E103" s="18" t="n"/>
+      <c r="A103" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B103" s="18" t="inlineStr">
+        <is>
+          <t>Lapec</t>
+        </is>
+      </c>
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>Refil E3 + Refil Everest</t>
+        </is>
+      </c>
+      <c r="D103" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="E103" s="18" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F103" s="19" t="n"/>
       <c r="G103" s="19" t="n"/>
       <c r="H103" s="21" t="n"/>
-      <c r="I103" s="18" t="n"/>
-      <c r="J103" s="18" t="n"/>
+      <c r="I103" s="18" t="inlineStr">
+        <is>
+          <t>Refil E3 R$ 80,00 + Refil Everest R$ 120,00.</t>
+        </is>
+      </c>
+      <c r="J103" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0199</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="44" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 15/10/2026 17:05
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -53003,7 +53003,7 @@
     </row>
     <row r="5">
       <c r="A5" s="77" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B5" s="78" t="inlineStr">
         <is>
@@ -53020,7 +53020,7 @@
       </c>
       <c r="E5" s="78" t="inlineStr">
         <is>
-          <t>Aguardando Pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F5" s="79" t="n"/>
@@ -53028,7 +53028,7 @@
       <c r="H5" s="78" t="n"/>
       <c r="I5" s="78" t="inlineStr">
         <is>
-          <t>Grupo Ânima — OC AEMPPO00004453 · NF 000.004.332 de 26/08/2026 · prazo 45 dias · vencimento 10/10/2026 (desc. 3%) · previsão de pagamento confirmada no portal V360 em 02/09/2026</t>
+          <t>Grupo Ânima — OC AEMPPO00004453 · NF 000.004.332 de 26/08/2026 · prazo 45 dias · vencimento 10/10/2026 (desc. 3%) · previsão de pagamento confirmada no portal V360 em 02/09/2026 · Venda de 10/10/2026 — pagamento recebido em 13/10/2026 na conta do BNB (data em que o portal V360 marcou Nota Paga; dia/hora exatos a confirmar com a Edilânia)</t>
         </is>
       </c>
       <c r="J5" s="78" t="inlineStr">
@@ -70092,7 +70092,7 @@
       </c>
       <c r="E124" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F124" s="112">
@@ -70101,7 +70101,7 @@
       </c>
       <c r="G124" s="78" t="inlineStr">
         <is>
-          <t>Grupo Ânima — NF 000.004.332 de 26/08/2026 · OC AEMPPO00004453 · 45 dias</t>
+          <t>Grupo Ânima — NF 000.004.332 de 26/08/2026 · OC AEMPPO00004453 · 45 dias · Recebido em 13/10/2026 no BNB (Nota Paga no portal V360).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao do painel - 15/10/2026 18:22
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -56260,104 +56260,259 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="44" t="n"/>
-      <c r="B104" s="45" t="n"/>
-      <c r="C104" s="45" t="n"/>
-      <c r="D104" s="46" t="n"/>
-      <c r="E104" s="45" t="n"/>
+      <c r="A104" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B104" s="45" t="inlineStr">
+        <is>
+          <t>Edinaldo Nunes - Marilene de Souza Oliveira</t>
+        </is>
+      </c>
+      <c r="C104" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D104" s="46" t="n">
+        <v>190</v>
+      </c>
+      <c r="E104" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F104" s="47" t="n"/>
       <c r="G104" s="48" t="n"/>
       <c r="H104" s="49" t="n"/>
       <c r="I104" s="45" t="n"/>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>CLI-0499</t>
+        </is>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="17" t="n"/>
-      <c r="B105" s="18" t="n"/>
-      <c r="C105" s="18" t="n"/>
-      <c r="D105" s="27" t="n"/>
-      <c r="E105" s="18" t="n"/>
+      <c r="A105" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B105" s="18" t="inlineStr">
+        <is>
+          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
+        </is>
+      </c>
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D105" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E105" s="18" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F105" s="19" t="n"/>
       <c r="G105" s="19" t="n"/>
       <c r="H105" s="21" t="n"/>
       <c r="I105" s="18" t="n"/>
-      <c r="J105" s="18" t="n"/>
+      <c r="J105" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0253</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="44" t="n"/>
-      <c r="B106" s="45" t="n"/>
+      <c r="A106" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B106" s="45" t="inlineStr">
+        <is>
+          <t>Eversoft</t>
+        </is>
+      </c>
       <c r="C106" s="45" t="n"/>
       <c r="D106" s="46" t="n"/>
       <c r="E106" s="45" t="n"/>
       <c r="F106" s="47" t="n"/>
-      <c r="G106" s="48" t="n"/>
-      <c r="H106" s="49" t="n"/>
-      <c r="I106" s="45" t="n"/>
+      <c r="G106" s="48" t="n">
+        <v>980.83</v>
+      </c>
+      <c r="H106" s="49" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I106" s="45" t="inlineStr">
+        <is>
+          <t>Boleto doc. 74454 (emissão 17/07/2026) · parcela 3/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="17" t="n"/>
-      <c r="B107" s="18" t="n"/>
+      <c r="A107" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B107" s="18" t="inlineStr">
+        <is>
+          <t>Everest Refrigeração</t>
+        </is>
+      </c>
       <c r="C107" s="18" t="n"/>
       <c r="D107" s="27" t="n"/>
       <c r="E107" s="18" t="n"/>
       <c r="F107" s="19" t="n"/>
-      <c r="G107" s="19" t="n"/>
-      <c r="H107" s="21" t="n"/>
-      <c r="I107" s="18" t="n"/>
+      <c r="G107" s="19" t="n">
+        <v>892.3</v>
+      </c>
+      <c r="H107" s="21" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I107" s="18" t="inlineStr">
+        <is>
+          <t>Boleto doc. 381554 (emissão 17/07/2026) · parcela 3/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
+        </is>
+      </c>
       <c r="J107" s="18" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="44" t="n"/>
-      <c r="B108" s="45" t="n"/>
+      <c r="A108" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B108" s="45" t="inlineStr">
+        <is>
+          <t>Everest Refrigeração</t>
+        </is>
+      </c>
       <c r="C108" s="45" t="n"/>
       <c r="D108" s="46" t="n"/>
       <c r="E108" s="45" t="n"/>
       <c r="F108" s="47" t="n"/>
-      <c r="G108" s="48" t="n"/>
-      <c r="H108" s="49" t="n"/>
-      <c r="I108" s="45" t="n"/>
+      <c r="G108" s="48" t="n">
+        <v>574.27</v>
+      </c>
+      <c r="H108" s="49" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I108" s="45" t="inlineStr">
+        <is>
+          <t>Boleto doc. 386188 (emissão 15/09/2026) · parcela 1/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="17" t="n"/>
-      <c r="B109" s="18" t="n"/>
+      <c r="A109" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B109" s="18" t="inlineStr">
+        <is>
+          <t>Tarcisio Oliveira Lima</t>
+        </is>
+      </c>
       <c r="C109" s="18" t="n"/>
       <c r="D109" s="27" t="n"/>
       <c r="E109" s="18" t="n"/>
       <c r="F109" s="19" t="n"/>
-      <c r="G109" s="19" t="n"/>
-      <c r="H109" s="21" t="n"/>
-      <c r="I109" s="18" t="n"/>
+      <c r="G109" s="19" t="n">
+        <v>486.32</v>
+      </c>
+      <c r="H109" s="21" t="inlineStr">
+        <is>
+          <t>Contabilidade</t>
+        </is>
+      </c>
+      <c r="I109" s="18" t="inlineStr">
+        <is>
+          <t>Serviço contábil — boleto Banco do Brasil, venc. 15/10/2026. Pago em 15/10/2026.</t>
+        </is>
+      </c>
       <c r="J109" s="18" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="44" t="n"/>
-      <c r="B110" s="45" t="n"/>
+      <c r="A110" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B110" s="45" t="inlineStr">
+        <is>
+          <t>Proxxima Telecomunicações</t>
+        </is>
+      </c>
       <c r="C110" s="45" t="n"/>
       <c r="D110" s="46" t="n"/>
       <c r="E110" s="45" t="n"/>
       <c r="F110" s="47" t="n"/>
-      <c r="G110" s="48" t="n"/>
-      <c r="H110" s="49" t="n"/>
-      <c r="I110" s="45" t="n"/>
+      <c r="G110" s="48" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="H110" s="49" t="inlineStr">
+        <is>
+          <t>Água, Energia e Internet</t>
+        </is>
+      </c>
+      <c r="I110" s="45" t="inlineStr">
+        <is>
+          <t>Internet da loja — plano Turbinados 700 MB, contrato 578646. Fatura FAT26091809010676, venc. 15/10/2026. Pago em 15/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
-      <c r="A111" s="17" t="n"/>
-      <c r="B111" s="18" t="n"/>
+      <c r="A111" s="17" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t>Everest Refrigeração</t>
+        </is>
+      </c>
       <c r="C111" s="18" t="n"/>
       <c r="D111" s="27" t="n"/>
       <c r="E111" s="18" t="n"/>
       <c r="F111" s="19" t="n"/>
-      <c r="G111" s="19" t="n"/>
-      <c r="H111" s="21" t="n"/>
-      <c r="I111" s="18" t="n"/>
+      <c r="G111" s="19" t="n">
+        <v>856.34</v>
+      </c>
+      <c r="H111" s="21" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I111" s="18" t="inlineStr">
+        <is>
+          <t>Boleto doc. 377739 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago antecipado em 15/10/2026.</t>
+        </is>
+      </c>
       <c r="J111" s="18" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="44" t="n"/>
-      <c r="B112" s="45" t="n"/>
-      <c r="C112" s="45" t="n"/>
-      <c r="D112" s="46" t="n"/>
-      <c r="E112" s="45" t="n"/>
-      <c r="F112" s="47" t="n"/>
+      <c r="A112" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B112" s="45" t="inlineStr">
+        <is>
+          <t>Consumidor Final</t>
+        </is>
+      </c>
+      <c r="C112" s="45" t="inlineStr">
+        <is>
+          <t>Refil Plissado</t>
+        </is>
+      </c>
+      <c r="D112" s="46" t="n">
+        <v>80</v>
+      </c>
+      <c r="E112" s="45" t="inlineStr">
+        <is>
+          <t>Crédito à Vista</t>
+        </is>
+      </c>
+      <c r="F112" s="47" t="n">
+        <v>3.76</v>
+      </c>
       <c r="G112" s="48" t="n"/>
       <c r="H112" s="49" t="n"/>
       <c r="I112" s="45" t="n"/>
@@ -66482,7 +66637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G160"/>
+  <dimension ref="A1:G164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="157" min="1" max="1"/>
@@ -67280,7 +67435,7 @@
       </c>
       <c r="E32" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F32" s="113">
@@ -67289,7 +67444,7 @@
       </c>
       <c r="G32" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/28638818-9. Linha digitável 34191.12283 63881.890303 55679.010003 2 16000000098083. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 74454 (emissão 17/07/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260708782043000188550060000744541603671381.</t>
+          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/28638818-9. Linha digitável 34191.12283 63881.890303 55679.010003 2 16000000098083. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 74454 (emissão 17/07/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260708782043000188550060000744541603671381. Pago em 15/10/2026 — lançado em "Out 2026" como "Eversoft".</t>
         </is>
       </c>
     </row>
@@ -67536,7 +67691,7 @@
       </c>
       <c r="E40" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F40" s="113">
@@ -67545,7 +67700,7 @@
       </c>
       <c r="G40" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/28637900-6. Linha digitável 34191.12283 63790.060303 52238.850003 9 16000000089230. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 381554 (emissão 17/07/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.461,49 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260733079641000132550020003815541993407325.</t>
+          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/28637900-6. Linha digitável 34191.12283 63790.060303 52238.850003 9 16000000089230. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 381554 (emissão 17/07/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.461,49 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260733079641000132550020003815541993407325. Pago em 15/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -67632,7 +67787,7 @@
       </c>
       <c r="E43" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F43" s="112">
@@ -67641,7 +67796,7 @@
       </c>
       <c r="G43" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335118-5. Linha digitável 34191.12218 33511.850308 52238.850003 9 16010000085634. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377739 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.281,74 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777391313049192.</t>
+          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335118-5. Linha digitável 34191.12218 33511.850308 52238.850003 9 16010000085634. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377739 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.281,74 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777391313049192. Pago em 15/10/2026 (antecipado, venc. 16/10) — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68240,7 +68395,7 @@
       </c>
       <c r="E62" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F62" s="113">
@@ -68249,7 +68404,7 @@
       </c>
       <c r="G62" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35841919. Linha digitável 34191.12358 84191.930308 52238.850003 3 16000000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
+          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35841919. Linha digitável 34191.12358 84191.930308 52238.850003 3 16000000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116. Pago em 15/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -69136,7 +69291,7 @@
       </c>
       <c r="E90" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F90" s="113">
@@ -69145,7 +69300,7 @@
       </c>
       <c r="G90" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Contabilidade. Boleto Banco do Brasil 001-9. Linha digitável 00190.00009 03128.364001 00003.179173 8 16000000048632.</t>
+          <t>Categoria quando pagar: Contabilidade. Boleto Banco do Brasil 001-9. Linha digitável 00190.00009 03128.364001 00003.179173 8 16000000048632. Pago em 15/10/2026 — lançado em "Out 2026" como "Tarcisio Oliveira Lima".</t>
         </is>
       </c>
     </row>
@@ -69264,7 +69419,7 @@
       </c>
       <c r="E94" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F94" s="112">
@@ -69273,7 +69428,7 @@
       </c>
       <c r="G94" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Água, Energia e Internet. Fatura FAT26091809010676 (emissão 18/09/2026), NFCom 410732, boleto Bradesco 237. Linha digitável 23790.49303 90000.443094 56025.103005 3 16000000006999. Nosso número 09000044309567. Após o vencimento: multa de 2% + mora de 1,20% a.m. A fatura sai em nome do sócio, mas o serviço é da loja.</t>
+          <t>Categoria quando pagar: Água, Energia e Internet. Fatura FAT26091809010676 (emissão 18/09/2026), NFCom 410732, boleto Bradesco 237. Linha digitável 23790.49303 90000.443094 56025.103005 3 16000000006999. Nosso número 09000044309567. Após o vencimento: multa de 2% + mora de 1,20% a.m. A fatura sai em nome do sócio, mas o serviço é da loja. Pago em 15/10/2026 — lançado em "Out 2026" como "Proxxima Telecomunicações".</t>
         </is>
       </c>
     </row>
@@ -70860,7 +71015,7 @@
       </c>
       <c r="E148" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F148" s="112">
@@ -70869,7 +71024,7 @@
       </c>
       <c r="G148" s="78" t="inlineStr">
         <is>
-          <t>Pagamento previsto para 30/09/2026.</t>
+          <t>Pagamento previsto para 30/09/2026. Recebido em dinheiro em 14/10/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
@@ -71130,46 +71285,170 @@
       </c>
     </row>
     <row r="157" s="157">
-      <c r="A157" s="86" t="inlineStr">
+      <c r="A157" s="78" t="inlineStr">
+        <is>
+          <t>Casa do Construtor</t>
+        </is>
+      </c>
+      <c r="B157" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="C157" s="77" t="n">
+        <v>46310</v>
+      </c>
+      <c r="D157" s="79" t="n">
+        <v>140</v>
+      </c>
+      <c r="E157" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F157" s="112">
+        <f>IF(OR($E157="Recebido",$C157=""),"",MAX(0,TODAY()-$C157))</f>
+        <v/>
+      </c>
+      <c r="G157" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 15/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" s="157">
+      <c r="A158" s="78" t="inlineStr">
+        <is>
+          <t>Lapec</t>
+        </is>
+      </c>
+      <c r="B158" s="78" t="inlineStr">
+        <is>
+          <t>Refil E3 + Refil Everest</t>
+        </is>
+      </c>
+      <c r="C158" s="77" t="n">
+        <v>46310</v>
+      </c>
+      <c r="D158" s="79" t="n">
+        <v>200</v>
+      </c>
+      <c r="E158" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F158" s="112">
+        <f>IF(OR($E158="Recebido",$C158=""),"",MAX(0,TODAY()-$C158))</f>
+        <v/>
+      </c>
+      <c r="G158" s="78" t="inlineStr">
+        <is>
+          <t>Compra do dia 15/10/2026 — Refil E3 R$ 80,00 + Refil Everest R$ 120,00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" s="157">
+      <c r="A159" s="78" t="inlineStr">
+        <is>
+          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
+        </is>
+      </c>
+      <c r="B159" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="C159" s="77" t="n">
+        <v>46310</v>
+      </c>
+      <c r="D159" s="79" t="n">
+        <v>140</v>
+      </c>
+      <c r="E159" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F159" s="112">
+        <f>IF(OR($E159="Recebido",$C159=""),"",MAX(0,TODAY()-$C159))</f>
+        <v/>
+      </c>
+      <c r="G159" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 15/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" s="157">
+      <c r="A160" s="78" t="inlineStr">
+        <is>
+          <t>Colegio Oasis de Jacobina - Unopar</t>
+        </is>
+      </c>
+      <c r="B160" s="78" t="inlineStr">
+        <is>
+          <t>2x Refil Plissado + 2x Carcaça 9"</t>
+        </is>
+      </c>
+      <c r="C160" s="77" t="n">
+        <v>46305</v>
+      </c>
+      <c r="D160" s="79" t="n">
+        <v>400</v>
+      </c>
+      <c r="E160" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F160" s="112">
+        <f>IF(OR($E160="Recebido",$C160=""),"",MAX(0,TODAY()-$C160))</f>
+        <v/>
+      </c>
+      <c r="G160" s="78" t="inlineStr">
+        <is>
+          <t>2x Refil Plissado R$ 80,00 cada + 2x Carcaça 9" R$ 120,00 cada. Cláudio assinou para pagar depois. Falta enviar a NF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" s="157">
+      <c r="A161" s="86" t="inlineStr">
         <is>
           <t>TOTAL EM ABERTO A RECEBER (detalhe)</t>
         </is>
       </c>
-      <c r="D157" s="115">
-        <f>SUMIF(E102:E156,"Pendente",D102:D156)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="158" s="157">
-      <c r="A158" s="202" t="inlineStr">
+      <c r="D161" s="115">
+        <f>SUMIF(E102:E160,"Pendente",D102:D160)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162" s="157">
+      <c r="A162" s="202" t="inlineStr">
         <is>
           <t>CONFERÊNCIA COM AS ABAS DOS MESES</t>
         </is>
       </c>
-      <c r="B158" s="159" t="n"/>
-      <c r="C158" s="159" t="n"/>
-      <c r="D158" s="159" t="n"/>
-      <c r="E158" s="159" t="n"/>
-      <c r="F158" s="159" t="n"/>
-      <c r="G158" s="160" t="n"/>
-    </row>
-    <row r="159" s="157">
-      <c r="A159" s="203">
-        <f>IF(ROUND(D157-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D157-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="160" s="157">
-      <c r="A160" s="203" t="inlineStr">
+      <c r="B162" s="159" t="n"/>
+      <c r="C162" s="159" t="n"/>
+      <c r="D162" s="159" t="n"/>
+      <c r="E162" s="159" t="n"/>
+      <c r="F162" s="159" t="n"/>
+      <c r="G162" s="160" t="n"/>
+    </row>
+    <row r="163" s="157">
+      <c r="A163" s="203">
+        <f>IF(ROUND(D161-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D161-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164" s="157">
+      <c r="A164" s="203" t="inlineStr">
         <is>
           <t>As contas a pagar do DigiSat (pendentes até 27/07/2026) foram todas quitadas — confirmado em 19/08/2026. A única dívida em aberto hoje é o Capital de Giro do Banco do Brasil. Lance aqui novos compromissos conforme surgirem.</t>
         </is>
       </c>
     </row>
-    <row r="161" s="157"/>
-    <row r="162" s="157"/>
-    <row r="163" s="157"/>
-    <row r="164" s="157"/>
     <row r="165" s="157"/>
     <row r="166" s="157"/>
     <row r="167" s="157"/>
@@ -71214,10 +71493,10 @@
   <mergeCells count="13">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="A159:G159"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A158:G158"/>
+    <mergeCell ref="A162:G162"/>
+    <mergeCell ref="A163:G163"/>
     <mergeCell ref="A100:G100"/>
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="A5:B6"/>
@@ -71230,7 +71509,7 @@
     <dataValidation sqref="E11:E94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Pago,Previsto"</formula1>
     </dataValidation>
-    <dataValidation sqref="E102:E156" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E102:E160" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Recebido"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Atualizacao do painel - 16/10/2026 12:26
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -56518,23 +56518,65 @@
       <c r="I112" s="45" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="17" t="n"/>
-      <c r="B113" s="18" t="n"/>
-      <c r="C113" s="18" t="n"/>
-      <c r="D113" s="27" t="n"/>
-      <c r="E113" s="18" t="n"/>
-      <c r="F113" s="19" t="n"/>
+      <c r="A113" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B113" s="18" t="inlineStr">
+        <is>
+          <t>Alcina Rocha Lima Azevedo</t>
+        </is>
+      </c>
+      <c r="C113" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D113" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E113" s="18" t="inlineStr">
+        <is>
+          <t>Crédito Parcelado</t>
+        </is>
+      </c>
+      <c r="F113" s="19" t="n">
+        <v>11.73</v>
+      </c>
       <c r="G113" s="19" t="n"/>
       <c r="H113" s="21" t="n"/>
-      <c r="I113" s="18" t="n"/>
-      <c r="J113" s="18" t="n"/>
+      <c r="I113" s="18" t="inlineStr">
+        <is>
+          <t>Crédito em 2x. Instalação à tarde.</t>
+        </is>
+      </c>
+      <c r="J113" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0033</t>
+        </is>
+      </c>
     </row>
     <row r="114">
-      <c r="A114" s="44" t="n"/>
-      <c r="B114" s="45" t="n"/>
-      <c r="C114" s="45" t="n"/>
-      <c r="D114" s="46" t="n"/>
-      <c r="E114" s="45" t="n"/>
+      <c r="A114" s="44" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B114" s="45" t="inlineStr">
+        <is>
+          <t>Consumidor Final</t>
+        </is>
+      </c>
+      <c r="C114" s="45" t="inlineStr">
+        <is>
+          <t>Refil E3</t>
+        </is>
+      </c>
+      <c r="D114" s="46" t="n">
+        <v>60</v>
+      </c>
+      <c r="E114" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F114" s="47" t="n"/>
       <c r="G114" s="48" t="n"/>
       <c r="H114" s="49" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 16/10/2026 18:13
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -56274,7 +56274,7 @@
         </is>
       </c>
       <c r="D104" s="46" t="n">
-        <v>190</v>
+        <v>100</v>
       </c>
       <c r="E104" s="45" t="inlineStr">
         <is>
@@ -56284,7 +56284,11 @@
       <c r="F104" s="47" t="n"/>
       <c r="G104" s="48" t="n"/>
       <c r="H104" s="49" t="n"/>
-      <c r="I104" s="45" t="n"/>
+      <c r="I104" s="45" t="inlineStr">
+        <is>
+          <t>Venda de R$ 190,00 com pagamento dividido: R$ 100,00 em dinheiro + R$ 90,00 no Pix.</t>
+        </is>
+      </c>
       <c r="J104" t="inlineStr">
         <is>
           <t>CLI-0499</t>
@@ -56293,7 +56297,7 @@
     </row>
     <row r="105">
       <c r="A105" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B105" s="18" t="inlineStr">
         <is>
@@ -56310,13 +56314,17 @@
       </c>
       <c r="E105" s="18" t="inlineStr">
         <is>
-          <t>Aguardando Pagamento</t>
+          <t>Pix</t>
         </is>
       </c>
       <c r="F105" s="19" t="n"/>
       <c r="G105" s="19" t="n"/>
       <c r="H105" s="21" t="n"/>
-      <c r="I105" s="18" t="n"/>
+      <c r="I105" s="18" t="inlineStr">
+        <is>
+          <t>Venda de 15/10/2026 — pagamento recebido em 16/10/2026 via Pix.</t>
+        </is>
+      </c>
       <c r="J105" s="18" t="inlineStr">
         <is>
           <t>EMP-0253</t>
@@ -56583,73 +56591,207 @@
       <c r="I114" s="45" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="17" t="n"/>
-      <c r="B115" s="18" t="n"/>
-      <c r="C115" s="18" t="n"/>
-      <c r="D115" s="27" t="n"/>
-      <c r="E115" s="18" t="n"/>
+      <c r="A115" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B115" s="18" t="inlineStr">
+        <is>
+          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+        </is>
+      </c>
+      <c r="C115" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D115" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E115" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F115" s="19" t="n"/>
       <c r="G115" s="19" t="n"/>
       <c r="H115" s="21" t="n"/>
-      <c r="I115" s="18" t="n"/>
-      <c r="J115" s="18" t="n"/>
+      <c r="I115" s="18" t="inlineStr">
+        <is>
+          <t>Venda de R$ 200,00 com pagamento dividido: R$ 140,00 em dinheiro + R$ 60,00 a receber. Bebedouro da recepção.</t>
+        </is>
+      </c>
+      <c r="J115" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0116</t>
+        </is>
+      </c>
     </row>
     <row r="116">
-      <c r="A116" s="44" t="n"/>
-      <c r="B116" s="45" t="n"/>
-      <c r="C116" s="45" t="n"/>
-      <c r="D116" s="46" t="n"/>
-      <c r="E116" s="45" t="n"/>
+      <c r="A116" s="44" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B116" s="45" t="inlineStr">
+        <is>
+          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+        </is>
+      </c>
+      <c r="C116" s="45" t="inlineStr">
+        <is>
+          <t>(Mesma venda acima — 2ª forma de pagamento, sem produtos novos)</t>
+        </is>
+      </c>
+      <c r="D116" s="46" t="n">
+        <v>60</v>
+      </c>
+      <c r="E116" s="45" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F116" s="47" t="n"/>
       <c r="G116" s="48" t="n"/>
       <c r="H116" s="49" t="n"/>
-      <c r="I116" s="45" t="n"/>
+      <c r="I116" s="45" t="inlineStr">
+        <is>
+          <t>Restante da venda de R$ 200,00 (R$ 140,00 pagos em dinheiro). Cliente vai pagar depois.</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>EMP-0116</t>
+        </is>
+      </c>
     </row>
     <row r="117">
-      <c r="A117" s="17" t="n"/>
-      <c r="B117" s="18" t="n"/>
-      <c r="C117" s="18" t="n"/>
-      <c r="D117" s="27" t="n"/>
-      <c r="E117" s="18" t="n"/>
+      <c r="A117" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B117" s="18" t="inlineStr">
+        <is>
+          <t>Contabilidade Abreu</t>
+        </is>
+      </c>
+      <c r="C117" s="18" t="inlineStr">
+        <is>
+          <t>Termostato</t>
+        </is>
+      </c>
+      <c r="D117" s="27" t="n">
+        <v>170</v>
+      </c>
+      <c r="E117" s="18" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F117" s="19" t="n"/>
       <c r="G117" s="19" t="n"/>
       <c r="H117" s="21" t="n"/>
-      <c r="I117" s="18" t="n"/>
-      <c r="J117" s="18" t="n"/>
+      <c r="I117" s="18" t="inlineStr">
+        <is>
+          <t>Troca de termostato.</t>
+        </is>
+      </c>
+      <c r="J117" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0105</t>
+        </is>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="44" t="n"/>
-      <c r="B118" s="45" t="n"/>
-      <c r="C118" s="45" t="n"/>
-      <c r="D118" s="46" t="n"/>
-      <c r="E118" s="45" t="n"/>
+      <c r="A118" s="44" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B118" s="45" t="inlineStr">
+        <is>
+          <t>Edinaldo Nunes - Marilene de Souza Oliveira</t>
+        </is>
+      </c>
+      <c r="C118" s="45" t="inlineStr">
+        <is>
+          <t>(Mesma venda acima — 2ª forma de pagamento, sem produtos novos)</t>
+        </is>
+      </c>
+      <c r="D118" s="46" t="n">
+        <v>90</v>
+      </c>
+      <c r="E118" s="45" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F118" s="47" t="n"/>
       <c r="G118" s="48" t="n"/>
       <c r="H118" s="49" t="n"/>
-      <c r="I118" s="45" t="n"/>
+      <c r="I118" s="45" t="inlineStr">
+        <is>
+          <t>Restante da venda de R$ 190,00 de 15/10 (R$ 100,00 em dinheiro + R$ 90,00 no Pix).</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>CLI-0499</t>
+        </is>
+      </c>
     </row>
     <row r="119">
-      <c r="A119" s="17" t="n"/>
-      <c r="B119" s="18" t="n"/>
-      <c r="C119" s="18" t="n"/>
-      <c r="D119" s="27" t="n"/>
-      <c r="E119" s="18" t="n"/>
+      <c r="A119" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B119" s="18" t="inlineStr">
+        <is>
+          <t>Eduardo Santos da Silva</t>
+        </is>
+      </c>
+      <c r="C119" s="18" t="inlineStr">
+        <is>
+          <t>Refil Pro Life</t>
+        </is>
+      </c>
+      <c r="D119" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E119" s="18" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F119" s="19" t="n"/>
       <c r="G119" s="19" t="n"/>
       <c r="H119" s="21" t="n"/>
       <c r="I119" s="18" t="n"/>
-      <c r="J119" s="18" t="n"/>
+      <c r="J119" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0408</t>
+        </is>
+      </c>
     </row>
     <row r="120">
-      <c r="A120" s="44" t="n"/>
-      <c r="B120" s="45" t="n"/>
+      <c r="A120" s="44" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B120" s="45" t="inlineStr">
+        <is>
+          <t>Cezar Silva Atacado e Varejo - A Lojinha Utilidades (Iene Quedila Nunes Dourado)</t>
+        </is>
+      </c>
       <c r="C120" s="45" t="n"/>
       <c r="D120" s="46" t="n"/>
       <c r="E120" s="45" t="n"/>
       <c r="F120" s="47" t="n"/>
-      <c r="G120" s="48" t="n"/>
-      <c r="H120" s="49" t="n"/>
-      <c r="I120" s="45" t="n"/>
+      <c r="G120" s="48" t="n">
+        <v>170</v>
+      </c>
+      <c r="H120" s="49" t="inlineStr">
+        <is>
+          <t>Manutenção e Reparos</t>
+        </is>
+      </c>
+      <c r="I120" s="45" t="inlineStr">
+        <is>
+          <t>Escada média (ferramenta para as instalações). Recibo de 16/10/2026. CNPJ 47.415.949/0002-05 — Rua Manoel Novais, 232, Jacobina-BA.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="17" t="n"/>
@@ -66679,7 +66821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G164"/>
+  <dimension ref="A1:G166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="157" min="1" max="1"/>
@@ -71409,7 +71551,7 @@
       </c>
       <c r="E159" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F159" s="112">
@@ -71418,7 +71560,7 @@
       </c>
       <c r="G159" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 15/10/2026.</t>
+          <t>Troca do dia 15/10/2026. Recebido via Pix em 16/10/2026 — lançado em "Out 2026".</t>
         </is>
       </c>
     </row>
@@ -71455,44 +71597,106 @@
       </c>
     </row>
     <row r="161" s="157">
-      <c r="A161" s="86" t="inlineStr">
+      <c r="A161" s="78" t="inlineStr">
+        <is>
+          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+        </is>
+      </c>
+      <c r="B161" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro (restante)</t>
+        </is>
+      </c>
+      <c r="C161" s="77" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D161" s="79" t="n">
+        <v>60</v>
+      </c>
+      <c r="E161" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F161" s="112">
+        <f>IF(OR($E161="Recebido",$C161=""),"",MAX(0,TODAY()-$C161))</f>
+        <v/>
+      </c>
+      <c r="G161" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 16/10/2026 — bebedouro da recepção. Venda de R$ 200,00: R$ 140,00 pagos em dinheiro em 16/10/2026; falta R$ 60,00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" s="157">
+      <c r="A162" s="78" t="inlineStr">
+        <is>
+          <t>Contabilidade Abreu</t>
+        </is>
+      </c>
+      <c r="B162" s="78" t="inlineStr">
+        <is>
+          <t>Termostato</t>
+        </is>
+      </c>
+      <c r="C162" s="77" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D162" s="79" t="n">
+        <v>170</v>
+      </c>
+      <c r="E162" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F162" s="112">
+        <f>IF(OR($E162="Recebido",$C162=""),"",MAX(0,TODAY()-$C162))</f>
+        <v/>
+      </c>
+      <c r="G162" s="78" t="inlineStr">
+        <is>
+          <t>Troca de termostato do dia 16/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" s="157">
+      <c r="A163" s="86" t="inlineStr">
         <is>
           <t>TOTAL EM ABERTO A RECEBER (detalhe)</t>
         </is>
       </c>
-      <c r="D161" s="115">
-        <f>SUMIF(E102:E160,"Pendente",D102:D160)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="162" s="157">
-      <c r="A162" s="202" t="inlineStr">
+      <c r="D163" s="115">
+        <f>SUMIF(E102:E162,"Pendente",D102:D162)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="164" s="157">
+      <c r="A164" s="202" t="inlineStr">
         <is>
           <t>CONFERÊNCIA COM AS ABAS DOS MESES</t>
         </is>
       </c>
-      <c r="B162" s="159" t="n"/>
-      <c r="C162" s="159" t="n"/>
-      <c r="D162" s="159" t="n"/>
-      <c r="E162" s="159" t="n"/>
-      <c r="F162" s="159" t="n"/>
-      <c r="G162" s="160" t="n"/>
-    </row>
-    <row r="163" s="157">
-      <c r="A163" s="203">
-        <f>IF(ROUND(D161-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D161-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="164" s="157">
-      <c r="A164" s="203" t="inlineStr">
+      <c r="B164" s="159" t="n"/>
+      <c r="C164" s="159" t="n"/>
+      <c r="D164" s="159" t="n"/>
+      <c r="E164" s="159" t="n"/>
+      <c r="F164" s="159" t="n"/>
+      <c r="G164" s="160" t="n"/>
+    </row>
+    <row r="165" s="157">
+      <c r="A165" s="203">
+        <f>IF(ROUND(D163-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D163-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="166" s="157">
+      <c r="A166" s="203" t="inlineStr">
         <is>
           <t>As contas a pagar do DigiSat (pendentes até 27/07/2026) foram todas quitadas — confirmado em 19/08/2026. A única dívida em aberto hoje é o Capital de Giro do Banco do Brasil. Lance aqui novos compromissos conforme surgirem.</t>
         </is>
       </c>
     </row>
-    <row r="165" s="157"/>
-    <row r="166" s="157"/>
     <row r="167" s="157"/>
     <row r="168" s="157"/>
     <row r="169" s="157"/>
@@ -71537,21 +71741,21 @@
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A162:G162"/>
-    <mergeCell ref="A163:G163"/>
     <mergeCell ref="A100:G100"/>
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="A5:B6"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E5:F6"/>
+    <mergeCell ref="A165:G165"/>
     <mergeCell ref="A99:G99"/>
+    <mergeCell ref="A164:G164"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="E11:E94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Pago,Previsto"</formula1>
     </dataValidation>
-    <dataValidation sqref="E102:E160" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E102:E162" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Recebido"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Atualizacao do painel - 16/10/2026 18:15
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -56794,38 +56794,86 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="17" t="n"/>
-      <c r="B121" s="18" t="n"/>
+      <c r="A121" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B121" s="18" t="inlineStr">
+        <is>
+          <t>Everest Refrigeração</t>
+        </is>
+      </c>
       <c r="C121" s="18" t="n"/>
       <c r="D121" s="27" t="n"/>
       <c r="E121" s="18" t="n"/>
       <c r="F121" s="19" t="n"/>
-      <c r="G121" s="19" t="n"/>
-      <c r="H121" s="21" t="n"/>
-      <c r="I121" s="18" t="n"/>
+      <c r="G121" s="19" t="n">
+        <v>139.32</v>
+      </c>
+      <c r="H121" s="21" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I121" s="18" t="inlineStr">
+        <is>
+          <t>Boleto doc. 377737 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago em 16/10/2026.</t>
+        </is>
+      </c>
       <c r="J121" s="18" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="44" t="n"/>
-      <c r="B122" s="45" t="n"/>
+      <c r="A122" s="44" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B122" s="45" t="inlineStr">
+        <is>
+          <t>Everest Refrigeração</t>
+        </is>
+      </c>
       <c r="C122" s="45" t="n"/>
       <c r="D122" s="46" t="n"/>
       <c r="E122" s="45" t="n"/>
       <c r="F122" s="47" t="n"/>
-      <c r="G122" s="48" t="n"/>
-      <c r="H122" s="49" t="n"/>
-      <c r="I122" s="45" t="n"/>
+      <c r="G122" s="48" t="n">
+        <v>865.52</v>
+      </c>
+      <c r="H122" s="49" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I122" s="45" t="inlineStr">
+        <is>
+          <t>Boleto doc. 377738 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago em 16/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
-      <c r="A123" s="17" t="n"/>
-      <c r="B123" s="18" t="n"/>
+      <c r="A123" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B123" s="18" t="inlineStr">
+        <is>
+          <t>Patrus Transportes</t>
+        </is>
+      </c>
       <c r="C123" s="18" t="n"/>
       <c r="D123" s="27" t="n"/>
       <c r="E123" s="18" t="n"/>
       <c r="F123" s="19" t="n"/>
-      <c r="G123" s="19" t="n"/>
-      <c r="H123" s="21" t="n"/>
-      <c r="I123" s="18" t="n"/>
+      <c r="G123" s="19" t="n">
+        <v>277.48</v>
+      </c>
+      <c r="H123" s="21" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I123" s="18" t="inlineStr">
+        <is>
+          <t>Frete — boleto Bradesco, venc. 16/10/2026. Pago em 16/10/2026.</t>
+        </is>
+      </c>
       <c r="J123" s="18" t="n"/>
     </row>
     <row r="124">
@@ -67907,7 +67955,7 @@
       </c>
       <c r="E41" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F41" s="112">
@@ -67916,7 +67964,7 @@
       </c>
       <c r="G41" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335994-9. Linha digitável 34191.12218 33599.490308 52238.850003 1 16010000013932. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377737 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 725,16 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777371117471168.</t>
+          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335994-9. Linha digitável 34191.12218 33599.490308 52238.850003 1 16010000013932. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377737 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 725,16 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777371117471168. Pago em 16/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -67939,7 +67987,7 @@
       </c>
       <c r="E42" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F42" s="113">
@@ -67948,7 +67996,7 @@
       </c>
       <c r="G42" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335634-1. Linha digitável 34191.12218 33563.410308 52238.850003 5 16010000086552. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377738 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.327,52 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777381143358478.</t>
+          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335634-1. Linha digitável 34191.12218 33563.410308 52238.850003 5 16010000086552. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377738 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.327,52 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777381143358478. Pago em 16/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -69443,7 +69491,7 @@
       </c>
       <c r="E89" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F89" s="112">
@@ -69452,7 +69500,7 @@
       </c>
       <c r="G89" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Transporte e Entregas. Boleto Bradesco 237-2. Linha digitável 23791.43007 93484.000265 98003.073701 2 16010000027748.</t>
+          <t>Categoria quando pagar: Transporte e Entregas. Boleto Bradesco 237-2. Linha digitável 23791.43007 93484.000265 98003.073701 2 16010000027748. Pago em 16/10/2026 — lançado em "Out 2026" como "Patrus Transportes".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao do painel - 17/10/2026 12:34
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -56877,49 +56877,113 @@
       <c r="J123" s="18" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="44" t="n"/>
-      <c r="B124" s="45" t="n"/>
+      <c r="A124" s="44" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B124" s="45" t="inlineStr">
+        <is>
+          <t>Cloro e Cia (Mello e Castiglioni Ltda)</t>
+        </is>
+      </c>
       <c r="C124" s="45" t="n"/>
       <c r="D124" s="46" t="n"/>
       <c r="E124" s="45" t="n"/>
       <c r="F124" s="47" t="n"/>
-      <c r="G124" s="48" t="n"/>
-      <c r="H124" s="49" t="n"/>
-      <c r="I124" s="45" t="n"/>
+      <c r="G124" s="48" t="n">
+        <v>36</v>
+      </c>
+      <c r="H124" s="49" t="inlineStr">
+        <is>
+          <t>Material de Limpeza e Escritório</t>
+        </is>
+      </c>
+      <c r="I124" s="45" t="inlineStr">
+        <is>
+          <t>DAV 000398 de 17/10/2026 — papel toalha interfolhado, álcool gel 1 L e sabonete líquido 1 L (R$ 37,50 com R$ 1,50 de desconto). Pago em dinheiro.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
-      <c r="A125" s="17" t="n"/>
-      <c r="B125" s="18" t="n"/>
+      <c r="A125" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B125" s="18" t="inlineStr">
+        <is>
+          <t>Diarista Eva</t>
+        </is>
+      </c>
       <c r="C125" s="18" t="n"/>
       <c r="D125" s="27" t="n"/>
       <c r="E125" s="18" t="n"/>
       <c r="F125" s="19" t="n"/>
-      <c r="G125" s="19" t="n"/>
-      <c r="H125" s="21" t="n"/>
-      <c r="I125" s="18" t="n"/>
+      <c r="G125" s="19" t="n">
+        <v>400</v>
+      </c>
+      <c r="H125" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I125" s="18" t="inlineStr">
+        <is>
+          <t>Pedido da Edilânia em 17/10/2026 — despesa pessoal.</t>
+        </is>
+      </c>
       <c r="J125" s="18" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="44" t="n"/>
-      <c r="B126" s="45" t="n"/>
+      <c r="A126" s="44" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B126" s="45" t="inlineStr">
+        <is>
+          <t>Compras para casa</t>
+        </is>
+      </c>
       <c r="C126" s="45" t="n"/>
       <c r="D126" s="46" t="n"/>
       <c r="E126" s="45" t="n"/>
       <c r="F126" s="47" t="n"/>
-      <c r="G126" s="48" t="n"/>
-      <c r="H126" s="49" t="n"/>
-      <c r="I126" s="45" t="n"/>
+      <c r="G126" s="48" t="n">
+        <v>200</v>
+      </c>
+      <c r="H126" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I126" s="45" t="inlineStr">
+        <is>
+          <t>Pedido da Edilânia em 17/10/2026 — despesa pessoal.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
-      <c r="A127" s="17" t="n"/>
-      <c r="B127" s="18" t="n"/>
+      <c r="A127" s="17" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B127" s="18" t="inlineStr">
+        <is>
+          <t>Comissão Wiliam</t>
+        </is>
+      </c>
       <c r="C127" s="18" t="n"/>
       <c r="D127" s="27" t="n"/>
       <c r="E127" s="18" t="n"/>
       <c r="F127" s="19" t="n"/>
-      <c r="G127" s="19" t="n"/>
-      <c r="H127" s="21" t="n"/>
-      <c r="I127" s="18" t="n"/>
+      <c r="G127" s="19" t="n">
+        <v>610</v>
+      </c>
+      <c r="H127" s="21" t="inlineStr">
+        <is>
+          <t>Salários, Comissões e Encargos</t>
+        </is>
+      </c>
+      <c r="I127" s="18" t="inlineStr">
+        <is>
+          <t>Comissões da quinzena de 05/10 a 16/10/2026 — R$ 610,00 de R$ 615,00; os R$ 5,00 restantes (venda de pré-filtro de 10/10) ficam para a próxima semana, por falta de troco no caixa.</t>
+        </is>
+      </c>
       <c r="J127" s="18" t="n"/>
     </row>
     <row r="128">

</xml_diff>

<commit_message>
Atualizacao do painel - 19/10/2026 18:28
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -41159,7 +41159,7 @@
       </c>
       <c r="J46" s="45" t="inlineStr">
         <is>
-          <t>EMP-0165</t>
+          <t>EMP-0138</t>
         </is>
       </c>
     </row>
@@ -56987,141 +56987,400 @@
       <c r="J127" s="18" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="44" t="n"/>
-      <c r="B128" s="45" t="n"/>
-      <c r="C128" s="45" t="n"/>
-      <c r="D128" s="46" t="n"/>
-      <c r="E128" s="45" t="n"/>
+      <c r="A128" s="44" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B128" s="45" t="inlineStr">
+        <is>
+          <t>Carneiro Ultra Drogaria LTDA - Filial 02</t>
+        </is>
+      </c>
+      <c r="C128" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D128" s="46" t="n">
+        <v>140</v>
+      </c>
+      <c r="E128" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F128" s="47" t="n"/>
       <c r="G128" s="48" t="n"/>
       <c r="H128" s="49" t="n"/>
       <c r="I128" s="45" t="n"/>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>EMP-0043</t>
+        </is>
+      </c>
     </row>
     <row r="129">
-      <c r="A129" s="17" t="n"/>
-      <c r="B129" s="18" t="n"/>
-      <c r="C129" s="18" t="n"/>
-      <c r="D129" s="27" t="n"/>
-      <c r="E129" s="18" t="n"/>
+      <c r="A129" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B129" s="18" t="inlineStr">
+        <is>
+          <t>Otica Imagem - José Luciano Viera Costa</t>
+        </is>
+      </c>
+      <c r="C129" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D129" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E129" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F129" s="19" t="n"/>
       <c r="G129" s="19" t="n"/>
       <c r="H129" s="21" t="n"/>
-      <c r="I129" s="18" t="n"/>
-      <c r="J129" s="18" t="n"/>
+      <c r="I129" s="18" t="inlineStr">
+        <is>
+          <t>Ótica pagou R$ 280,00 pelas duas trocas (térreo e 1º andar).</t>
+        </is>
+      </c>
+      <c r="J129" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0238</t>
+        </is>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="44" t="n"/>
-      <c r="B130" s="45" t="n"/>
-      <c r="C130" s="45" t="n"/>
-      <c r="D130" s="46" t="n"/>
-      <c r="E130" s="45" t="n"/>
+      <c r="A130" s="44" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B130" s="45" t="inlineStr">
+        <is>
+          <t>Otica Imagem - José Luciano Viera Costa 1 Andar</t>
+        </is>
+      </c>
+      <c r="C130" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D130" s="46" t="n">
+        <v>140</v>
+      </c>
+      <c r="E130" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F130" s="47" t="n"/>
       <c r="G130" s="48" t="n"/>
       <c r="H130" s="49" t="n"/>
-      <c r="I130" s="45" t="n"/>
+      <c r="I130" s="45" t="inlineStr">
+        <is>
+          <t>Ótica pagou R$ 280,00 pelas duas trocas (térreo e 1º andar).</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>EMP-0238</t>
+        </is>
+      </c>
     </row>
     <row r="131">
-      <c r="A131" s="17" t="n"/>
-      <c r="B131" s="18" t="n"/>
-      <c r="C131" s="18" t="n"/>
-      <c r="D131" s="27" t="n"/>
-      <c r="E131" s="18" t="n"/>
+      <c r="A131" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B131" s="18" t="inlineStr">
+        <is>
+          <t>Pedras e Pisos - Loja</t>
+        </is>
+      </c>
+      <c r="C131" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D131" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E131" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F131" s="19" t="n"/>
       <c r="G131" s="19" t="n"/>
       <c r="H131" s="21" t="n"/>
       <c r="I131" s="18" t="n"/>
-      <c r="J131" s="18" t="n"/>
+      <c r="J131" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0245</t>
+        </is>
+      </c>
     </row>
     <row r="132">
-      <c r="A132" s="44" t="n"/>
-      <c r="B132" s="45" t="n"/>
-      <c r="C132" s="45" t="n"/>
-      <c r="D132" s="46" t="n"/>
-      <c r="E132" s="45" t="n"/>
+      <c r="A132" s="44" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B132" s="45" t="inlineStr">
+        <is>
+          <t>Marsilia Marmores e Granitos Erelli</t>
+        </is>
+      </c>
+      <c r="C132" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D132" s="46" t="n">
+        <v>140</v>
+      </c>
+      <c r="E132" s="45" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F132" s="47" t="n"/>
       <c r="G132" s="48" t="n"/>
       <c r="H132" s="49" t="n"/>
       <c r="I132" s="45" t="n"/>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>EMP-0216</t>
+        </is>
+      </c>
     </row>
     <row r="133">
-      <c r="A133" s="17" t="n"/>
-      <c r="B133" s="18" t="n"/>
-      <c r="C133" s="18" t="n"/>
-      <c r="D133" s="27" t="n"/>
-      <c r="E133" s="18" t="n"/>
+      <c r="A133" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B133" s="18" t="inlineStr">
+        <is>
+          <t>Gilberto de Aguiar</t>
+        </is>
+      </c>
+      <c r="C133" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D133" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E133" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F133" s="19" t="n"/>
       <c r="G133" s="19" t="n"/>
       <c r="H133" s="21" t="n"/>
       <c r="I133" s="18" t="n"/>
-      <c r="J133" s="18" t="n"/>
+      <c r="J133" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0629</t>
+        </is>
+      </c>
     </row>
     <row r="134">
-      <c r="A134" s="44" t="n"/>
-      <c r="B134" s="45" t="n"/>
-      <c r="C134" s="45" t="n"/>
-      <c r="D134" s="46" t="n"/>
-      <c r="E134" s="45" t="n"/>
+      <c r="A134" s="44" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B134" s="45" t="inlineStr">
+        <is>
+          <t>A. S. Supermercado</t>
+        </is>
+      </c>
+      <c r="C134" s="45" t="inlineStr">
+        <is>
+          <t>Refil Pro Life + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D134" s="46" t="n">
+        <v>190</v>
+      </c>
+      <c r="E134" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F134" s="47" t="n"/>
       <c r="G134" s="48" t="n"/>
       <c r="H134" s="49" t="n"/>
       <c r="I134" s="45" t="n"/>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>EMP-0321</t>
+        </is>
+      </c>
     </row>
     <row r="135">
-      <c r="A135" s="17" t="n"/>
-      <c r="B135" s="18" t="n"/>
-      <c r="C135" s="18" t="n"/>
-      <c r="D135" s="27" t="n"/>
-      <c r="E135" s="18" t="n"/>
-      <c r="F135" s="19" t="n"/>
+      <c r="A135" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B135" s="18" t="inlineStr">
+        <is>
+          <t>Raulino Gonçalves dos Santos</t>
+        </is>
+      </c>
+      <c r="C135" s="18" t="inlineStr">
+        <is>
+          <t>Purificador Everest Foz Branco</t>
+        </is>
+      </c>
+      <c r="D135" s="27" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E135" s="18" t="inlineStr">
+        <is>
+          <t>Crédito Parcelado</t>
+        </is>
+      </c>
+      <c r="F135" s="19" t="n">
+        <v>119.85</v>
+      </c>
       <c r="G135" s="19" t="n"/>
       <c r="H135" s="21" t="n"/>
-      <c r="I135" s="18" t="n"/>
-      <c r="J135" s="18" t="n"/>
+      <c r="I135" s="18" t="inlineStr">
+        <is>
+          <t>Parcelado em 4x. Instalado em 19/10/2026.</t>
+        </is>
+      </c>
+      <c r="J135" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0906</t>
+        </is>
+      </c>
     </row>
     <row r="136">
-      <c r="A136" s="44" t="n"/>
-      <c r="B136" s="45" t="n"/>
-      <c r="C136" s="45" t="n"/>
-      <c r="D136" s="46" t="n"/>
-      <c r="E136" s="45" t="n"/>
+      <c r="A136" s="44" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B136" s="45" t="inlineStr">
+        <is>
+          <t>Larissa Sena</t>
+        </is>
+      </c>
+      <c r="C136" s="45" t="inlineStr">
+        <is>
+          <t>Refil FPA14</t>
+        </is>
+      </c>
+      <c r="D136" s="46" t="n">
+        <v>110</v>
+      </c>
+      <c r="E136" s="45" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F136" s="47" t="n"/>
       <c r="G136" s="48" t="n"/>
       <c r="H136" s="49" t="n"/>
-      <c r="I136" s="45" t="n"/>
+      <c r="I136" s="45" t="inlineStr">
+        <is>
+          <t>Pix de R$ 250,00 junto com o refil da Int Odontologia (R$ 140,00).</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>CLI-0907</t>
+        </is>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" s="17" t="n"/>
-      <c r="B137" s="18" t="n"/>
-      <c r="C137" s="18" t="n"/>
-      <c r="D137" s="27" t="n"/>
-      <c r="E137" s="18" t="n"/>
+      <c r="A137" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B137" s="18" t="inlineStr">
+        <is>
+          <t>Int Odontologia - Larissa Sena</t>
+        </is>
+      </c>
+      <c r="C137" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D137" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E137" s="18" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F137" s="19" t="n"/>
       <c r="G137" s="19" t="n"/>
       <c r="H137" s="21" t="n"/>
-      <c r="I137" s="18" t="n"/>
-      <c r="J137" s="18" t="n"/>
+      <c r="I137" s="18" t="inlineStr">
+        <is>
+          <t>Pago adiantado em 19/10/2026 no mesmo Pix de R$ 250,00 da Larissa Sena; troca prevista para 20/10/2026.</t>
+        </is>
+      </c>
+      <c r="J137" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0184</t>
+        </is>
+      </c>
     </row>
     <row r="138">
-      <c r="A138" s="44" t="n"/>
-      <c r="B138" s="45" t="n"/>
+      <c r="A138" s="44" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B138" s="45" t="inlineStr">
+        <is>
+          <t>Combustível</t>
+        </is>
+      </c>
       <c r="C138" s="45" t="n"/>
       <c r="D138" s="46" t="n"/>
       <c r="E138" s="45" t="n"/>
       <c r="F138" s="47" t="n"/>
-      <c r="G138" s="48" t="n"/>
-      <c r="H138" s="49" t="n"/>
-      <c r="I138" s="45" t="n"/>
+      <c r="G138" s="48" t="n">
+        <v>30</v>
+      </c>
+      <c r="H138" s="49" t="inlineStr">
+        <is>
+          <t>Transporte e Entregas</t>
+        </is>
+      </c>
+      <c r="I138" s="45" t="inlineStr">
+        <is>
+          <t>Etanol aditivado V-Power 6,186 L a R$ 4,85/L — Posto Avenida Jacobina (Avenida Posto de Combustíveis LTDA, CNPJ 46.115.794/0001-30, Av. Orlando Oliveira Pires, 1430, Centro, Jacobina), NFC-e nº 000930413 série 002 de 19/10/2026 16:34. Pago R$ 30,00 em dinheiro.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
-      <c r="A139" s="17" t="n"/>
-      <c r="B139" s="18" t="n"/>
+      <c r="A139" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B139" s="18" t="inlineStr">
+        <is>
+          <t>Vale Edilânia</t>
+        </is>
+      </c>
       <c r="C139" s="18" t="n"/>
       <c r="D139" s="27" t="n"/>
       <c r="E139" s="18" t="n"/>
       <c r="F139" s="19" t="n"/>
-      <c r="G139" s="19" t="n"/>
-      <c r="H139" s="21" t="n"/>
-      <c r="I139" s="18" t="n"/>
+      <c r="G139" s="19" t="n">
+        <v>20</v>
+      </c>
+      <c r="H139" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I139" s="18" t="inlineStr">
+        <is>
+          <t>Vale de R$ 20,00 retirado do caixa em 19/10/2026.</t>
+        </is>
+      </c>
       <c r="J139" s="18" t="n"/>
     </row>
     <row r="140">

</xml_diff>

<commit_message>
Atualizacao do painel - 20/10/2026 12:17
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -57384,15 +57384,36 @@
       <c r="J139" s="18" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="44" t="n"/>
-      <c r="B140" s="45" t="n"/>
-      <c r="C140" s="45" t="n"/>
-      <c r="D140" s="46" t="n"/>
-      <c r="E140" s="45" t="n"/>
+      <c r="A140" s="44" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B140" s="45" t="inlineStr">
+        <is>
+          <t>Banco do Nordeste do Brasil</t>
+        </is>
+      </c>
+      <c r="C140" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D140" s="46" t="n">
+        <v>200</v>
+      </c>
+      <c r="E140" s="45" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F140" s="47" t="n"/>
       <c r="G140" s="48" t="n"/>
       <c r="H140" s="49" t="n"/>
       <c r="I140" s="45" t="n"/>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>EMP-0220</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 20/10/2026 18:21
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -57416,96 +57416,250 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="17" t="n"/>
-      <c r="B141" s="18" t="n"/>
+      <c r="A141" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B141" s="18" t="inlineStr">
+        <is>
+          <t>Receita Federal — Simples Nacional (DAS)</t>
+        </is>
+      </c>
       <c r="C141" s="18" t="n"/>
       <c r="D141" s="27" t="n"/>
       <c r="E141" s="18" t="n"/>
       <c r="F141" s="19" t="n"/>
-      <c r="G141" s="19" t="n"/>
-      <c r="H141" s="21" t="n"/>
-      <c r="I141" s="18" t="n"/>
+      <c r="G141" s="19" t="n">
+        <v>1430.03</v>
+      </c>
+      <c r="H141" s="21" t="inlineStr">
+        <is>
+          <t>Impostos e Taxas</t>
+        </is>
+      </c>
+      <c r="I141" s="18" t="inlineStr">
+        <is>
+          <t>DAS competência setembro/2026 (doc. 07.20.26292.9598304-7) — venc. 20/10/2026. Detalhe: IRPJ R$ 78,65 · CSLL R$ 50,05 · COFINS R$ 182,19 · PIS R$ 39,47 · INSS R$ 593,46 · ICMS (BA) R$ 486,21. Pago em 20/10/2026 pelo Banco do Nordeste.</t>
+        </is>
+      </c>
       <c r="J141" s="18" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="44" t="n"/>
-      <c r="B142" s="45" t="n"/>
-      <c r="C142" s="45" t="n"/>
-      <c r="D142" s="46" t="n"/>
-      <c r="E142" s="45" t="n"/>
+      <c r="A142" s="44" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B142" s="45" t="inlineStr">
+        <is>
+          <t>Sindicato dos Trabalhadores Rurais</t>
+        </is>
+      </c>
+      <c r="C142" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D142" s="46" t="n">
+        <v>140</v>
+      </c>
+      <c r="E142" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F142" s="47" t="n"/>
       <c r="G142" s="48" t="n"/>
       <c r="H142" s="49" t="n"/>
-      <c r="I142" s="45" t="n"/>
+      <c r="I142" s="45" t="inlineStr">
+        <is>
+          <t>Comprou na loja.</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>OUT-0087</t>
+        </is>
+      </c>
     </row>
     <row r="143">
-      <c r="A143" s="17" t="n"/>
-      <c r="B143" s="18" t="n"/>
-      <c r="C143" s="18" t="n"/>
-      <c r="D143" s="27" t="n"/>
-      <c r="E143" s="18" t="n"/>
+      <c r="A143" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B143" s="18" t="inlineStr">
+        <is>
+          <t>Magna dos Santos Carneiro Goncalves - Mirna</t>
+        </is>
+      </c>
+      <c r="C143" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D143" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E143" s="18" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F143" s="19" t="n"/>
       <c r="G143" s="19" t="n"/>
       <c r="H143" s="21" t="n"/>
       <c r="I143" s="18" t="n"/>
-      <c r="J143" s="18" t="n"/>
+      <c r="J143" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0488</t>
+        </is>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="44" t="n"/>
-      <c r="B144" s="45" t="n"/>
-      <c r="C144" s="45" t="n"/>
-      <c r="D144" s="46" t="n"/>
-      <c r="E144" s="45" t="n"/>
+      <c r="A144" s="44" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B144" s="45" t="inlineStr">
+        <is>
+          <t>Real Calçados Loja 1</t>
+        </is>
+      </c>
+      <c r="C144" s="45" t="inlineStr">
+        <is>
+          <t>2x Refil Everest + Refil Pro Life + 2x Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D144" s="46" t="n">
+        <v>515</v>
+      </c>
+      <c r="E144" s="45" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F144" s="47" t="n"/>
       <c r="G144" s="48" t="n"/>
       <c r="H144" s="49" t="n"/>
-      <c r="I144" s="45" t="n"/>
+      <c r="I144" s="45" t="inlineStr">
+        <is>
+          <t>Loja 1 — térreo: Refil Everest + Pré Filtro · 1º andar: Refil Everest · 2º andar: Refil Pro Life + Pré Filtro. Total R$ 540,00 com desconto de R$ 25,00.</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>EMP-0255</t>
+        </is>
+      </c>
     </row>
     <row r="145">
-      <c r="A145" s="17" t="n"/>
-      <c r="B145" s="18" t="n"/>
+      <c r="A145" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B145" s="18" t="inlineStr">
+        <is>
+          <t>Everest Refrigeração</t>
+        </is>
+      </c>
       <c r="C145" s="18" t="n"/>
       <c r="D145" s="27" t="n"/>
       <c r="E145" s="18" t="n"/>
       <c r="F145" s="19" t="n"/>
-      <c r="G145" s="19" t="n"/>
-      <c r="H145" s="21" t="n"/>
-      <c r="I145" s="18" t="n"/>
+      <c r="G145" s="19" t="n">
+        <v>874.6799999999999</v>
+      </c>
+      <c r="H145" s="21" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I145" s="18" t="inlineStr">
+        <is>
+          <t>Boleto doc. 379826 (emissão 22/06/2026) · parcela 4/5 — venc. 20/10/2026. Pago em 20/10/2026.</t>
+        </is>
+      </c>
       <c r="J145" s="18" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="44" t="n"/>
-      <c r="B146" s="45" t="n"/>
+      <c r="A146" s="44" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B146" s="45" t="inlineStr">
+        <is>
+          <t>FGTS Digital (GFD)</t>
+        </is>
+      </c>
       <c r="C146" s="45" t="n"/>
       <c r="D146" s="46" t="n"/>
       <c r="E146" s="45" t="n"/>
       <c r="F146" s="47" t="n"/>
-      <c r="G146" s="48" t="n"/>
-      <c r="H146" s="49" t="n"/>
-      <c r="I146" s="45" t="n"/>
+      <c r="G146" s="48" t="n">
+        <v>136</v>
+      </c>
+      <c r="H146" s="49" t="inlineStr">
+        <is>
+          <t>Impostos e Taxas</t>
+        </is>
+      </c>
+      <c r="I146" s="45" t="inlineStr">
+        <is>
+          <t>FGTS mensal — competência 09/2026. Venc. 20/10/2026, pago em 20/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
-      <c r="A147" s="17" t="n"/>
-      <c r="B147" s="18" t="n"/>
+      <c r="A147" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B147" s="18" t="inlineStr">
+        <is>
+          <t>Receita Federal — DARF / INSS</t>
+        </is>
+      </c>
       <c r="C147" s="18" t="n"/>
       <c r="D147" s="27" t="n"/>
       <c r="E147" s="18" t="n"/>
       <c r="F147" s="19" t="n"/>
-      <c r="G147" s="19" t="n"/>
-      <c r="H147" s="21" t="n"/>
-      <c r="I147" s="18" t="n"/>
+      <c r="G147" s="19" t="n">
+        <v>306.99</v>
+      </c>
+      <c r="H147" s="21" t="inlineStr">
+        <is>
+          <t>Impostos e Taxas</t>
+        </is>
+      </c>
+      <c r="I147" s="18" t="inlineStr">
+        <is>
+          <t>DARF / INSS — período de apuração setembro/2026. Venc. 20/10/2026, pago em 20/10/2026.</t>
+        </is>
+      </c>
       <c r="J147" s="18" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="44" t="n"/>
-      <c r="B148" s="45" t="n"/>
-      <c r="C148" s="45" t="n"/>
-      <c r="D148" s="46" t="n"/>
-      <c r="E148" s="45" t="n"/>
+      <c r="A148" s="44" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B148" s="45" t="inlineStr">
+        <is>
+          <t>Loja da Claro</t>
+        </is>
+      </c>
+      <c r="C148" s="45" t="inlineStr">
+        <is>
+          <t>Refil Lacqua</t>
+        </is>
+      </c>
+      <c r="D148" s="46" t="n">
+        <v>80</v>
+      </c>
+      <c r="E148" s="45" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F148" s="47" t="n"/>
       <c r="G148" s="48" t="n"/>
       <c r="H148" s="49" t="n"/>
-      <c r="I148" s="45" t="n"/>
+      <c r="I148" s="45" t="inlineStr">
+        <is>
+          <t>Cliente ainda não cadastrado na Planilha de Clientes.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="17" t="n"/>
@@ -68395,7 +68549,7 @@
       </c>
       <c r="E44" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F44" s="113">
@@ -68404,7 +68558,7 @@
       </c>
       <c r="G44" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/25528695-0. Linha digitável 34191.12259 52869.500307 52238.850003 1 16050000087468. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 379826 (emissão 22/06/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.373,40 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260633079641000132550020003798261298066249.</t>
+          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/25528695-0. Linha digitável 34191.12259 52869.500307 52238.850003 1 16050000087468. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 379826 (emissão 22/06/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.373,40 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260633079641000132550020003798261298066249. Pago em 20/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -69899,7 +70053,7 @@
       </c>
       <c r="E91" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F91" s="112">
@@ -69908,7 +70062,7 @@
       </c>
       <c r="G91" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Impostos e Taxas. Pagamento via QR Code Pix no documento original da guia (GFD).</t>
+          <t>Categoria: Impostos e Taxas. Pagamento via QR Code Pix no documento original da guia (GFD). Pago em 20/10/2026 — lançado em "Out 2026" como "FGTS Digital (GFD)".</t>
         </is>
       </c>
     </row>
@@ -69931,7 +70085,7 @@
       </c>
       <c r="E92" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F92" s="113">
@@ -69940,7 +70094,7 @@
       </c>
       <c r="G92" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Impostos e Taxas. Código de barras 858300000033 069903852621 930716262672 196301377104.</t>
+          <t>Categoria: Impostos e Taxas. Código de barras 858300000033 069903852621 930716262672 196301377104. Pago em 20/10/2026 — lançado em "Out 2026" como "Receita Federal — DARF / INSS".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao do painel - 20/10/2026 18:29
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -57454,11 +57454,11 @@
       </c>
       <c r="C142" s="45" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>2x Refil Everest</t>
         </is>
       </c>
       <c r="D142" s="46" t="n">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="E142" s="45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualizacao do painel - 21/10/2026 11:55
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -54239,7 +54239,7 @@
       </c>
       <c r="I38" s="45" t="inlineStr">
         <is>
-          <t>Boleto Itaú — NF-e 72869 (emissão 07/05/2026), parcela 5/5 (última), vencimento 04/10/2026 (domingo), pago em 05/10/2026.</t>
+          <t>Comprado: 100x Refil Everest + 50x Pré Filtro (NF-e 72869 de 07/05/2026, nota de R$ 4.904,13 em 5 boletos). Boleto Itaú — NF-e 72869 (emissão 07/05/2026), parcela 5/5 (última), vencimento 04/10/2026 (domingo), pago em 05/10/2026.</t>
         </is>
       </c>
     </row>
@@ -54506,7 +54506,7 @@
       </c>
       <c r="I47" s="18" t="inlineStr">
         <is>
-          <t>NF 133138 parcela 3/4 — boleto Itaú nosso número 109/00257851-4. Venc. 07/10/2026, pago antecipado em 06/10/2026.</t>
+          <t>Comprado: 10x Refil Fit PP 9.3/4" + 5x Refil Universal Rosca Curta + 5x Refil Universal Rosca Longa + 5x Refil Universal Rosca Média + 5x Refil Top Color + 3x Refil Acquatec + 5x Refil CP500 + 30x Refil Carbon Tech 9" + 20x Refil Plissado 9.3/4" (Poli Flu) + 5x Refil E3 Compacto + Carcaça Fit 9.3/4" Branca (rosca 1/2") (NF-e 133138 de 12/08/2026, nota de R$ 2.263,62 em 4 boletos). NF 133138 parcela 3/4 — boleto Itaú nosso número 109/00257851-4. Venc. 07/10/2026, pago antecipado em 06/10/2026.</t>
         </is>
       </c>
       <c r="J47" s="18" t="n"/>
@@ -54900,7 +54900,7 @@
       </c>
       <c r="I59" s="18" t="inlineStr">
         <is>
-          <t>Boleto Itaú — NF-e 73636 (emissão 10/06/2026), parcela 4/5, vencimento 08/10/2026, pago em 08/10/2026.</t>
+          <t>Comprado: 100x Refil Everest (NF-e 73636 de 10/06/2026, nota de R$ 4.394,61 em 5 boletos). Boleto Itaú — NF-e 73636 (emissão 10/06/2026), parcela 4/5, vencimento 08/10/2026, pago em 08/10/2026.</t>
         </is>
       </c>
       <c r="J59" s="18" t="n"/>
@@ -54928,7 +54928,7 @@
       </c>
       <c r="I60" s="45" t="inlineStr">
         <is>
-          <t>NF 133812 parcela 2 — boleto Itaú. Venc. 09/10/2026, pago antecipado em 08/10/2026.</t>
+          <t>Comprado: 30x Refil Pro Life + 2x Refil Carbon Block 9.3/4" + 15x Refil Carbon Tech 5" + 4x Refil Plissado 9.3/4" (Poli Flu) + 6x Carcaça Fit 9.3/4" Branca (rosca 3/4") + 5x Regulador de Pressão 3/8" (NF-e 133812 de 28/08/2026, nota de R$ 2.093,55 em 4 boletos). NF 133812 parcela 2 — boleto Itaú. Venc. 09/10/2026, pago antecipado em 08/10/2026.</t>
         </is>
       </c>
     </row>
@@ -56354,7 +56354,7 @@
       </c>
       <c r="I106" s="45" t="inlineStr">
         <is>
-          <t>Boleto doc. 74454 (emissão 17/07/2026) · parcela 3/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
+          <t>Comprado: 100x Refil Everest + 50x Pré Filtro (NF-e 74454 de 17/07/2026, nota de R$ 4.904,13 em 5 boletos). Boleto doc. 74454 (emissão 17/07/2026) · parcela 3/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
         </is>
       </c>
     </row>
@@ -56381,7 +56381,7 @@
       </c>
       <c r="I107" s="18" t="inlineStr">
         <is>
-          <t>Boleto doc. 381554 (emissão 17/07/2026) · parcela 3/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
+          <t>Comprado: Purificador Everest Fit Branco + Purificador Everest Fit Preto + 2x Purificador Everest Star Branco + Purificador Everest Star Preto + Purificador Everest Plus Prata (NF-e 381554 de 17/07/2026, nota de R$ 4.461,49 em 5 boletos). Boleto doc. 381554 (emissão 17/07/2026) · parcela 3/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
         </is>
       </c>
       <c r="J107" s="18" t="n"/>
@@ -56409,7 +56409,7 @@
       </c>
       <c r="I108" s="45" t="inlineStr">
         <is>
-          <t>Boleto doc. 386188 (emissão 15/09/2026) · parcela 1/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
+          <t>Comprado: 2x Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Star Prata (NF-e 386188 de 15/09/2026, nota de R$ 2.871,36 em 5 boletos). Boleto doc. 386188 (emissão 15/09/2026) · parcela 1/5 — venc. 15/10/2026. Pago em 15/10/2026.</t>
         </is>
       </c>
     </row>
@@ -56491,7 +56491,7 @@
       </c>
       <c r="I111" s="18" t="inlineStr">
         <is>
-          <t>Boleto doc. 377739 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago antecipado em 15/10/2026.</t>
+          <t>Comprado: Purificador Everest Slim Branco + Purificador Everest Slim Preto + Purificador Everest Plus Branco + Purificador Everest Star Branco + Purificador Everest Fit Branco + Purificador Everest Plus Prata (NF-e 377739 de 19/05/2026, nota de R$ 4.281,74 em 5 boletos). Boleto doc. 377739 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago antecipado em 15/10/2026.</t>
         </is>
       </c>
       <c r="J111" s="18" t="n"/>
@@ -56816,7 +56816,7 @@
       </c>
       <c r="I121" s="18" t="inlineStr">
         <is>
-          <t>Boleto doc. 377737 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago em 16/10/2026.</t>
+          <t>Comprado: 12x Conexão T + 30x Registro + 20x Botão Completo de Purificador + 30x Suporte de Parede (NF-e 377737 de 19/05/2026, nota de R$ 725,16 em 5 boletos). Boleto doc. 377737 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago em 16/10/2026.</t>
         </is>
       </c>
       <c r="J121" s="18" t="n"/>
@@ -56844,7 +56844,7 @@
       </c>
       <c r="I122" s="45" t="inlineStr">
         <is>
-          <t>Boleto doc. 377738 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago em 16/10/2026.</t>
+          <t>Comprado: Purificador Everest Plus Branco + Purificador Everest Plus Prata + Purificador Everest Slim Branco + 2x Purificador Everest Fit Prata + Purificador Everest Fit Preto (NF-e 377738 de 19/05/2026, nota de R$ 4.327,52 em 5 boletos). Boleto doc. 377738 (emissão 19/05/2026) · parcela 5/5 (última) — venc. 16/10/2026. Pago em 16/10/2026.</t>
         </is>
       </c>
     </row>
@@ -57570,7 +57570,7 @@
       </c>
       <c r="I145" s="18" t="inlineStr">
         <is>
-          <t>Boleto doc. 379826 (emissão 22/06/2026) · parcela 4/5 — venc. 20/10/2026. Pago em 20/10/2026.</t>
+          <t>Comprado: 2x Purificador Everest Slim Prata + 2x Purificador Everest Star Prata + Purificador Everest Star Branco + Purificador Everest Fit Branco (NF-e 379826 de 22/06/2026, nota de R$ 4.373,40 em 5 boletos). Boleto doc. 379826 (emissão 22/06/2026) · parcela 4/5 — venc. 20/10/2026. Pago em 20/10/2026.</t>
         </is>
       </c>
       <c r="J145" s="18" t="n"/>
@@ -67367,7 +67367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G166"/>
+  <dimension ref="A1:G171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="157" min="1" max="1"/>
@@ -67418,7 +67418,7 @@
     </row>
     <row r="5">
       <c r="A5" s="189">
-        <f>D97</f>
+        <f>D102</f>
         <v/>
       </c>
       <c r="C5" s="204">
@@ -67534,7 +67534,7 @@
       </c>
       <c r="G12" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Pago em 31/08/2026 — lançado em "Ago 2026" como "Eversoft" (R$ 878,93).</t>
+          <t>Comprado: 100x Refil Everest (NF-e 72153 de 02/04/2026, nota de R$ 4.394,61 em 5 boletos). Categoria: Fornecedores / Mercadoria. Pago em 31/08/2026 — lançado em "Ago 2026" como "Eversoft" (R$ 878,93).</t>
         </is>
       </c>
     </row>
@@ -67694,7 +67694,7 @@
       </c>
       <c r="G17" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Pago em 02/09/2026 — lançado em "Set 2026" como "Filtros Planeta Água".</t>
+          <t>Comprado: 5x Refil FP4 + 8x Refil Carbon Tech 5" + 120x Refil E3 + 90x Refil Pré-E3 + 10x Refil Top Multifilter + 4x Refil FPA16 (NF-e 131997 de 08/07/2026, nota de R$ 5.831,67 em 4 boletos). Categoria: Fornecedores / Mercadoria. Pago em 02/09/2026 — lançado em "Set 2026" como "Filtros Planeta Água".</t>
         </is>
       </c>
     </row>
@@ -67726,7 +67726,7 @@
       </c>
       <c r="G18" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Pago em 03/09/2026 — lançado em "Set 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: Purificador Everest Plus Prata + Purificador Everest Star Branco + Purificador Everest Star Preto + Purificador Everest Slim Prata + Purificador Everest Fit Branco (NF-e 374271 de 06/04/2026, nota de R$ 3.533,27 em 5 boletos). Categoria: Fornecedores / Mercadoria. Pago em 03/09/2026 — lançado em "Set 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -67758,7 +67758,7 @@
       </c>
       <c r="G19" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Pago em 04/09/2026 pelo Banco do Nordeste (DOC 5301) — lançado em "Set 2026" como "Eversoft" (R$ 980,83).</t>
+          <t>Comprado: 100x Refil Everest + 50x Pré Filtro (NF-e 72869 de 07/05/2026, nota de R$ 4.904,13 em 5 boletos). Categoria: Fornecedores / Mercadoria. Pago em 04/09/2026 pelo Banco do Nordeste (DOC 5301) — lançado em "Set 2026" como "Eversoft" (R$ 980,83).</t>
         </is>
       </c>
     </row>
@@ -67822,7 +67822,7 @@
       </c>
       <c r="G21" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Pago em 08/09/2026 — lançado em Set 2026 como "Eversoft".</t>
+          <t>Comprado: 100x Refil Everest (NF-e 73636 de 10/06/2026, nota de R$ 4.394,61 em 5 boletos). Categoria: Fornecedores / Mercadoria. Pago em 08/09/2026 — lançado em Set 2026 como "Eversoft".</t>
         </is>
       </c>
     </row>
@@ -67854,7 +67854,7 @@
       </c>
       <c r="G22" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7, nosso número 109/00257849-8. Pago em 09/09/2026 — lançado em "Set 2026" como "Filtros Planeta Água".</t>
+          <t>Comprado: 10x Refil Fit PP 9.3/4" + 5x Refil Universal Rosca Curta + 5x Refil Universal Rosca Longa + 5x Refil Universal Rosca Média + 5x Refil Top Color + 3x Refil Acquatec + 5x Refil CP500 + 30x Refil Carbon Tech 9" + 20x Refil Plissado 9.3/4" (Poli Flu) + 5x Refil E3 Compacto + Carcaça Fit 9.3/4" Branca (rosca 1/2") (NF-e 133138 de 12/08/2026, nota de R$ 2.263,62 em 4 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7, nosso número 109/00257849-8. Pago em 09/09/2026 — lançado em "Set 2026" como "Filtros Planeta Água".</t>
         </is>
       </c>
     </row>
@@ -68046,7 +68046,7 @@
       </c>
       <c r="G28" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/28638767-8. Linha digitável 34191.12283 63876.780303 55679.010003 5 15700000098083. Pago em 15/09/2026 pelo Banco do Nordeste (DOC 91607814) — lançado em "Set 2026" como "Eversoft".</t>
+          <t>Comprado: 100x Refil Everest + 50x Pré Filtro (NF-e 74454 de 17/07/2026, nota de R$ 4.904,13 em 5 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/28638767-8. Linha digitável 34191.12283 63876.780303 55679.010003 5 15700000098083. Pago em 15/09/2026 pelo Banco do Nordeste (DOC 91607814) — lançado em "Set 2026" como "Eversoft".</t>
         </is>
       </c>
     </row>
@@ -68078,7 +68078,7 @@
       </c>
       <c r="G29" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/33604587-0. Linha digitável 34191.12333 60458.700303 55679.010003 3 15800000094006. Após o vencimento: juros ao dia + multa de 2%. Pago em 24/09/2026 (antecipado, venc. 25/09) — lançado em "Set 2026" como "Eversoft".</t>
+          <t>Comprado: 100x Refil Everest + 30x Pré Filtro (NF-e 75472 de 26/08/2026, nota de R$ 4.700,32 em 5 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/33604587-0. Linha digitável 34191.12333 60458.700303 55679.010003 3 15800000094006. Após o vencimento: juros ao dia + multa de 2%. Pago em 24/09/2026 (antecipado, venc. 25/09) — lançado em "Set 2026" como "Eversoft".</t>
         </is>
       </c>
     </row>
@@ -68110,7 +68110,7 @@
       </c>
       <c r="G30" s="82" t="inlineStr">
         <is>
-          <t>Pago em 05/10/2026 — lançado em "Out 2026" como "Eversoft" (R$ 980,81). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/19915315-9. Linha digitável 34191.12192 91531.590304 55679.010003 3 15890000098081. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 72869 (emissão 07/05/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260508782043000188550060000728691612874239.</t>
+          <t>Comprado: 100x Refil Everest + 50x Pré Filtro (NF-e 72869 de 07/05/2026, nota de R$ 4.904,13 em 5 boletos). Pago em 05/10/2026 — lançado em "Out 2026" como "Eversoft" (R$ 980,81). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/19915315-9. Linha digitável 34191.12192 91531.590304 55679.010003 3 15890000098081. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 72869 (emissão 07/05/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260508782043000188550060000728691612874239.</t>
         </is>
       </c>
     </row>
@@ -68142,7 +68142,7 @@
       </c>
       <c r="G31" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Pago em 08/10/2026 — lançado em Out 2026 como "Eversoft". Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/24142201-6. Linha digitável 34191.12242 14220.160304 55679.010003 7 15930000087892. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 73636 (emissão 10/06/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.394,61 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260608782043000188550060000736361998873394.</t>
+          <t>Comprado: 100x Refil Everest (NF-e 73636 de 10/06/2026, nota de R$ 4.394,61 em 5 boletos). Categoria: Fornecedores / Mercadoria. Pago em 08/10/2026 — lançado em Out 2026 como "Eversoft". Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/24142201-6. Linha digitável 34191.12242 14220.160304 55679.010003 7 15930000087892. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 73636 (emissão 10/06/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.394,61 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260608782043000188550060000736361998873394.</t>
         </is>
       </c>
     </row>
@@ -68174,7 +68174,7 @@
       </c>
       <c r="G32" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/28638818-9. Linha digitável 34191.12283 63881.890303 55679.010003 2 16000000098083. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 74454 (emissão 17/07/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260708782043000188550060000744541603671381. Pago em 15/10/2026 — lançado em "Out 2026" como "Eversoft".</t>
+          <t>Comprado: 100x Refil Everest + 50x Pré Filtro (NF-e 74454 de 17/07/2026, nota de R$ 4.904,13 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/28638818-9. Linha digitável 34191.12283 63881.890303 55679.010003 2 16000000098083. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 74454 (emissão 17/07/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260708782043000188550060000744541603671381. Pago em 15/10/2026 — lançado em "Out 2026" como "Eversoft".</t>
         </is>
       </c>
     </row>
@@ -68206,7 +68206,7 @@
       </c>
       <c r="G33" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/33604663-9. Linha digitável 34191.12333 60466.390303 55679.010003 1 16100000094006. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 75472 (emissão 26/08/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.700,32 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 33260808782043000188550060000754721160252683.</t>
+          <t>Comprado: 100x Refil Everest + 30x Pré Filtro (NF-e 75472 de 26/08/2026, nota de R$ 4.700,32 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/33604663-9. Linha digitável 34191.12333 60466.390303 55679.010003 1 16100000094006. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 75472 (emissão 26/08/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.700,32 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 33260808782043000188550060000754721160252683.</t>
         </is>
       </c>
     </row>
@@ -68238,7 +68238,7 @@
       </c>
       <c r="G34" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/24142177-8. Linha digitável 34191.12242 14217.780304 55679.010003 4 16230000087893. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 73636 (emissão 10/06/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.394,61 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260608782043000188550060000736361998873394.</t>
+          <t>Comprado: 100x Refil Everest (NF-e 73636 de 10/06/2026, nota de R$ 4.394,61 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (Eversoft, CNPJ 08.782.043/0001-88). Nosso número 112/24142177-8. Linha digitável 34191.12242 14217.780304 55679.010003 4 16230000087893. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 73636 (emissão 10/06/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.394,61 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260608782043000188550060000736361998873394.</t>
         </is>
       </c>
     </row>
@@ -68270,7 +68270,7 @@
       </c>
       <c r="G35" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/28638136-6. Linha digitável 34191.12283 63813.660303 52238.850003 1 15700000089230. Pago em 15/09/2026 pelo Banco do Nordeste (DOC 91630932) — lançado em "Set 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: Purificador Everest Fit Branco + Purificador Everest Fit Preto + 2x Purificador Everest Star Branco + Purificador Everest Star Preto + Purificador Everest Plus Prata (NF-e 381554 de 17/07/2026, nota de R$ 4.461,49 em 5 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/28638136-6. Linha digitável 34191.12283 63813.660303 52238.850003 1 15700000089230. Pago em 15/09/2026 pelo Banco do Nordeste (DOC 91630932) — lançado em "Set 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68302,7 +68302,7 @@
       </c>
       <c r="G36" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21336084-8. Pago em 16/09/2026 — lançado em "Set 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: 12x Conexão T + 30x Registro + 20x Botão Completo de Purificador + 30x Suporte de Parede (NF-e 377737 de 19/05/2026, nota de R$ 725,16 em 5 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21336084-8. Pago em 16/09/2026 — lançado em "Set 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68334,7 +68334,7 @@
       </c>
       <c r="G37" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21336022-8. Pago em 16/09/2026 pelo Banco do Nordeste — lançado em "Set 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: Purificador Everest Plus Branco + Purificador Everest Plus Prata + Purificador Everest Slim Branco + 2x Purificador Everest Fit Prata + Purificador Everest Fit Preto (NF-e 377738 de 19/05/2026, nota de R$ 4.327,52 em 5 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21336022-8. Pago em 16/09/2026 pelo Banco do Nordeste — lançado em "Set 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68366,7 +68366,7 @@
       </c>
       <c r="G38" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21336008-7. Pago em 16/09/2026 — lançado em "Set 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: Purificador Everest Slim Branco + Purificador Everest Slim Preto + Purificador Everest Plus Branco + Purificador Everest Star Branco + Purificador Everest Fit Branco + Purificador Everest Plus Prata (NF-e 377739 de 19/05/2026, nota de R$ 4.281,74 em 5 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21336008-7. Pago em 16/09/2026 — lançado em "Set 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68398,7 +68398,7 @@
       </c>
       <c r="G39" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/25528668-7. Linha digitável 34191.12259 52866.870307 52238.850003 7 15750000087468. Após o vencimento: juros ao dia + multa de 2%. Pago em 21/09/2026 pelo Banco do Nordeste — lançado em "Set 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: 2x Purificador Everest Slim Prata + 2x Purificador Everest Star Prata + Purificador Everest Star Branco + Purificador Everest Fit Branco (NF-e 379826 de 22/06/2026, nota de R$ 4.373,40 em 5 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/25528668-7. Linha digitável 34191.12259 52866.870307 52238.850003 7 15750000087468. Após o vencimento: juros ao dia + multa de 2%. Pago em 21/09/2026 pelo Banco do Nordeste — lançado em "Set 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68430,7 +68430,7 @@
       </c>
       <c r="G40" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/28637900-6. Linha digitável 34191.12283 63790.060303 52238.850003 9 16000000089230. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 381554 (emissão 17/07/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.461,49 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260733079641000132550020003815541993407325. Pago em 15/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: Purificador Everest Fit Branco + Purificador Everest Fit Preto + 2x Purificador Everest Star Branco + Purificador Everest Star Preto + Purificador Everest Plus Prata (NF-e 381554 de 17/07/2026, nota de R$ 4.461,49 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/28637900-6. Linha digitável 34191.12283 63790.060303 52238.850003 9 16000000089230. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 381554 (emissão 17/07/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.461,49 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260733079641000132550020003815541993407325. Pago em 15/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68462,7 +68462,7 @@
       </c>
       <c r="G41" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335994-9. Linha digitável 34191.12218 33599.490308 52238.850003 1 16010000013932. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377737 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 725,16 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777371117471168. Pago em 16/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: 12x Conexão T + 30x Registro + 20x Botão Completo de Purificador + 30x Suporte de Parede (NF-e 377737 de 19/05/2026, nota de R$ 725,16 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335994-9. Linha digitável 34191.12218 33599.490308 52238.850003 1 16010000013932. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377737 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 725,16 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777371117471168. Pago em 16/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68494,7 +68494,7 @@
       </c>
       <c r="G42" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335634-1. Linha digitável 34191.12218 33563.410308 52238.850003 5 16010000086552. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377738 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.327,52 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777381143358478. Pago em 16/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: Purificador Everest Plus Branco + Purificador Everest Plus Prata + Purificador Everest Slim Branco + 2x Purificador Everest Fit Prata + Purificador Everest Fit Preto (NF-e 377738 de 19/05/2026, nota de R$ 4.327,52 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335634-1. Linha digitável 34191.12218 33563.410308 52238.850003 5 16010000086552. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377738 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.327,52 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777381143358478. Pago em 16/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68526,7 +68526,7 @@
       </c>
       <c r="G43" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335118-5. Linha digitável 34191.12218 33511.850308 52238.850003 9 16010000085634. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377739 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.281,74 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777391313049192. Pago em 15/10/2026 (antecipado, venc. 16/10) — lançado em "Out 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: Purificador Everest Slim Branco + Purificador Everest Slim Preto + Purificador Everest Plus Branco + Purificador Everest Star Branco + Purificador Everest Fit Branco + Purificador Everest Plus Prata (NF-e 377739 de 19/05/2026, nota de R$ 4.281,74 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/21335118-5. Linha digitável 34191.12218 33511.850308 52238.850003 9 16010000085634. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 377739 (emissão 19/05/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.281,74 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260533079641000132550020003777391313049192. Pago em 15/10/2026 (antecipado, venc. 16/10) — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68558,7 +68558,7 @@
       </c>
       <c r="G44" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/25528695-0. Linha digitável 34191.12259 52869.500307 52238.850003 1 16050000087468. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 379826 (emissão 22/06/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.373,40 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260633079641000132550020003798261298066249. Pago em 20/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: 2x Purificador Everest Slim Prata + 2x Purificador Everest Star Prata + Purificador Everest Star Branco + Purificador Everest Fit Branco (NF-e 379826 de 22/06/2026, nota de R$ 4.373,40 em 5 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/25528695-0. Linha digitável 34191.12259 52869.500307 52238.850003 1 16050000087468. Após o vencimento: juros ao dia + multa de 2%. | Conferido com o XML da NF-e nº 379826 (emissão 22/06/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.373,40 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260633079641000132550020003798261298066249. Pago em 20/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -68590,7 +68590,7 @@
       </c>
       <c r="G45" s="139" t="inlineStr">
         <is>
-          <t>PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 74454 (emissão 17/07/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 74454 (emissão 17/07/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260708782043000188550060000744541603671381.</t>
+          <t>Comprado: 100x Refil Everest + 50x Pré Filtro (NF-e 74454 de 17/07/2026, nota de R$ 4.904,13 em 5 boletos). PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 74454 (emissão 17/07/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 74454 (emissão 17/07/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260708782043000188550060000744541603671381.</t>
         </is>
       </c>
     </row>
@@ -68622,7 +68622,7 @@
       </c>
       <c r="G46" s="139" t="inlineStr">
         <is>
-          <t>PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 381554 (emissão 17/07/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 381554 (emissão 17/07/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.461,49 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260733079641000132550020003815541993407325.</t>
+          <t>Comprado: Purificador Everest Fit Branco + Purificador Everest Fit Preto + 2x Purificador Everest Star Branco + Purificador Everest Star Preto + Purificador Everest Plus Prata (NF-e 381554 de 17/07/2026, nota de R$ 4.461,49 em 5 boletos). PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 381554 (emissão 17/07/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 381554 (emissão 17/07/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.461,49 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260733079641000132550020003815541993407325.</t>
         </is>
       </c>
     </row>
@@ -68654,7 +68654,7 @@
       </c>
       <c r="G47" s="139" t="inlineStr">
         <is>
-          <t>PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 379826 (emissão 22/06/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 379826 (emissão 22/06/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.373,40 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260633079641000132550020003798261298066249.</t>
+          <t>Comprado: 2x Purificador Everest Slim Prata + 2x Purificador Everest Star Prata + Purificador Everest Star Branco + Purificador Everest Fit Branco (NF-e 379826 de 22/06/2026, nota de R$ 4.373,40 em 5 boletos). PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 379826 (emissão 22/06/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 379826 (emissão 22/06/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.373,40 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260633079641000132550020003798261298066249.</t>
         </is>
       </c>
     </row>
@@ -68686,7 +68686,7 @@
       </c>
       <c r="G48" s="139" t="inlineStr">
         <is>
-          <t>PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 75472 (emissão 26/08/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 75472 (emissão 26/08/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.700,32 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 33260808782043000188550060000754721160252683.</t>
+          <t>Comprado: 100x Refil Everest + 30x Pré Filtro (NF-e 75472 de 26/08/2026, nota de R$ 4.700,32 em 5 boletos). PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 75472 (emissão 26/08/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 75472 (emissão 26/08/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.700,32 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 33260808782043000188550060000754721160252683.</t>
         </is>
       </c>
     </row>
@@ -68718,7 +68718,7 @@
       </c>
       <c r="G49" s="139" t="inlineStr">
         <is>
-          <t>PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 381554 (emissão 17/07/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 381554 (emissão 17/07/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.461,49 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260733079641000132550020003815541993407325.</t>
+          <t>Comprado: Purificador Everest Fit Branco + Purificador Everest Fit Preto + 2x Purificador Everest Star Branco + Purificador Everest Star Preto + Purificador Everest Plus Prata (NF-e 381554 de 17/07/2026, nota de R$ 4.461,49 em 5 boletos). PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 381554 (emissão 17/07/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 381554 (emissão 17/07/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.461,49 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260733079641000132550020003815541993407325.</t>
         </is>
       </c>
     </row>
@@ -68750,7 +68750,7 @@
       </c>
       <c r="G50" s="139" t="inlineStr">
         <is>
-          <t>PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 74454 (emissão 17/07/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 74454 (emissão 17/07/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260708782043000188550060000744541603671381.</t>
+          <t>Comprado: 100x Refil Everest + 50x Pré Filtro (NF-e 74454 de 17/07/2026, nota de R$ 4.904,13 em 5 boletos). PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 74454 (emissão 17/07/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 74454 (emissão 17/07/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.904,13 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora FRACIONE TRANSPORTES EIRELI - ME. Chave da NF-e 33260708782043000188550060000744541603671381.</t>
         </is>
       </c>
     </row>
@@ -68782,7 +68782,7 @@
       </c>
       <c r="G51" s="139" t="inlineStr">
         <is>
-          <t>PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 75472 (emissão 26/08/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 75472 (emissão 26/08/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.700,32 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 33260808782043000188550060000754721160252683.</t>
+          <t>Comprado: 100x Refil Everest + 30x Pré Filtro (NF-e 75472 de 26/08/2026, nota de R$ 4.700,32 em 5 boletos). PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 75472 (emissão 26/08/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 75472 (emissão 26/08/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.700,32 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 33260808782043000188550060000754721160252683.</t>
         </is>
       </c>
     </row>
@@ -68814,7 +68814,7 @@
       </c>
       <c r="G52" s="139" t="inlineStr">
         <is>
-          <t>PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 75472 (emissão 26/08/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 75472 (emissão 26/08/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.700,32 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 33260808782043000188550060000754721160252683.</t>
+          <t>Comprado: 100x Refil Everest + 30x Pré Filtro (NF-e 75472 de 26/08/2026, nota de R$ 4.700,32 em 5 boletos). PREVISÃO (aguarda boleto) — o fornecedor ainda não emitiu este boleto. Valor e vencimento conforme as duplicatas da NF 75472 (emissão 26/08/2026). Categoria quando pagar: Fornecedores / Mercadoria. Conferir o boleto quando chegar. | Conferido com o XML da NF-e nº 75472 (emissão 26/08/2026): EVERSOFT INDUSTRIA E COMERCIO DE PLASTICOS LTDA, CNPJ 08.782.043/0001-88, RUA CARDOSO QUINTAO, 671, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 4.700,32 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 33260808782043000188550060000754721160252683.</t>
         </is>
       </c>
     </row>
@@ -68846,7 +68846,7 @@
       </c>
       <c r="G53" s="78" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109). Nosso número 109/00255359-0. Pago em 16/09/2026 pelo Banco do Nordeste — lançado em "Set 2026" como "Filtros Planeta Água".</t>
+          <t>Comprado: 5x Refil FP4 + 8x Refil Carbon Tech 5" + 120x Refil E3 + 90x Refil Pré-E3 + 10x Refil Top Multifilter + 4x Refil FPA16 (NF-e 131997 de 08/07/2026, nota de R$ 5.831,67 em 4 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109). Nosso número 109/00255359-0. Pago em 16/09/2026 pelo Banco do Nordeste — lançado em "Set 2026" como "Filtros Planeta Água".</t>
         </is>
       </c>
     </row>
@@ -68942,7 +68942,7 @@
       </c>
       <c r="G56" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109). Nosso número 109/00257850-6. Linha digitável 34191.09008 25785.061430 81531.550002 4 15780000053793. Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. Pago em 23/09/2026 — lançado em "Set 2026" como "Filtros Planeta Água".</t>
+          <t>Comprado: 10x Refil Fit PP 9.3/4" + 5x Refil Universal Rosca Curta + 5x Refil Universal Rosca Longa + 5x Refil Universal Rosca Média + 5x Refil Top Color + 3x Refil Acquatec + 5x Refil CP500 + 30x Refil Carbon Tech 9" + 20x Refil Plissado 9.3/4" (Poli Flu) + 5x Refil E3 Compacto + Carcaça Fit 9.3/4" Branca (rosca 1/2") (NF-e 133138 de 12/08/2026, nota de R$ 2.263,62 em 4 boletos). Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109). Nosso número 109/00257850-6. Linha digitável 34191.09008 25785.061430 81531.550002 4 15780000053793. Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. Pago em 23/09/2026 — lançado em "Set 2026" como "Filtros Planeta Água".</t>
         </is>
       </c>
     </row>
@@ -69006,7 +69006,7 @@
       </c>
       <c r="G58" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Pago em 06/10/2026 (antecipado, venc. 07/10) — lançado em "Out 2026" como "Filtros Planeta Água". Boleto Itaú 341-7 (carteira 109). Nosso número 109/00257851-4. Linha digitável 34191.09008 25785.141430 81531.550002 6 15920000053793. Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133138 (emissão 12/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.263,62 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 43260805097806000163550010001331381847671397.</t>
+          <t>Comprado: 10x Refil Fit PP 9.3/4" + 5x Refil Universal Rosca Curta + 5x Refil Universal Rosca Longa + 5x Refil Universal Rosca Média + 5x Refil Top Color + 3x Refil Acquatec + 5x Refil CP500 + 30x Refil Carbon Tech 9" + 20x Refil Plissado 9.3/4" (Poli Flu) + 5x Refil E3 Compacto + Carcaça Fit 9.3/4" Branca (rosca 1/2") (NF-e 133138 de 12/08/2026, nota de R$ 2.263,62 em 4 boletos). Categoria: Fornecedores / Mercadoria. Pago em 06/10/2026 (antecipado, venc. 07/10) — lançado em "Out 2026" como "Filtros Planeta Água". Boleto Itaú 341-7 (carteira 109). Nosso número 109/00257851-4. Linha digitável 34191.09008 25785.141430 81531.550002 6 15920000053793. Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133138 (emissão 12/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.263,62 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 43260805097806000163550010001331381847671397.</t>
         </is>
       </c>
     </row>
@@ -69038,7 +69038,7 @@
       </c>
       <c r="G59" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109). Nosso número 109/00257852-2. Linha digitável 34191.09008 25785.221430 81531.550002 6 16060000053793. Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133138 (emissão 12/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.263,62 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 43260805097806000163550010001331381847671397.</t>
+          <t>Comprado: 10x Refil Fit PP 9.3/4" + 5x Refil Universal Rosca Curta + 5x Refil Universal Rosca Longa + 5x Refil Universal Rosca Média + 5x Refil Top Color + 3x Refil Acquatec + 5x Refil CP500 + 30x Refil Carbon Tech 9" + 20x Refil Plissado 9.3/4" (Poli Flu) + 5x Refil E3 Compacto + Carcaça Fit 9.3/4" Branca (rosca 1/2") (NF-e 133138 de 12/08/2026, nota de R$ 2.263,62 em 4 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109). Nosso número 109/00257852-2. Linha digitável 34191.09008 25785.221430 81531.550002 6 16060000053793. Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133138 (emissão 12/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.263,62 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 43260805097806000163550010001331381847671397.</t>
         </is>
       </c>
     </row>
@@ -69134,7 +69134,7 @@
       </c>
       <c r="G62" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35841919. Linha digitável 34191.12358 84191.930308 52238.850003 3 16000000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116. Pago em 15/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
+          <t>Comprado: 2x Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Star Prata (NF-e 386188 de 15/09/2026, nota de R$ 2.871,36 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35841919. Linha digitável 34191.12358 84191.930308 52238.850003 3 16000000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116. Pago em 15/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>
@@ -69166,7 +69166,7 @@
       </c>
       <c r="G63" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35842013. Linha digitável 34191.12358 84201.340308 52238.850003 8 16300000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
+          <t>Comprado: 2x Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Star Prata (NF-e 386188 de 15/09/2026, nota de R$ 2.871,36 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35842013. Linha digitável 34191.12358 84201.340308 52238.850003 8 16300000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
         </is>
       </c>
     </row>
@@ -69198,7 +69198,7 @@
       </c>
       <c r="G64" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35841927. Linha digitável 34191.12358 84192.760308 52238.850003 8 16600000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
+          <t>Comprado: 2x Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Star Prata (NF-e 386188 de 15/09/2026, nota de R$ 2.871,36 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35841927. Linha digitável 34191.12358 84192.760308 52238.850003 8 16600000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
         </is>
       </c>
     </row>
@@ -69230,7 +69230,7 @@
       </c>
       <c r="G65" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35842031. Linha digitável 34191.12358 84203.160308 52238.850003 1 16900000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
+          <t>Comprado: 2x Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Star Prata (NF-e 386188 de 15/09/2026, nota de R$ 2.871,36 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35842031. Linha digitável 34191.12358 84203.160308 52238.850003 1 16900000057427. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
         </is>
       </c>
     </row>
@@ -69262,7 +69262,7 @@
       </c>
       <c r="G66" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35842128. Linha digitável 34191.12358 84212.800308 52238.850003 3 17200000057428. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
+          <t>Comprado: 2x Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Star Prata (NF-e 386188 de 15/09/2026, nota de R$ 2.871,36 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/35842128. Linha digitável 34191.12358 84212.800308 52238.850003 3 17200000057428. Boleto recebido por e-mail em 15/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386188". Após o vencimento: multa de 2% + juros de R$ 0,19 ao dia. | Conferido com o XML da NF-e nº 386188 (emissão 15/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 2.871,36 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003861881095200116.</t>
         </is>
       </c>
     </row>
@@ -69390,7 +69390,7 @@
       </c>
       <c r="G70" s="82" t="inlineStr">
         <is>
-          <t>Boleto substituído pela 2ª via emitida em 21/09/2026 (original: venc. 18/09/2026, R$ 591,12 — pagamento adiado para segunda 21/09). A 2ª via vale SOMENTE para 21/09/2026; se não pagar hoje, precisa gerar outra. Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/15315-5. Nosso número 109/00259098-5. Linha digitável 34191.09008 25909.801430 81531.550002 7 15760000059289. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. Pago em 21/09/2026 pelo Banco do Nordeste — lançado em "Set 2026" como "Filtros Planeta Água".</t>
+          <t>Comprado: 30x Refil Pro Life + 2x Refil Carbon Block 9.3/4" + 15x Refil Carbon Tech 5" + 4x Refil Plissado 9.3/4" (Poli Flu) + 6x Carcaça Fit 9.3/4" Branca (rosca 3/4") + 5x Regulador de Pressão 3/8" (NF-e 133812 de 28/08/2026, nota de R$ 2.093,55 em 4 boletos). Boleto substituído pela 2ª via emitida em 21/09/2026 (original: venc. 18/09/2026, R$ 591,12 — pagamento adiado para segunda 21/09). A 2ª via vale SOMENTE para 21/09/2026; se não pagar hoje, precisa gerar outra. Categoria: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/15315-5. Nosso número 109/00259098-5. Linha digitável 34191.09008 25909.801430 81531.550002 7 15760000059289. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. Pago em 21/09/2026 pelo Banco do Nordeste — lançado em "Set 2026" como "Filtros Planeta Água".</t>
         </is>
       </c>
     </row>
@@ -69422,7 +69422,7 @@
       </c>
       <c r="G71" s="82" t="inlineStr">
         <is>
-          <t>Categoria: Fornecedores / Mercadoria. Pago em 08/10/2026 — lançado em Out 2026 como "Filtros Planeta Água". Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/153155. Nosso número 109/00259099-8. Linha digitável 34191.09008 25909.981430 81531.550002 7 15940000050081. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133812 (emissão 28/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.093,55 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora JAMEF TRANSPORTES LIMITADA. Chave da NF-e 43260805097806000163550010001338121014276984.</t>
+          <t>Comprado: 30x Refil Pro Life + 2x Refil Carbon Block 9.3/4" + 15x Refil Carbon Tech 5" + 4x Refil Plissado 9.3/4" (Poli Flu) + 6x Carcaça Fit 9.3/4" Branca (rosca 3/4") + 5x Regulador de Pressão 3/8" (NF-e 133812 de 28/08/2026, nota de R$ 2.093,55 em 4 boletos). Categoria: Fornecedores / Mercadoria. Pago em 08/10/2026 — lançado em Out 2026 como "Filtros Planeta Água". Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/153155. Nosso número 109/00259099-8. Linha digitável 34191.09008 25909.981430 81531.550002 7 15940000050081. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133812 (emissão 28/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.093,55 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora JAMEF TRANSPORTES LIMITADA. Chave da NF-e 43260805097806000163550010001338121014276984.</t>
         </is>
       </c>
     </row>
@@ -69454,7 +69454,7 @@
       </c>
       <c r="G72" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/153155. Nosso número 109/00259100-4. Linha digitável 34191.09008 25910.041430 81531.550002 2 16150000050081. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133812 (emissão 28/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.093,55 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora JAMEF TRANSPORTES LIMITADA. Chave da NF-e 43260805097806000163550010001338121014276984.</t>
+          <t>Comprado: 30x Refil Pro Life + 2x Refil Carbon Block 9.3/4" + 15x Refil Carbon Tech 5" + 4x Refil Plissado 9.3/4" (Poli Flu) + 6x Carcaça Fit 9.3/4" Branca (rosca 3/4") + 5x Regulador de Pressão 3/8" (NF-e 133812 de 28/08/2026, nota de R$ 2.093,55 em 4 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/153155. Nosso número 109/00259100-4. Linha digitável 34191.09008 25910.041430 81531.550002 2 16150000050081. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133812 (emissão 28/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.093,55 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora JAMEF TRANSPORTES LIMITADA. Chave da NF-e 43260805097806000163550010001338121014276984.</t>
         </is>
       </c>
     </row>
@@ -69486,7 +69486,7 @@
       </c>
       <c r="G73" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/153155. Nosso número 109/00259101-2. Linha digitável 34191.09008 25910.121430 81531.550002 2 16360000050081. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133812 (emissão 28/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.093,55 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora JAMEF TRANSPORTES LIMITADA. Chave da NF-e 43260805097806000163550010001338121014276984.</t>
+          <t>Comprado: 30x Refil Pro Life + 2x Refil Carbon Block 9.3/4" + 15x Refil Carbon Tech 5" + 4x Refil Plissado 9.3/4" (Poli Flu) + 6x Carcaça Fit 9.3/4" Branca (rosca 3/4") + 5x Regulador de Pressão 3/8" (NF-e 133812 de 28/08/2026, nota de R$ 2.093,55 em 4 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109), agência/código beneficiário 1438/153155. Nosso número 109/00259101-2. Linha digitável 34191.09008 25910.121430 81531.550002 2 16360000050081. NF 133812 de 28/08/2026 (total R$ 2.093,55 em 4 parcelas). Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133812 (emissão 28/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.093,55 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora JAMEF TRANSPORTES LIMITADA. Chave da NF-e 43260805097806000163550010001338121014276984.</t>
         </is>
       </c>
     </row>
@@ -69550,7 +69550,7 @@
       </c>
       <c r="G75" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910774. Linha digitável 34191.12366 91077.460300 52238.850003 1 16080000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
+          <t>Comprado: Purificador Everest Fit Prata + Purificador Everest Slim Preto + Purificador Everest Star Preto + Purificador Everest Plus Preto (NF-e 386838 de 23/09/2026, nota de R$ 3.065,60 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910774. Linha digitável 34191.12366 91077.460300 52238.850003 1 16080000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
         </is>
       </c>
     </row>
@@ -69582,7 +69582,7 @@
       </c>
       <c r="G76" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910775. Linha digitável 34191.12366 91077.530300 52238.850003 6 16380000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
+          <t>Comprado: Purificador Everest Fit Prata + Purificador Everest Slim Preto + Purificador Everest Star Preto + Purificador Everest Plus Preto (NF-e 386838 de 23/09/2026, nota de R$ 3.065,60 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910775. Linha digitável 34191.12366 91077.530300 52238.850003 6 16380000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
         </is>
       </c>
     </row>
@@ -69614,7 +69614,7 @@
       </c>
       <c r="G77" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910730. Linha digitável 34191.12366 91073.080300 52238.850003 7 16680000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
+          <t>Comprado: Purificador Everest Fit Prata + Purificador Everest Slim Preto + Purificador Everest Star Preto + Purificador Everest Plus Preto (NF-e 386838 de 23/09/2026, nota de R$ 3.065,60 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910730. Linha digitável 34191.12366 91073.080300 52238.850003 7 16680000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
         </is>
       </c>
     </row>
@@ -69646,7 +69646,7 @@
       </c>
       <c r="G78" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910821. Linha digitável 34191.12366 91082.150300 52238.850003 9 16980000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
+          <t>Comprado: Purificador Everest Fit Prata + Purificador Everest Slim Preto + Purificador Everest Star Preto + Purificador Everest Plus Preto (NF-e 386838 de 23/09/2026, nota de R$ 3.065,60 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910821. Linha digitável 34191.12366 91082.150300 52238.850003 9 16980000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
         </is>
       </c>
     </row>
@@ -69678,7 +69678,7 @@
       </c>
       <c r="G79" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910791. Linha digitável 34191.12366 91079.100300 52238.850003 7 17280000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
+          <t>Comprado: Purificador Everest Fit Prata + Purificador Everest Slim Preto + Purificador Everest Star Preto + Purificador Everest Plus Preto (NF-e 386838 de 23/09/2026, nota de R$ 3.065,60 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910791. Linha digitável 34191.12366 91079.100300 52238.850003 7 17280000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
         </is>
       </c>
     </row>
@@ -69838,7 +69838,7 @@
       </c>
       <c r="G84" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879986. Linha digitável 34191.12374 87998.630302 52238.850003 9 16150000063352. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
+          <t>Comprado: 2x Purificador Everest Foz Branco + 2x Purificador Everest Foz Grafite (NF-e 387488 de 30/09/2026, nota de R$ 3.167,58 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879986. Linha digitável 34191.12374 87998.630302 52238.850003 9 16150000063352. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
         </is>
       </c>
     </row>
@@ -69870,7 +69870,7 @@
       </c>
       <c r="G85" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879706. Linha digitável 34191.12374 87970.650302 52238.850003 9 16450000063352. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
+          <t>Comprado: 2x Purificador Everest Foz Branco + 2x Purificador Everest Foz Grafite (NF-e 387488 de 30/09/2026, nota de R$ 3.167,58 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879706. Linha digitável 34191.12374 87970.650302 52238.850003 9 16450000063352. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
         </is>
       </c>
     </row>
@@ -69902,7 +69902,7 @@
       </c>
       <c r="G86" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879936. Linha digitável 34191.12374 87993.680302 52238.850003 5 16750000063352. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
+          <t>Comprado: 2x Purificador Everest Foz Branco + 2x Purificador Everest Foz Grafite (NF-e 387488 de 30/09/2026, nota de R$ 3.167,58 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879936. Linha digitável 34191.12374 87993.680302 52238.850003 5 16750000063352. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
         </is>
       </c>
     </row>
@@ -69934,7 +69934,7 @@
       </c>
       <c r="G87" s="78" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879730. Linha digitável 34191.12374 87973.050302 52238.850003 3 17050000063352. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
+          <t>Comprado: 2x Purificador Everest Foz Branco + 2x Purificador Everest Foz Grafite (NF-e 387488 de 30/09/2026, nota de R$ 3.167,58 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879730. Linha digitável 34191.12374 87973.050302 52238.850003 3 17050000063352. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
         </is>
       </c>
     </row>
@@ -69966,7 +69966,7 @@
       </c>
       <c r="G88" s="82" t="inlineStr">
         <is>
-          <t>Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879582. Linha digitável 34191.12374 87958.200302 52238.850003 2 17350000063350. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
+          <t>Comprado: 2x Purificador Everest Foz Branco + 2x Purificador Everest Foz Grafite (NF-e 387488 de 30/09/2026, nota de R$ 3.167,58 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/37879582. Linha digitável 34191.12374 87958.200302 52238.850003 2 17350000063350. Boleto recebido por e-mail em 30/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 387488". Após o vencimento: multa de 2% + juros de R$ 0,21 ao dia.</t>
         </is>
       </c>
     </row>
@@ -70163,1009 +70163,1009 @@
       </c>
     </row>
     <row r="95" s="157">
-      <c r="A95" s="86" t="inlineStr">
+      <c r="A95" s="82" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B95" s="82" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 388850 (emissão 19/10/2026) · parcela 1/5</t>
+        </is>
+      </c>
+      <c r="C95" s="81" t="n">
+        <v>46344</v>
+      </c>
+      <c r="D95" s="83" t="n">
+        <v>874.67</v>
+      </c>
+      <c r="E95" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F95" s="113">
+        <f>IF(OR($E95="Pago",$C95=""),"",MAX(0,TODAY()-$C95))</f>
+        <v/>
+      </c>
+      <c r="G95" s="82" t="inlineStr">
+        <is>
+          <t>Comprado: 2x Purificador Everest Star Branco + Purificador Everest Fit Prata + Purificador Everest Star Preto + Purificador Everest Star Prata + Purificador Everest Fit Preto (NF-e 388850 de 19/10/2026, nota de R$ 4.373,37 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/39837740. Linha digitável 34191.12390 83774.010306 52238.850003 8 16340000087467. Boleto recebido por e-mail em 19/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 388850". Após o vencimento: multa de 2% + juros de R$ 0,29 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" s="157">
+      <c r="A96" s="78" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B96" s="78" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 388850 (emissão 19/10/2026) · parcela 2/5</t>
+        </is>
+      </c>
+      <c r="C96" s="77" t="n">
+        <v>46374</v>
+      </c>
+      <c r="D96" s="79" t="n">
+        <v>874.67</v>
+      </c>
+      <c r="E96" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F96" s="112">
+        <f>IF(OR($E96="Pago",$C96=""),"",MAX(0,TODAY()-$C96))</f>
+        <v/>
+      </c>
+      <c r="G96" s="78" t="inlineStr">
+        <is>
+          <t>Comprado: 2x Purificador Everest Star Branco + Purificador Everest Fit Prata + Purificador Everest Star Preto + Purificador Everest Star Prata + Purificador Everest Fit Preto (NF-e 388850 de 19/10/2026, nota de R$ 4.373,37 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/39837859. Linha digitável 34191.12390 83785.990306 52238.850003 5 16640000087467. Boleto recebido por e-mail em 19/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 388850". Após o vencimento: multa de 2% + juros de R$ 0,29 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" s="157">
+      <c r="A97" s="82" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B97" s="82" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 388850 (emissão 19/10/2026) · parcela 3/5</t>
+        </is>
+      </c>
+      <c r="C97" s="81" t="n">
+        <v>46404</v>
+      </c>
+      <c r="D97" s="83" t="n">
+        <v>874.67</v>
+      </c>
+      <c r="E97" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F97" s="113">
+        <f>IF(OR($E97="Pago",$C97=""),"",MAX(0,TODAY()-$C97))</f>
+        <v/>
+      </c>
+      <c r="G97" s="82" t="inlineStr">
+        <is>
+          <t>Comprado: 2x Purificador Everest Star Branco + Purificador Everest Fit Prata + Purificador Everest Star Preto + Purificador Everest Star Prata + Purificador Everest Fit Preto (NF-e 388850 de 19/10/2026, nota de R$ 4.373,37 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/39837936. Linha digitável 34191.12390 83793.650306 52238.850003 1 16940000087467. Boleto recebido por e-mail em 19/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 388850". Após o vencimento: multa de 2% + juros de R$ 0,29 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" s="157">
+      <c r="A98" s="78" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B98" s="78" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 388850 (emissão 19/10/2026) · parcela 4/5</t>
+        </is>
+      </c>
+      <c r="C98" s="77" t="n">
+        <v>46434</v>
+      </c>
+      <c r="D98" s="79" t="n">
+        <v>874.67</v>
+      </c>
+      <c r="E98" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F98" s="112">
+        <f>IF(OR($E98="Pago",$C98=""),"",MAX(0,TODAY()-$C98))</f>
+        <v/>
+      </c>
+      <c r="G98" s="78" t="inlineStr">
+        <is>
+          <t>Comprado: 2x Purificador Everest Star Branco + Purificador Everest Fit Prata + Purificador Everest Star Preto + Purificador Everest Star Prata + Purificador Everest Fit Preto (NF-e 388850 de 19/10/2026, nota de R$ 4.373,37 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/39838041. Linha digitável 34191.12390 83804.130306 52238.850003 7 17240000087467. Boleto recebido por e-mail em 19/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 388850". Após o vencimento: multa de 2% + juros de R$ 0,29 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" s="157">
+      <c r="A99" s="82" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B99" s="82" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 388850 (emissão 19/10/2026) · parcela 5/5 (última)</t>
+        </is>
+      </c>
+      <c r="C99" s="81" t="n">
+        <v>46464</v>
+      </c>
+      <c r="D99" s="83" t="n">
+        <v>874.6900000000001</v>
+      </c>
+      <c r="E99" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F99" s="113">
+        <f>IF(OR($E99="Pago",$C99=""),"",MAX(0,TODAY()-$C99))</f>
+        <v/>
+      </c>
+      <c r="G99" s="82" t="inlineStr">
+        <is>
+          <t>Comprado: 2x Purificador Everest Star Branco + Purificador Everest Fit Prata + Purificador Everest Star Preto + Purificador Everest Star Prata + Purificador Everest Fit Preto (NF-e 388850 de 19/10/2026, nota de R$ 4.373,37 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/39837725. Linha digitável 34191.12390 83772.520306 52238.850003 9 17540000087469. Boleto recebido por e-mail em 19/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 388850". Após o vencimento: multa de 2% + juros de R$ 0,29 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" s="157">
+      <c r="A100" s="86" t="inlineStr">
         <is>
           <t>TOTAL A PAGAR — COM BOLETO EM MÃOS</t>
         </is>
       </c>
-      <c r="B95" s="86" t="n"/>
-      <c r="C95" s="114" t="n"/>
-      <c r="D95" s="115">
-        <f>SUMIF(E11:E94,"Pendente",D11:D94)</f>
-        <v/>
-      </c>
-      <c r="E95" s="116" t="n"/>
-      <c r="F95" s="116" t="n"/>
-      <c r="G95" s="86" t="n"/>
-    </row>
-    <row r="96" s="157">
-      <c r="A96" s="144" t="inlineStr">
+      <c r="B100" s="86" t="n"/>
+      <c r="C100" s="114" t="n"/>
+      <c r="D100" s="115">
+        <f>SUMIF(E11:E99,"Pendente",D11:D99)</f>
+        <v/>
+      </c>
+      <c r="E100" s="116" t="n"/>
+      <c r="F100" s="116" t="n"/>
+      <c r="G100" s="86" t="n"/>
+    </row>
+    <row r="101" s="157">
+      <c r="A101" s="144" t="inlineStr">
         <is>
           <t>PREVISTO — compromisso certo que ainda não está documentado</t>
         </is>
       </c>
-      <c r="B96" s="144" t="n"/>
-      <c r="C96" s="145" t="n"/>
-      <c r="D96" s="146">
-        <f>SUMIF(E11:E94,"Previsto",D11:D94)</f>
-        <v/>
-      </c>
-      <c r="E96" s="142" t="n"/>
-      <c r="F96" s="142" t="n"/>
-      <c r="G96" s="144" t="n"/>
-    </row>
-    <row r="97" s="157">
-      <c r="A97" s="86" t="inlineStr">
+      <c r="B101" s="144" t="n"/>
+      <c r="C101" s="145" t="n"/>
+      <c r="D101" s="146">
+        <f>SUMIF(E11:E99,"Previsto",D11:D99)</f>
+        <v/>
+      </c>
+      <c r="E101" s="142" t="n"/>
+      <c r="F101" s="142" t="n"/>
+      <c r="G101" s="144" t="n"/>
+    </row>
+    <row r="102" s="157">
+      <c r="A102" s="86" t="inlineStr">
         <is>
           <t>TOTAL GERAL A PAGAR (boletos + previsão)</t>
         </is>
       </c>
-      <c r="B97" s="86" t="n"/>
-      <c r="C97" s="114" t="n"/>
-      <c r="D97" s="115">
-        <f>D95+D96</f>
-        <v/>
-      </c>
-      <c r="E97" s="116" t="n"/>
-      <c r="F97" s="116" t="n"/>
-      <c r="G97" s="86" t="n"/>
-    </row>
-    <row r="98" ht="15.75" customHeight="1" s="157"/>
-    <row r="99" ht="15.75" customHeight="1" s="157">
-      <c r="A99" s="200" t="inlineStr">
+      <c r="B102" s="86" t="n"/>
+      <c r="C102" s="114" t="n"/>
+      <c r="D102" s="115">
+        <f>D100+D101</f>
+        <v/>
+      </c>
+      <c r="E102" s="116" t="n"/>
+      <c r="F102" s="116" t="n"/>
+      <c r="G102" s="86" t="n"/>
+    </row>
+    <row r="103" ht="15.75" customHeight="1" s="157"/>
+    <row r="104" ht="15.75" customHeight="1" s="157">
+      <c r="A104" s="200" t="inlineStr">
         <is>
           <t>CONTAS A RECEBER  —  vendas feitas e ainda não pagas</t>
         </is>
       </c>
     </row>
-    <row r="100" s="157">
-      <c r="A100" s="194" t="inlineStr">
+    <row r="105" s="157">
+      <c r="A105" s="194" t="inlineStr">
         <is>
           <t>Espelho das vendas marcadas como "Aguardando Pagamento" nas abas dos meses. Ao receber, mude a Forma de Pagamento na aba do mês E o Status aqui. A linha de conferência avisa se os dois deixarem de bater.</t>
         </is>
       </c>
     </row>
-    <row r="101" s="157">
-      <c r="A101" s="111" t="inlineStr">
+    <row r="106" s="157">
+      <c r="A106" s="111" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="B101" s="111" t="inlineStr">
+      <c r="B106" s="111" t="inlineStr">
         <is>
           <t>Produto / Referência</t>
         </is>
       </c>
-      <c r="C101" s="111" t="inlineStr">
+      <c r="C106" s="111" t="inlineStr">
         <is>
           <t>Data da Venda</t>
         </is>
       </c>
-      <c r="D101" s="111" t="inlineStr">
+      <c r="D106" s="111" t="inlineStr">
         <is>
           <t>Valor (R$)</t>
         </is>
       </c>
-      <c r="E101" s="111" t="inlineStr">
+      <c r="E106" s="111" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F101" s="111" t="inlineStr">
+      <c r="F106" s="111" t="inlineStr">
         <is>
           <t>Dias em Atraso</t>
         </is>
       </c>
-      <c r="G101" s="111" t="inlineStr">
+      <c r="G106" s="111" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
       </c>
     </row>
-    <row r="102" s="157">
-      <c r="A102" s="78" t="inlineStr">
+    <row r="107" s="157">
+      <c r="A107" s="78" t="inlineStr">
         <is>
           <t>Centro de Especialidades Odontomédicas</t>
         </is>
       </c>
-      <c r="B102" s="78" t="inlineStr">
+      <c r="B107" s="78" t="inlineStr">
         <is>
           <t>Refil Everest</t>
         </is>
       </c>
-      <c r="C102" s="77" t="n">
+      <c r="C107" s="77" t="n">
         <v>46239</v>
       </c>
-      <c r="D102" s="79" t="n">
+      <c r="D107" s="79" t="n">
         <v>140</v>
       </c>
-      <c r="E102" s="112" t="inlineStr">
+      <c r="E107" s="112" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="F102" s="112">
-        <f>IF(OR($E102="Recebido",$C102=""),"",MAX(0,TODAY()-$C102))</f>
-        <v/>
-      </c>
-      <c r="G102" s="78" t="n"/>
-    </row>
-    <row r="103" s="157">
-      <c r="A103" s="82" t="inlineStr">
+      <c r="F107" s="112">
+        <f>IF(OR($E107="Recebido",$C107=""),"",MAX(0,TODAY()-$C107))</f>
+        <v/>
+      </c>
+      <c r="G107" s="78" t="n"/>
+    </row>
+    <row r="108" s="157">
+      <c r="A108" s="82" t="inlineStr">
         <is>
           <t>Supermercado Brasil</t>
         </is>
       </c>
-      <c r="B103" s="82" t="inlineStr">
+      <c r="B108" s="82" t="inlineStr">
         <is>
           <t>2x Refil Pro Life</t>
         </is>
       </c>
-      <c r="C103" s="81" t="n">
+      <c r="C108" s="81" t="n">
         <v>46239</v>
       </c>
-      <c r="D103" s="83" t="n">
+      <c r="D108" s="83" t="n">
         <v>280</v>
       </c>
-      <c r="E103" s="113" t="inlineStr">
+      <c r="E108" s="113" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="F103" s="113">
-        <f>IF(OR($E103="Recebido",$C103=""),"",MAX(0,TODAY()-$C103))</f>
-        <v/>
-      </c>
-      <c r="G103" s="82" t="n"/>
-    </row>
-    <row r="104" s="157">
-      <c r="A104" s="78" t="inlineStr">
+      <c r="F108" s="113">
+        <f>IF(OR($E108="Recebido",$C108=""),"",MAX(0,TODAY()-$C108))</f>
+        <v/>
+      </c>
+      <c r="G108" s="82" t="n"/>
+    </row>
+    <row r="109" s="157">
+      <c r="A109" s="78" t="inlineStr">
         <is>
           <t>Tropical Motos LTDA</t>
         </is>
       </c>
-      <c r="B104" s="78" t="inlineStr">
+      <c r="B109" s="78" t="inlineStr">
         <is>
           <t>3x Refil Everest + Refil Pro Life + 3x Pré Filtro + Válvula Reguladora de Pressão</t>
         </is>
       </c>
-      <c r="C104" s="77" t="n">
+      <c r="C109" s="77" t="n">
         <v>46245</v>
       </c>
-      <c r="D104" s="79" t="n">
+      <c r="D109" s="79" t="n">
         <v>820</v>
       </c>
-      <c r="E104" s="112" t="inlineStr">
+      <c r="E109" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F104" s="112">
-        <f>IF(OR($E104="Recebido",$C104=""),"",MAX(0,TODAY()-$C104))</f>
-        <v/>
-      </c>
-      <c r="G104" s="78" t="inlineStr">
+      <c r="F109" s="112">
+        <f>IF(OR($E109="Recebido",$C109=""),"",MAX(0,TODAY()-$C109))</f>
+        <v/>
+      </c>
+      <c r="G109" s="78" t="inlineStr">
         <is>
           <t>Recebido via TED em 25/08/2026. NF conferida: valor correto é R$820 (faltava a válvula no lançamento original de R$740).</t>
         </is>
       </c>
     </row>
-    <row r="105" s="157">
-      <c r="A105" s="82" t="inlineStr">
+    <row r="110" s="157">
+      <c r="A110" s="82" t="inlineStr">
         <is>
           <t>Free Way</t>
         </is>
       </c>
-      <c r="B105" s="82" t="inlineStr">
+      <c r="B110" s="82" t="inlineStr">
         <is>
           <t>5x Refil Everest</t>
         </is>
       </c>
-      <c r="C105" s="81" t="n">
+      <c r="C110" s="81" t="n">
         <v>46251</v>
       </c>
-      <c r="D105" s="83" t="n">
+      <c r="D110" s="83" t="n">
         <v>700</v>
       </c>
-      <c r="E105" s="113" t="inlineStr">
+      <c r="E110" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F105" s="113">
-        <f>IF(OR($E105="Recebido",$C105=""),"",MAX(0,TODAY()-$C105))</f>
-        <v/>
-      </c>
-      <c r="G105" s="82" t="inlineStr">
+      <c r="F110" s="113">
+        <f>IF(OR($E110="Recebido",$C110=""),"",MAX(0,TODAY()-$C110))</f>
+        <v/>
+      </c>
+      <c r="G110" s="82" t="inlineStr">
         <is>
           <t>Recebido via TED em 02/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="106" s="157">
-      <c r="A106" s="78" t="inlineStr">
+    <row r="111" s="157">
+      <c r="A111" s="78" t="inlineStr">
         <is>
           <t>Neli Sena Rego</t>
         </is>
       </c>
-      <c r="B106" s="78" t="inlineStr">
+      <c r="B111" s="78" t="inlineStr">
         <is>
           <t>Refil Pro Life</t>
         </is>
       </c>
-      <c r="C106" s="77" t="n">
+      <c r="C111" s="77" t="n">
         <v>46254</v>
       </c>
-      <c r="D106" s="79" t="n">
+      <c r="D111" s="79" t="n">
         <v>140</v>
       </c>
-      <c r="E106" s="112" t="inlineStr">
+      <c r="E111" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F106" s="112">
-        <f>IF(OR($E106="Recebido",$C106=""),"",MAX(0,TODAY()-$C106))</f>
-        <v/>
-      </c>
-      <c r="G106" s="78" t="inlineStr">
+      <c r="F111" s="112">
+        <f>IF(OR($E111="Recebido",$C111=""),"",MAX(0,TODAY()-$C111))</f>
+        <v/>
+      </c>
+      <c r="G111" s="78" t="inlineStr">
         <is>
           <t>Recebido em dinheiro em 01/09/2026 (R$ 170,00 pelas duas vendas)</t>
         </is>
       </c>
     </row>
-    <row r="107" s="157">
-      <c r="A107" s="82" t="inlineStr">
+    <row r="112" s="157">
+      <c r="A112" s="82" t="inlineStr">
         <is>
           <t>Neli Sena Rego</t>
         </is>
       </c>
-      <c r="B107" s="82" t="inlineStr">
+      <c r="B112" s="82" t="inlineStr">
         <is>
           <t>Conexão + Mangueira</t>
         </is>
       </c>
-      <c r="C107" s="81" t="n">
+      <c r="C112" s="81" t="n">
         <v>46255</v>
       </c>
-      <c r="D107" s="83" t="n">
+      <c r="D112" s="83" t="n">
         <v>40</v>
       </c>
-      <c r="E107" s="113" t="inlineStr">
+      <c r="E112" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F107" s="113">
-        <f>IF(OR($E107="Recebido",$C107=""),"",MAX(0,TODAY()-$C107))</f>
-        <v/>
-      </c>
-      <c r="G107" s="82" t="inlineStr">
+      <c r="F112" s="113">
+        <f>IF(OR($E112="Recebido",$C112=""),"",MAX(0,TODAY()-$C112))</f>
+        <v/>
+      </c>
+      <c r="G112" s="82" t="inlineStr">
         <is>
           <t>Recebido em dinheiro em 01/09/2026 (R$ 170,00 pelas duas vendas)</t>
         </is>
       </c>
     </row>
-    <row r="108" s="157">
-      <c r="A108" s="78" t="inlineStr">
+    <row r="113" s="157">
+      <c r="A113" s="78" t="inlineStr">
         <is>
           <t>Lapec</t>
         </is>
       </c>
-      <c r="B108" s="78" t="inlineStr">
+      <c r="B113" s="78" t="inlineStr">
         <is>
           <t>4x Refil Everest</t>
         </is>
       </c>
-      <c r="C108" s="77" t="n">
+      <c r="C113" s="77" t="n">
         <v>46258</v>
       </c>
-      <c r="D108" s="79" t="n">
+      <c r="D113" s="79" t="n">
         <v>480</v>
       </c>
-      <c r="E108" s="112" t="inlineStr">
+      <c r="E113" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F108" s="112">
-        <f>IF(OR($E108="Recebido",$C108=""),"",MAX(0,TODAY()-$C108))</f>
-        <v/>
-      </c>
-      <c r="G108" s="78" t="inlineStr">
+      <c r="F113" s="112">
+        <f>IF(OR($E113="Recebido",$C113=""),"",MAX(0,TODAY()-$C113))</f>
+        <v/>
+      </c>
+      <c r="G113" s="78" t="inlineStr">
         <is>
           <t>Recebido em dinheiro em 08/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
-    <row r="109" s="157">
-      <c r="A109" s="82" t="inlineStr">
+    <row r="114" s="157">
+      <c r="A114" s="82" t="inlineStr">
         <is>
           <t>Cícero Lima</t>
         </is>
       </c>
-      <c r="B109" s="82" t="inlineStr">
+      <c r="B114" s="82" t="inlineStr">
         <is>
           <t>Refil Everest</t>
         </is>
       </c>
-      <c r="C109" s="81" t="n">
+      <c r="C114" s="81" t="n">
         <v>46261</v>
       </c>
-      <c r="D109" s="83" t="n">
+      <c r="D114" s="83" t="n">
         <v>140</v>
       </c>
-      <c r="E109" s="113" t="inlineStr">
+      <c r="E114" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F109" s="113">
-        <f>IF(OR($E109="Recebido",$C109=""),"",MAX(0,TODAY()-$C109))</f>
-        <v/>
-      </c>
-      <c r="G109" s="82" t="inlineStr">
+      <c r="F114" s="113">
+        <f>IF(OR($E114="Recebido",$C114=""),"",MAX(0,TODAY()-$C114))</f>
+        <v/>
+      </c>
+      <c r="G114" s="82" t="inlineStr">
         <is>
           <t>Recebido via Pix em 27/08/2026</t>
         </is>
       </c>
     </row>
-    <row r="110" s="157">
-      <c r="A110" s="78" t="inlineStr">
+    <row r="115" s="157">
+      <c r="A115" s="78" t="inlineStr">
         <is>
           <t>Promotoria Regional de Jacobina</t>
         </is>
       </c>
-      <c r="B110" s="78" t="inlineStr">
+      <c r="B115" s="78" t="inlineStr">
         <is>
           <t>2x Carcaça 9" + 2x Refil Plissado 9" + Conexão Reta Rosca</t>
         </is>
       </c>
-      <c r="C110" s="77" t="n">
+      <c r="C115" s="77" t="n">
         <v>46261</v>
       </c>
-      <c r="D110" s="79" t="n">
+      <c r="D115" s="79" t="n">
         <v>470</v>
       </c>
-      <c r="E110" s="112" t="inlineStr">
+      <c r="E115" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F110" s="112">
-        <f>IF(OR($E110="Recebido",$C110=""),"",MAX(0,TODAY()-$C110))</f>
-        <v/>
-      </c>
-      <c r="G110" s="78" t="inlineStr">
+      <c r="F115" s="112">
+        <f>IF(OR($E115="Recebido",$C115=""),"",MAX(0,TODAY()-$C115))</f>
+        <v/>
+      </c>
+      <c r="G115" s="78" t="inlineStr">
         <is>
           <t>Pago em 28/08/2026 em duas formas: R$ 270,00 Pix + R$ 200,00 crédito 2x</t>
         </is>
       </c>
     </row>
-    <row r="111" s="157">
-      <c r="A111" s="82" t="inlineStr">
+    <row r="116" s="157">
+      <c r="A116" s="82" t="inlineStr">
         <is>
           <t>Lucas Souza</t>
         </is>
       </c>
-      <c r="B111" s="82" t="inlineStr">
+      <c r="B116" s="82" t="inlineStr">
         <is>
           <t>Refil Everest + Pré Filtro</t>
         </is>
       </c>
-      <c r="C111" s="81" t="n">
+      <c r="C116" s="81" t="n">
         <v>46261</v>
       </c>
-      <c r="D111" s="83" t="n">
+      <c r="D116" s="83" t="n">
         <v>200</v>
       </c>
-      <c r="E111" s="113" t="inlineStr">
+      <c r="E116" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F111" s="113">
-        <f>IF(OR($E111="Recebido",$C111=""),"",MAX(0,TODAY()-$C111))</f>
-        <v/>
-      </c>
-      <c r="G111" s="82" t="inlineStr">
+      <c r="F116" s="113">
+        <f>IF(OR($E116="Recebido",$C116=""),"",MAX(0,TODAY()-$C116))</f>
+        <v/>
+      </c>
+      <c r="G116" s="82" t="inlineStr">
         <is>
           <t>Recebido em dinheiro em 03/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
-    <row r="112" s="157">
-      <c r="A112" s="78" t="inlineStr">
+    <row r="117" s="157">
+      <c r="A117" s="78" t="inlineStr">
         <is>
           <t>FG Boa Vista (Recife/PE)</t>
         </is>
       </c>
-      <c r="B112" s="78" t="inlineStr">
+      <c r="B117" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C112" s="77" t="n">
+      <c r="C117" s="77" t="n">
         <v>46261</v>
       </c>
-      <c r="D112" s="79" t="n">
+      <c r="D117" s="79" t="n">
         <v>1008.8</v>
       </c>
-      <c r="E112" s="112" t="inlineStr">
+      <c r="E117" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F112" s="112">
-        <f>IF(OR($E112="Recebido",$C112=""),"",MAX(0,TODAY()-$C112))</f>
-        <v/>
-      </c>
-      <c r="G112" s="78" t="inlineStr">
+      <c r="F117" s="112">
+        <f>IF(OR($E117="Recebido",$C117=""),"",MAX(0,TODAY()-$C117))</f>
+        <v/>
+      </c>
+      <c r="G117" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.280 · recebido em 30/08/2026 (Nota Paga no portal V360)</t>
         </is>
       </c>
     </row>
-    <row r="113" s="157">
-      <c r="A113" s="82" t="inlineStr">
+    <row r="118" s="157">
+      <c r="A118" s="82" t="inlineStr">
         <is>
           <t>UNIFG Guanambi (Guanambi/BA)</t>
         </is>
       </c>
-      <c r="B113" s="82" t="inlineStr">
+      <c r="B118" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C113" s="81" t="n">
+      <c r="C118" s="81" t="n">
         <v>46261</v>
       </c>
-      <c r="D113" s="83" t="n">
+      <c r="D118" s="83" t="n">
         <v>4534.75</v>
       </c>
-      <c r="E113" s="113" t="inlineStr">
+      <c r="E118" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F113" s="113">
-        <f>IF(OR($E113="Recebido",$C113=""),"",MAX(0,TODAY()-$C113))</f>
-        <v/>
-      </c>
-      <c r="G113" s="82" t="inlineStr">
+      <c r="F118" s="113">
+        <f>IF(OR($E118="Recebido",$C118=""),"",MAX(0,TODAY()-$C118))</f>
+        <v/>
+      </c>
+      <c r="G118" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.281 · recebido em 30/08/2026 (Nota Paga no portal V360)</t>
         </is>
       </c>
     </row>
-    <row r="114" s="157">
-      <c r="A114" s="78" t="inlineStr">
+    <row r="119" s="157">
+      <c r="A119" s="78" t="inlineStr">
         <is>
           <t>UNP Zona Norte (Natal/RN)</t>
         </is>
       </c>
-      <c r="B114" s="78" t="inlineStr">
+      <c r="B119" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C114" s="77" t="n">
+      <c r="C119" s="77" t="n">
         <v>46261</v>
       </c>
-      <c r="D114" s="79" t="n">
+      <c r="D119" s="79" t="n">
         <v>870</v>
       </c>
-      <c r="E114" s="112" t="inlineStr">
+      <c r="E119" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F114" s="112">
-        <f>IF(OR($E114="Recebido",$C114=""),"",MAX(0,TODAY()-$C114))</f>
-        <v/>
-      </c>
-      <c r="G114" s="78" t="inlineStr">
+      <c r="F119" s="112">
+        <f>IF(OR($E119="Recebido",$C119=""),"",MAX(0,TODAY()-$C119))</f>
+        <v/>
+      </c>
+      <c r="G119" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.282 · recebido em 30/08/2026 (Nota Paga no portal V360)</t>
         </is>
       </c>
     </row>
-    <row r="115" s="157">
-      <c r="A115" s="82" t="inlineStr">
+    <row r="120" s="157">
+      <c r="A120" s="82" t="inlineStr">
         <is>
           <t>UNP Caicó (Caicó/RN)</t>
         </is>
       </c>
-      <c r="B115" s="82" t="inlineStr">
+      <c r="B120" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C115" s="81" t="n">
+      <c r="C120" s="81" t="n">
         <v>46261</v>
       </c>
-      <c r="D115" s="83" t="n">
+      <c r="D120" s="83" t="n">
         <v>440</v>
       </c>
-      <c r="E115" s="113" t="inlineStr">
+      <c r="E120" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F115" s="113">
-        <f>IF(OR($E115="Recebido",$C115=""),"",MAX(0,TODAY()-$C115))</f>
-        <v/>
-      </c>
-      <c r="G115" s="82" t="inlineStr">
+      <c r="F120" s="113">
+        <f>IF(OR($E120="Recebido",$C120=""),"",MAX(0,TODAY()-$C120))</f>
+        <v/>
+      </c>
+      <c r="G120" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.283 · recebido via Pix em 27/08/2026</t>
         </is>
       </c>
     </row>
-    <row r="116" s="157">
-      <c r="A116" s="78" t="inlineStr">
+    <row r="121" s="157">
+      <c r="A121" s="78" t="inlineStr">
         <is>
           <t>AGES Irecê (Irecê/BA)</t>
         </is>
       </c>
-      <c r="B116" s="78" t="inlineStr">
+      <c r="B121" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C116" s="77" t="n">
+      <c r="C121" s="77" t="n">
         <v>46269</v>
       </c>
-      <c r="D116" s="79" t="n">
+      <c r="D121" s="79" t="n">
         <v>1338.6</v>
       </c>
-      <c r="E116" s="112" t="inlineStr">
+      <c r="E121" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F116" s="112">
-        <f>IF(OR($E116="Recebido",$C116=""),"",MAX(0,TODAY()-$C116))</f>
-        <v/>
-      </c>
-      <c r="G116" s="78" t="inlineStr">
+      <c r="F121" s="112">
+        <f>IF(OR($E121="Recebido",$C121=""),"",MAX(0,TODAY()-$C121))</f>
+        <v/>
+      </c>
+      <c r="G121" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.294 · recebido via Pix em 04/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="117" s="157">
-      <c r="A117" s="82" t="inlineStr">
+    <row r="122" s="157">
+      <c r="A122" s="82" t="inlineStr">
         <is>
           <t>CIS Irecê (Irecê/BA)</t>
         </is>
       </c>
-      <c r="B117" s="82" t="inlineStr">
+      <c r="B122" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C117" s="81" t="n">
+      <c r="C122" s="81" t="n">
         <v>46269</v>
       </c>
-      <c r="D117" s="83" t="n">
+      <c r="D122" s="83" t="n">
         <v>1358</v>
       </c>
-      <c r="E117" s="113" t="inlineStr">
+      <c r="E122" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F117" s="113">
-        <f>IF(OR($E117="Recebido",$C117=""),"",MAX(0,TODAY()-$C117))</f>
-        <v/>
-      </c>
-      <c r="G117" s="82" t="inlineStr">
+      <c r="F122" s="113">
+        <f>IF(OR($E122="Recebido",$C122=""),"",MAX(0,TODAY()-$C122))</f>
+        <v/>
+      </c>
+      <c r="G122" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.295 · recebido via Pix em 04/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="118" s="157">
-      <c r="A118" s="78" t="inlineStr">
+    <row r="123" s="157">
+      <c r="A123" s="78" t="inlineStr">
         <is>
           <t>AGES Senhor do Bonfim (S. do Bonfim/BA)</t>
         </is>
       </c>
-      <c r="B118" s="78" t="inlineStr">
+      <c r="B123" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C118" s="77" t="n">
+      <c r="C123" s="77" t="n">
         <v>46270</v>
       </c>
-      <c r="D118" s="79" t="n">
+      <c r="D123" s="79" t="n">
         <v>649.9</v>
       </c>
-      <c r="E118" s="112" t="inlineStr">
+      <c r="E123" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F118" s="112">
-        <f>IF(OR($E118="Recebido",$C118=""),"",MAX(0,TODAY()-$C118))</f>
-        <v/>
-      </c>
-      <c r="G118" s="78" t="inlineStr">
+      <c r="F123" s="112">
+        <f>IF(OR($E123="Recebido",$C123=""),"",MAX(0,TODAY()-$C123))</f>
+        <v/>
+      </c>
+      <c r="G123" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.298 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="119" s="157">
-      <c r="A119" s="82" t="inlineStr">
+    <row r="124" s="157">
+      <c r="A124" s="82" t="inlineStr">
         <is>
           <t>CIS Senhor do Bonfim (S. do Bonfim/BA)</t>
         </is>
       </c>
-      <c r="B119" s="82" t="inlineStr">
+      <c r="B124" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C119" s="81" t="n">
+      <c r="C124" s="81" t="n">
         <v>46270</v>
       </c>
-      <c r="D119" s="83" t="n">
+      <c r="D124" s="83" t="n">
         <v>562.6</v>
       </c>
-      <c r="E119" s="113" t="inlineStr">
+      <c r="E124" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F119" s="113">
-        <f>IF(OR($E119="Recebido",$C119=""),"",MAX(0,TODAY()-$C119))</f>
-        <v/>
-      </c>
-      <c r="G119" s="82" t="inlineStr">
+      <c r="F124" s="113">
+        <f>IF(OR($E124="Recebido",$C124=""),"",MAX(0,TODAY()-$C124))</f>
+        <v/>
+      </c>
+      <c r="G124" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.299 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="120" s="157">
-      <c r="A120" s="78" t="inlineStr">
+    <row r="125" s="157">
+      <c r="A125" s="78" t="inlineStr">
         <is>
           <t>AGES Paripiranga (Paripiranga/BA)</t>
         </is>
       </c>
-      <c r="B120" s="78" t="inlineStr">
+      <c r="B125" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C120" s="77" t="n">
+      <c r="C125" s="77" t="n">
         <v>46270</v>
       </c>
-      <c r="D120" s="79" t="n">
+      <c r="D125" s="79" t="n">
         <v>1086.4</v>
       </c>
-      <c r="E120" s="112" t="inlineStr">
+      <c r="E125" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F120" s="112">
-        <f>IF(OR($E120="Recebido",$C120=""),"",MAX(0,TODAY()-$C120))</f>
-        <v/>
-      </c>
-      <c r="G120" s="78" t="inlineStr">
+      <c r="F125" s="112">
+        <f>IF(OR($E125="Recebido",$C125=""),"",MAX(0,TODAY()-$C125))</f>
+        <v/>
+      </c>
+      <c r="G125" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.300 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="121" s="157">
-      <c r="A121" s="82" t="inlineStr">
+    <row r="126" s="157">
+      <c r="A126" s="82" t="inlineStr">
         <is>
           <t>Clínica Veterinária Paripiranga (Paripiranga/BA)</t>
         </is>
       </c>
-      <c r="B121" s="82" t="inlineStr">
+      <c r="B126" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C121" s="81" t="n">
+      <c r="C126" s="81" t="n">
         <v>46270</v>
       </c>
-      <c r="D121" s="83" t="n">
+      <c r="D126" s="83" t="n">
         <v>1265.85</v>
       </c>
-      <c r="E121" s="113" t="inlineStr">
+      <c r="E126" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F121" s="113">
-        <f>IF(OR($E121="Recebido",$C121=""),"",MAX(0,TODAY()-$C121))</f>
-        <v/>
-      </c>
-      <c r="G121" s="82" t="inlineStr">
+      <c r="F126" s="113">
+        <f>IF(OR($E126="Recebido",$C126=""),"",MAX(0,TODAY()-$C126))</f>
+        <v/>
+      </c>
+      <c r="G126" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.301 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="122" s="157">
-      <c r="A122" s="78" t="inlineStr">
+    <row r="127" s="157">
+      <c r="A127" s="78" t="inlineStr">
         <is>
           <t>UNP Mossoró (Mossoró/RN)</t>
         </is>
       </c>
-      <c r="B122" s="78" t="inlineStr">
+      <c r="B127" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C122" s="77" t="n">
+      <c r="C127" s="77" t="n">
         <v>46270</v>
       </c>
-      <c r="D122" s="79" t="n">
+      <c r="D127" s="79" t="n">
         <v>1867.25</v>
       </c>
-      <c r="E122" s="112" t="inlineStr">
+      <c r="E127" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F122" s="112">
-        <f>IF(OR($E122="Recebido",$C122=""),"",MAX(0,TODAY()-$C122))</f>
-        <v/>
-      </c>
-      <c r="G122" s="78" t="inlineStr">
+      <c r="F127" s="112">
+        <f>IF(OR($E127="Recebido",$C127=""),"",MAX(0,TODAY()-$C127))</f>
+        <v/>
+      </c>
+      <c r="G127" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.302 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="123" s="157">
-      <c r="A123" s="82" t="inlineStr">
+    <row r="128" s="157">
+      <c r="A128" s="82" t="inlineStr">
         <is>
           <t>CIS Jacobina (Jacobina/BA)</t>
         </is>
       </c>
-      <c r="B123" s="82" t="inlineStr">
+      <c r="B128" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C123" s="81" t="n">
+      <c r="C128" s="81" t="n">
         <v>46290</v>
       </c>
-      <c r="D123" s="83" t="n">
+      <c r="D128" s="83" t="n">
         <v>2095.2</v>
       </c>
-      <c r="E123" s="113" t="inlineStr">
+      <c r="E128" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F123" s="113">
-        <f>IF(OR($E123="Recebido",$C123=""),"",MAX(0,TODAY()-$C123))</f>
-        <v/>
-      </c>
-      <c r="G123" s="82" t="inlineStr">
+      <c r="F128" s="113">
+        <f>IF(OR($E128="Recebido",$C128=""),"",MAX(0,TODAY()-$C128))</f>
+        <v/>
+      </c>
+      <c r="G128" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.333 de 26/08/2026 · OC AEMPPO00004452 · 30 dias · recebido via Pix em 25/09/2026 (Nota Paga no portal V360).</t>
         </is>
       </c>
     </row>
-    <row r="124" s="157">
-      <c r="A124" s="78" t="inlineStr">
+    <row r="129" s="157">
+      <c r="A129" s="78" t="inlineStr">
         <is>
           <t>AGES Jacobina (Jacobina/BA)</t>
         </is>
       </c>
-      <c r="B124" s="78" t="inlineStr">
+      <c r="B129" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C124" s="77" t="n">
+      <c r="C129" s="77" t="n">
         <v>46305</v>
       </c>
-      <c r="D124" s="79" t="n">
+      <c r="D129" s="79" t="n">
         <v>1188.25</v>
       </c>
-      <c r="E124" s="112" t="inlineStr">
+      <c r="E129" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F124" s="112">
-        <f>IF(OR($E124="Recebido",$C124=""),"",MAX(0,TODAY()-$C124))</f>
-        <v/>
-      </c>
-      <c r="G124" s="78" t="inlineStr">
+      <c r="F129" s="112">
+        <f>IF(OR($E129="Recebido",$C129=""),"",MAX(0,TODAY()-$C129))</f>
+        <v/>
+      </c>
+      <c r="G129" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.332 de 26/08/2026 · OC AEMPPO00004453 · 45 dias · Recebido em 13/10/2026 no BNB (Nota Paga no portal V360).</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" s="157">
-      <c r="A125" s="82" t="inlineStr">
-        <is>
-          <t>Instituto Paulo Leão</t>
-        </is>
-      </c>
-      <c r="B125" s="82" t="inlineStr">
-        <is>
-          <t>Refil E3 + Pré Filtro</t>
-        </is>
-      </c>
-      <c r="C125" s="81" t="n">
-        <v>46265</v>
-      </c>
-      <c r="D125" s="83" t="n">
-        <v>160</v>
-      </c>
-      <c r="E125" s="113" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F125" s="113">
-        <f>IF(OR($E125="Recebido",$C125=""),"",MAX(0,TODAY()-$C125))</f>
-        <v/>
-      </c>
-      <c r="G125" s="82" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 08/09/2026 — lançado em "Set 2026".</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" s="157">
-      <c r="A126" s="78" t="inlineStr">
-        <is>
-          <t>Eletronic Segurança Eletronica</t>
-        </is>
-      </c>
-      <c r="B126" s="78" t="inlineStr">
-        <is>
-          <t>Pré Filtro</t>
-        </is>
-      </c>
-      <c r="C126" s="77" t="n">
-        <v>46265</v>
-      </c>
-      <c r="D126" s="79" t="n">
-        <v>60</v>
-      </c>
-      <c r="E126" s="112" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F126" s="112">
-        <f>IF(OR($E126="Recebido",$C126=""),"",MAX(0,TODAY()-$C126))</f>
-        <v/>
-      </c>
-      <c r="G126" s="78" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 03/09/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" s="157">
-      <c r="A127" s="82" t="inlineStr">
-        <is>
-          <t>Clube dos Mineiros</t>
-        </is>
-      </c>
-      <c r="B127" s="82" t="inlineStr">
-        <is>
-          <t>Refil Pro Life</t>
-        </is>
-      </c>
-      <c r="C127" s="81" t="n">
-        <v>46265</v>
-      </c>
-      <c r="D127" s="83" t="n">
-        <v>150</v>
-      </c>
-      <c r="E127" s="113" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F127" s="113">
-        <f>IF(OR($E127="Recebido",$C127=""),"",MAX(0,TODAY()-$C127))</f>
-        <v/>
-      </c>
-      <c r="G127" s="82" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 01/09/2026 (pagador: Sindicato dos Mineiros de Jacobina).</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" s="157">
-      <c r="A128" s="78" t="inlineStr">
-        <is>
-          <t>Armazem Cecilio Mota</t>
-        </is>
-      </c>
-      <c r="B128" s="78" t="inlineStr">
-        <is>
-          <t>Refil Everest + Refil Carbon 9"</t>
-        </is>
-      </c>
-      <c r="C128" s="77" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D128" s="79" t="n">
-        <v>225</v>
-      </c>
-      <c r="E128" s="112" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F128" s="112">
-        <f>IF(OR($E128="Recebido",$C128=""),"",MAX(0,TODAY()-$C128))</f>
-        <v/>
-      </c>
-      <c r="G128" s="78" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" s="157">
-      <c r="A129" s="82" t="inlineStr">
-        <is>
-          <t>Clebson Dantas Da Silva</t>
-        </is>
-      </c>
-      <c r="B129" s="82" t="inlineStr">
-        <is>
-          <t>Refil Everest</t>
-        </is>
-      </c>
-      <c r="C129" s="81" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D129" s="83" t="n">
-        <v>140</v>
-      </c>
-      <c r="E129" s="113" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F129" s="113">
-        <f>IF(OR($E129="Recebido",$C129=""),"",MAX(0,TODAY()-$C129))</f>
-        <v/>
-      </c>
-      <c r="G129" s="82" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 02/09/2026</t>
         </is>
       </c>
     </row>
     <row r="130" s="157">
       <c r="A130" s="82" t="inlineStr">
         <is>
-          <t>Tesla Imagem Medicina Diagnostica Ltda</t>
+          <t>Instituto Paulo Leão</t>
         </is>
       </c>
       <c r="B130" s="82" t="inlineStr">
         <is>
-          <t>3x Refil Everest + 2x Pré Filtro</t>
+          <t>Refil E3 + Pré Filtro</t>
         </is>
       </c>
       <c r="C130" s="81" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="D130" s="83" t="n">
-        <v>540</v>
+        <v>160</v>
       </c>
       <c r="E130" s="113" t="inlineStr">
         <is>
@@ -71178,26 +71178,26 @@
       </c>
       <c r="G130" s="82" t="inlineStr">
         <is>
-          <t>Troca do dia 02/09/2026 — 1º Andar, Térreo e Copa. Recebido via Pix em 08/09/2026 — lançado em "Set 2026".</t>
+          <t>Recebido via Pix em 08/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="131" s="157">
       <c r="A131" s="78" t="inlineStr">
         <is>
-          <t>Cecilio Mota Junior</t>
+          <t>Eletronic Segurança Eletronica</t>
         </is>
       </c>
       <c r="B131" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Pré Filtro</t>
         </is>
       </c>
       <c r="C131" s="77" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="D131" s="79" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="E131" s="112" t="inlineStr">
         <is>
@@ -71210,58 +71210,58 @@
       </c>
       <c r="G131" s="78" t="inlineStr">
         <is>
-          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
+          <t>Recebido via Pix em 03/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="132" s="157">
-      <c r="A132" s="78" t="inlineStr">
-        <is>
-          <t>Tereza Cristina Aquino Martins - Luiz Augusto</t>
-        </is>
-      </c>
-      <c r="B132" s="78" t="inlineStr">
-        <is>
-          <t>Refil Everest + Pré Filtro</t>
-        </is>
-      </c>
-      <c r="C132" s="77" t="n">
-        <v>46268</v>
-      </c>
-      <c r="D132" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="E132" s="112" t="inlineStr">
+      <c r="A132" s="82" t="inlineStr">
+        <is>
+          <t>Clube dos Mineiros</t>
+        </is>
+      </c>
+      <c r="B132" s="82" t="inlineStr">
+        <is>
+          <t>Refil Pro Life</t>
+        </is>
+      </c>
+      <c r="C132" s="81" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D132" s="83" t="n">
+        <v>150</v>
+      </c>
+      <c r="E132" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F132" s="112">
+      <c r="F132" s="113">
         <f>IF(OR($E132="Recebido",$C132=""),"",MAX(0,TODAY()-$C132))</f>
         <v/>
       </c>
-      <c r="G132" s="78" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 04/09/2026.</t>
+      <c r="G132" s="82" t="inlineStr">
+        <is>
+          <t>Recebido via Pix em 01/09/2026 (pagador: Sindicato dos Mineiros de Jacobina).</t>
         </is>
       </c>
     </row>
     <row r="133" s="157">
       <c r="A133" s="78" t="inlineStr">
         <is>
-          <t>Samille Fiscina Lima Lordello - Tiago (Cartório)</t>
+          <t>Armazem Cecilio Mota</t>
         </is>
       </c>
       <c r="B133" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life</t>
+          <t>Refil Everest + Refil Carbon 9"</t>
         </is>
       </c>
       <c r="C133" s="77" t="n">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="D133" s="79" t="n">
-        <v>140</v>
+        <v>225</v>
       </c>
       <c r="E133" s="112" t="inlineStr">
         <is>
@@ -71279,85 +71279,85 @@
       </c>
     </row>
     <row r="134" s="157">
-      <c r="A134" s="78" t="inlineStr">
-        <is>
-          <t>Bomboniere Doce Mania - Veronildo Basilio</t>
-        </is>
-      </c>
-      <c r="B134" s="78" t="inlineStr">
-        <is>
-          <t>Refil Plissado + Refil BAG</t>
-        </is>
-      </c>
-      <c r="C134" s="77" t="n">
-        <v>46274</v>
-      </c>
-      <c r="D134" s="79" t="n">
-        <v>150</v>
-      </c>
-      <c r="E134" s="112" t="inlineStr">
+      <c r="A134" s="82" t="inlineStr">
+        <is>
+          <t>Clebson Dantas Da Silva</t>
+        </is>
+      </c>
+      <c r="B134" s="82" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="C134" s="81" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D134" s="83" t="n">
+        <v>140</v>
+      </c>
+      <c r="E134" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F134" s="112">
+      <c r="F134" s="113">
         <f>IF(OR($E134="Recebido",$C134=""),"",MAX(0,TODAY()-$C134))</f>
         <v/>
       </c>
-      <c r="G134" s="78" t="inlineStr">
-        <is>
-          <t>Recebido em dinheiro em 16/09/2026 — lançado em "Set 2026".</t>
+      <c r="G134" s="82" t="inlineStr">
+        <is>
+          <t>Recebido via Pix em 02/09/2026</t>
         </is>
       </c>
     </row>
     <row r="135" s="157">
-      <c r="A135" s="78" t="inlineStr">
-        <is>
-          <t>Adriadne (Hotel Jovem Jota)</t>
-        </is>
-      </c>
-      <c r="B135" s="78" t="inlineStr">
-        <is>
-          <t>Refil Everest</t>
-        </is>
-      </c>
-      <c r="C135" s="77" t="n">
-        <v>46275</v>
-      </c>
-      <c r="D135" s="79" t="n">
-        <v>140</v>
-      </c>
-      <c r="E135" s="112" t="inlineStr">
+      <c r="A135" s="82" t="inlineStr">
+        <is>
+          <t>Tesla Imagem Medicina Diagnostica Ltda</t>
+        </is>
+      </c>
+      <c r="B135" s="82" t="inlineStr">
+        <is>
+          <t>3x Refil Everest + 2x Pré Filtro</t>
+        </is>
+      </c>
+      <c r="C135" s="81" t="n">
+        <v>46267</v>
+      </c>
+      <c r="D135" s="83" t="n">
+        <v>540</v>
+      </c>
+      <c r="E135" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F135" s="112">
+      <c r="F135" s="113">
         <f>IF(OR($E135="Recebido",$C135=""),"",MAX(0,TODAY()-$C135))</f>
         <v/>
       </c>
-      <c r="G135" s="78" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 11/09/2026 — lançado em "Set 2026".</t>
+      <c r="G135" s="82" t="inlineStr">
+        <is>
+          <t>Troca do dia 02/09/2026 — 1º Andar, Térreo e Copa. Recebido via Pix em 08/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="136" s="157">
       <c r="A136" s="78" t="inlineStr">
         <is>
-          <t>Pousada Triunfo Ltda (Hotel Triunfo)</t>
+          <t>Cecilio Mota Junior</t>
         </is>
       </c>
       <c r="B136" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Pré Filtro</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C136" s="77" t="n">
-        <v>46275</v>
+        <v>46267</v>
       </c>
       <c r="D136" s="79" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="E136" s="112" t="inlineStr">
         <is>
@@ -71370,26 +71370,26 @@
       </c>
       <c r="G136" s="78" t="inlineStr">
         <is>
-          <t>Recebido via Pix em 11/09/2026 — lançado em "Set 2026".</t>
+          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="137" s="157">
       <c r="A137" s="78" t="inlineStr">
         <is>
-          <t>Topvel Tropical Veiculos e Pecas</t>
+          <t>Tereza Cristina Aquino Martins - Luiz Augusto</t>
         </is>
       </c>
       <c r="B137" s="78" t="inlineStr">
         <is>
-          <t>2x Refil Everest + 2x Pré Filtro</t>
+          <t>Refil Everest + Pré Filtro</t>
         </is>
       </c>
       <c r="C137" s="77" t="n">
-        <v>46276</v>
+        <v>46268</v>
       </c>
       <c r="D137" s="79" t="n">
-        <v>370</v>
+        <v>200</v>
       </c>
       <c r="E137" s="112" t="inlineStr">
         <is>
@@ -71402,23 +71402,23 @@
       </c>
       <c r="G137" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 11/09/2026 — dois purificadores. Recebido via TED no BNB em 05/10/2026 — lançado em "Out 2026".</t>
+          <t>Recebido via Pix em 04/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="138" s="157">
       <c r="A138" s="78" t="inlineStr">
         <is>
-          <t>J Diesel Motores e Reparos - Gilmara</t>
+          <t>Samille Fiscina Lima Lordello - Tiago (Cartório)</t>
         </is>
       </c>
       <c r="B138" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Refil Pro Life</t>
         </is>
       </c>
       <c r="C138" s="77" t="n">
-        <v>46276</v>
+        <v>46269</v>
       </c>
       <c r="D138" s="79" t="n">
         <v>140</v>
@@ -71434,26 +71434,26 @@
       </c>
       <c r="G138" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 11/09/2026.</t>
+          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="139" s="157">
       <c r="A139" s="78" t="inlineStr">
         <is>
-          <t>IOB</t>
+          <t>Bomboniere Doce Mania - Veronildo Basilio</t>
         </is>
       </c>
       <c r="B139" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Pré Filtro</t>
+          <t>Refil Plissado + Refil BAG</t>
         </is>
       </c>
       <c r="C139" s="77" t="n">
-        <v>46279</v>
+        <v>46274</v>
       </c>
       <c r="D139" s="79" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="E139" s="112" t="inlineStr">
         <is>
@@ -71466,26 +71466,26 @@
       </c>
       <c r="G139" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 14/09/2026.</t>
+          <t>Recebido em dinheiro em 16/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="140" s="157">
       <c r="A140" s="78" t="inlineStr">
         <is>
-          <t>Clínica Santa Cecília</t>
+          <t>Adriadne (Hotel Jovem Jota)</t>
         </is>
       </c>
       <c r="B140" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Termostato</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C140" s="77" t="n">
-        <v>46281</v>
+        <v>46275</v>
       </c>
       <c r="D140" s="79" t="n">
-        <v>310</v>
+        <v>140</v>
       </c>
       <c r="E140" s="112" t="inlineStr">
         <is>
@@ -71498,14 +71498,14 @@
       </c>
       <c r="G140" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 16/09/2026 — refil + troca de termostato. Recebido via Pix em 29/09/2026.</t>
+          <t>Recebido via Pix em 11/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="141" s="157">
       <c r="A141" s="78" t="inlineStr">
         <is>
-          <t>Marilda Macedo / José Luciano Costa</t>
+          <t>Pousada Triunfo Ltda (Hotel Triunfo)</t>
         </is>
       </c>
       <c r="B141" s="78" t="inlineStr">
@@ -71514,7 +71514,7 @@
         </is>
       </c>
       <c r="C141" s="77" t="n">
-        <v>46283</v>
+        <v>46275</v>
       </c>
       <c r="D141" s="79" t="n">
         <v>200</v>
@@ -71530,26 +71530,26 @@
       </c>
       <c r="G141" s="78" t="inlineStr">
         <is>
-          <t>Recebido via Pix em 19/09/2026 — lançado em "Set 2026".</t>
+          <t>Recebido via Pix em 11/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="142" s="157">
       <c r="A142" s="78" t="inlineStr">
         <is>
-          <t>Tatiana Rocha</t>
+          <t>Topvel Tropical Veiculos e Pecas</t>
         </is>
       </c>
       <c r="B142" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>2x Refil Everest + 2x Pré Filtro</t>
         </is>
       </c>
       <c r="C142" s="77" t="n">
-        <v>46286</v>
+        <v>46276</v>
       </c>
       <c r="D142" s="79" t="n">
-        <v>140</v>
+        <v>370</v>
       </c>
       <c r="E142" s="112" t="inlineStr">
         <is>
@@ -71562,14 +71562,14 @@
       </c>
       <c r="G142" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 21/09/2026. Recebido via Pix em 22/09/2026 — lançado em "Set 2026".</t>
+          <t>Troca do dia 11/09/2026 — dois purificadores. Recebido via TED no BNB em 05/10/2026 — lançado em "Out 2026".</t>
         </is>
       </c>
     </row>
     <row r="143" s="157">
       <c r="A143" s="78" t="inlineStr">
         <is>
-          <t>Cleone Gomes de Andrade</t>
+          <t>J Diesel Motores e Reparos - Gilmara</t>
         </is>
       </c>
       <c r="B143" s="78" t="inlineStr">
@@ -71578,7 +71578,7 @@
         </is>
       </c>
       <c r="C143" s="77" t="n">
-        <v>46286</v>
+        <v>46276</v>
       </c>
       <c r="D143" s="79" t="n">
         <v>140</v>
@@ -71594,30 +71594,30 @@
       </c>
       <c r="G143" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 21/09/2026. Recebido via Pix em 21/09/2026.</t>
+          <t>Troca do dia 11/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="144" s="157">
       <c r="A144" s="78" t="inlineStr">
         <is>
-          <t>Centro de Especialidades Odontomédicas</t>
+          <t>IOB</t>
         </is>
       </c>
       <c r="B144" s="78" t="inlineStr">
         <is>
-          <t>2x Refil Everest</t>
+          <t>Refil Everest + Pré Filtro</t>
         </is>
       </c>
       <c r="C144" s="77" t="n">
-        <v>46044</v>
+        <v>46279</v>
       </c>
       <c r="D144" s="79" t="n">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="E144" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F144" s="112">
@@ -71626,30 +71626,30 @@
       </c>
       <c r="G144" s="78" t="inlineStr">
         <is>
-          <t>NF-e 4039 de 22/01/2026 (CNPJ 54.747.945/0001-09). Venda anterior ao controle manual (aba Jan 2026 vem do Livro Caixa). Conferido no DigiSat em 28/09/2026: não recebido. Mesmo cliente tem outra pendência de 05/08/2026 (R$ 140,00).</t>
+          <t>Troca do dia 14/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="145" s="157">
       <c r="A145" s="78" t="inlineStr">
         <is>
-          <t>Igreja Messiânica Mundial do Brasil</t>
+          <t>Clínica Santa Cecília</t>
         </is>
       </c>
       <c r="B145" s="78" t="inlineStr">
         <is>
-          <t>Mangueira</t>
+          <t>Refil Everest + Termostato</t>
         </is>
       </c>
       <c r="C145" s="77" t="n">
-        <v>46073</v>
+        <v>46281</v>
       </c>
       <c r="D145" s="79" t="n">
-        <v>30</v>
+        <v>310</v>
       </c>
       <c r="E145" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F145" s="112">
@@ -71658,30 +71658,30 @@
       </c>
       <c r="G145" s="78" t="inlineStr">
         <is>
-          <t>NF-e 4075 de 20/02/2026 (CNPJ 62.647.383/0063-44). Conferido no DigiSat em 28/09/2026: não recebido.</t>
+          <t>Troca do dia 16/09/2026 — refil + troca de termostato. Recebido via Pix em 29/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="146" s="157">
       <c r="A146" s="78" t="inlineStr">
         <is>
-          <t>Centro Médico de Jacobina</t>
+          <t>Marilda Macedo / José Luciano Costa</t>
         </is>
       </c>
       <c r="B146" s="78" t="inlineStr">
         <is>
-          <t>2x Botão Completo</t>
+          <t>Refil Everest + Pré Filtro</t>
         </is>
       </c>
       <c r="C146" s="77" t="n">
-        <v>46203</v>
+        <v>46283</v>
       </c>
       <c r="D146" s="79" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="E146" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F146" s="112">
@@ -71690,14 +71690,14 @@
       </c>
       <c r="G146" s="78" t="inlineStr">
         <is>
-          <t>NF-e 4242 de 30/06/2026 (CNPJ 13.228.432/0001-04). Conferido no DigiSat em 28/09/2026: não recebido.</t>
+          <t>Recebido via Pix em 19/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="147" s="157">
       <c r="A147" s="78" t="inlineStr">
         <is>
-          <t>Vivencie Turismo Agencia de Viagens - Aneildes Rios</t>
+          <t>Tatiana Rocha</t>
         </is>
       </c>
       <c r="B147" s="78" t="inlineStr">
@@ -71706,7 +71706,7 @@
         </is>
       </c>
       <c r="C147" s="77" t="n">
-        <v>46294</v>
+        <v>46286</v>
       </c>
       <c r="D147" s="79" t="n">
         <v>140</v>
@@ -71722,26 +71722,26 @@
       </c>
       <c r="G147" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 29/09/2026. Recebido via Pix em 05/10/2026 — R$ 135,00 (Pix único de R$ 270,00 com as duas trocas; R$ 10,00 de desconto dividido).</t>
+          <t>Troca do dia 21/09/2026. Recebido via Pix em 22/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="148" s="157">
       <c r="A148" s="78" t="inlineStr">
         <is>
-          <t>Lapec</t>
+          <t>Cleone Gomes de Andrade</t>
         </is>
       </c>
       <c r="B148" s="78" t="inlineStr">
         <is>
-          <t>Refil C+3</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C148" s="77" t="n">
-        <v>46294</v>
+        <v>46286</v>
       </c>
       <c r="D148" s="79" t="n">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="E148" s="112" t="inlineStr">
         <is>
@@ -71754,30 +71754,30 @@
       </c>
       <c r="G148" s="78" t="inlineStr">
         <is>
-          <t>Pagamento previsto para 30/09/2026. Recebido em dinheiro em 14/10/2026 — lançado em "Set 2026".</t>
+          <t>Troca do dia 21/09/2026. Recebido via Pix em 21/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="149" s="157">
       <c r="A149" s="78" t="inlineStr">
         <is>
-          <t>PC Jacobina Administradora de Cartões LTDA - Cartão de Todos</t>
+          <t>Centro de Especialidades Odontomédicas</t>
         </is>
       </c>
       <c r="B149" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>2x Refil Everest</t>
         </is>
       </c>
       <c r="C149" s="77" t="n">
-        <v>46295</v>
+        <v>46044</v>
       </c>
       <c r="D149" s="79" t="n">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="E149" s="112" t="inlineStr">
         <is>
-          <t>Recebido</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="F149" s="112">
@@ -71786,30 +71786,30 @@
       </c>
       <c r="G149" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 30/09/2026. Recebido via Pix em 01/10/2026 (comprovante enviado em 06/10/2026) — lançado em "Out 2026".</t>
+          <t>NF-e 4039 de 22/01/2026 (CNPJ 54.747.945/0001-09). Venda anterior ao controle manual (aba Jan 2026 vem do Livro Caixa). Conferido no DigiSat em 28/09/2026: não recebido. Mesmo cliente tem outra pendência de 05/08/2026 (R$ 140,00).</t>
         </is>
       </c>
     </row>
     <row r="150" s="157">
       <c r="A150" s="78" t="inlineStr">
         <is>
-          <t>Aneilde Rios de Oliveira</t>
+          <t>Igreja Messiânica Mundial do Brasil</t>
         </is>
       </c>
       <c r="B150" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Mangueira</t>
         </is>
       </c>
       <c r="C150" s="77" t="n">
-        <v>46296</v>
+        <v>46073</v>
       </c>
       <c r="D150" s="79" t="n">
-        <v>140</v>
+        <v>30</v>
       </c>
       <c r="E150" s="112" t="inlineStr">
         <is>
-          <t>Recebido</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="F150" s="112">
@@ -71818,30 +71818,30 @@
       </c>
       <c r="G150" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 01/10/2026 (casa, Caeira). Recebido via Pix em 05/10/2026 — R$ 135,00 (Pix único de R$ 270,00 com as duas trocas; R$ 10,00 de desconto dividido).</t>
+          <t>NF-e 4075 de 20/02/2026 (CNPJ 62.647.383/0063-44). Conferido no DigiSat em 28/09/2026: não recebido.</t>
         </is>
       </c>
     </row>
     <row r="151" s="157">
       <c r="A151" s="78" t="inlineStr">
         <is>
-          <t>Centro Medico da Chapada Diamantina LTDA</t>
+          <t>Centro Médico de Jacobina</t>
         </is>
       </c>
       <c r="B151" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life + 2x Botão Completo</t>
+          <t>2x Botão Completo</t>
         </is>
       </c>
       <c r="C151" s="77" t="n">
-        <v>46296</v>
+        <v>46203</v>
       </c>
       <c r="D151" s="79" t="n">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="E151" s="112" t="inlineStr">
         <is>
-          <t>Recebido</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="F151" s="112">
@@ -71850,26 +71850,26 @@
       </c>
       <c r="G151" s="78" t="inlineStr">
         <is>
-          <t>Subsolo — troca do dia 01/10/2026 (refil + 2 botões). Recebido em 05/10/2026 no crédito em 3x (pagamento único de R$ 400,00 pelas duas trocas).</t>
+          <t>NF-e 4242 de 30/06/2026 (CNPJ 13.228.432/0001-04). Conferido no DigiSat em 28/09/2026: não recebido.</t>
         </is>
       </c>
     </row>
     <row r="152" s="157">
       <c r="A152" s="78" t="inlineStr">
         <is>
-          <t>Centro Medico da Chapada Diamantina LTDA</t>
+          <t>Vivencie Turismo Agencia de Viagens - Aneildes Rios</t>
         </is>
       </c>
       <c r="B152" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life + 2x Botão Completo</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C152" s="77" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="D152" s="79" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="E152" s="112" t="inlineStr">
         <is>
@@ -71882,30 +71882,30 @@
       </c>
       <c r="G152" s="78" t="inlineStr">
         <is>
-          <t>1º Andar — troca do dia 02/10/2026 (refil + 2 botões). Recebido em 05/10/2026 no crédito em 3x (pagamento único de R$ 400,00 pelas duas trocas).</t>
+          <t>Troca do dia 29/09/2026. Recebido via Pix em 05/10/2026 — R$ 135,00 (Pix único de R$ 270,00 com as duas trocas; R$ 10,00 de desconto dividido).</t>
         </is>
       </c>
     </row>
     <row r="153" s="157">
       <c r="A153" s="78" t="inlineStr">
         <is>
-          <t>Igreja Messiânica Mundial do Brasil</t>
+          <t>Lapec</t>
         </is>
       </c>
       <c r="B153" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Refil C+3</t>
         </is>
       </c>
       <c r="C153" s="77" t="n">
-        <v>46300</v>
+        <v>46294</v>
       </c>
       <c r="D153" s="79" t="n">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="E153" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F153" s="112">
@@ -71914,14 +71914,14 @@
       </c>
       <c r="G153" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 05/10/2026. Mesmo cliente tem pendência de 20/02/2026 (Mangueira, R$ 30,00).</t>
+          <t>Pagamento previsto para 30/09/2026. Recebido em dinheiro em 14/10/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="154" s="157">
       <c r="A154" s="78" t="inlineStr">
         <is>
-          <t>Rafael Landin Ribeiro</t>
+          <t>PC Jacobina Administradora de Cartões LTDA - Cartão de Todos</t>
         </is>
       </c>
       <c r="B154" s="78" t="inlineStr">
@@ -71930,7 +71930,7 @@
         </is>
       </c>
       <c r="C154" s="77" t="n">
-        <v>46304</v>
+        <v>46295</v>
       </c>
       <c r="D154" s="79" t="n">
         <v>140</v>
@@ -71946,30 +71946,30 @@
       </c>
       <c r="G154" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 09/10/2026. Recebido via Pix em 09/10/2026.</t>
+          <t>Troca do dia 30/09/2026. Recebido via Pix em 01/10/2026 (comprovante enviado em 06/10/2026) — lançado em "Out 2026".</t>
         </is>
       </c>
     </row>
     <row r="155" s="157">
       <c r="A155" s="78" t="inlineStr">
         <is>
-          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
+          <t>Aneilde Rios de Oliveira</t>
         </is>
       </c>
       <c r="B155" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life + Refil Universal (restante)</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C155" s="77" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="D155" s="79" t="n">
-        <v>85</v>
+        <v>140</v>
       </c>
       <c r="E155" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F155" s="112">
@@ -71978,30 +71978,30 @@
       </c>
       <c r="G155" s="78" t="inlineStr">
         <is>
-          <t>Venda de R$ 170,00 — R$ 85,00 pagos no débito em 09/10/2026; restante via Pix previsto para 16/10/2026.</t>
+          <t>Troca do dia 01/10/2026 (casa, Caeira). Recebido via Pix em 05/10/2026 — R$ 135,00 (Pix único de R$ 270,00 com as duas trocas; R$ 10,00 de desconto dividido).</t>
         </is>
       </c>
     </row>
     <row r="156" s="157">
       <c r="A156" s="78" t="inlineStr">
         <is>
-          <t>Tropical Motos LTDA</t>
+          <t>Centro Medico da Chapada Diamantina LTDA</t>
         </is>
       </c>
       <c r="B156" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life</t>
+          <t>Refil Pro Life + 2x Botão Completo</t>
         </is>
       </c>
       <c r="C156" s="77" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="D156" s="79" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="E156" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F156" s="112">
@@ -72010,30 +72010,30 @@
       </c>
       <c r="G156" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 09/10/2026 — purificador do andar de cima.</t>
+          <t>Subsolo — troca do dia 01/10/2026 (refil + 2 botões). Recebido em 05/10/2026 no crédito em 3x (pagamento único de R$ 400,00 pelas duas trocas).</t>
         </is>
       </c>
     </row>
     <row r="157" s="157">
       <c r="A157" s="78" t="inlineStr">
         <is>
-          <t>Casa do Construtor</t>
+          <t>Centro Medico da Chapada Diamantina LTDA</t>
         </is>
       </c>
       <c r="B157" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Refil Pro Life + 2x Botão Completo</t>
         </is>
       </c>
       <c r="C157" s="77" t="n">
-        <v>46310</v>
+        <v>46297</v>
       </c>
       <c r="D157" s="79" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="E157" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F157" s="112">
@@ -72042,26 +72042,26 @@
       </c>
       <c r="G157" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 15/10/2026.</t>
+          <t>1º Andar — troca do dia 02/10/2026 (refil + 2 botões). Recebido em 05/10/2026 no crédito em 3x (pagamento único de R$ 400,00 pelas duas trocas).</t>
         </is>
       </c>
     </row>
     <row r="158" s="157">
       <c r="A158" s="78" t="inlineStr">
         <is>
-          <t>Lapec</t>
+          <t>Igreja Messiânica Mundial do Brasil</t>
         </is>
       </c>
       <c r="B158" s="78" t="inlineStr">
         <is>
-          <t>Refil E3 + Refil Everest</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C158" s="77" t="n">
-        <v>46310</v>
+        <v>46300</v>
       </c>
       <c r="D158" s="79" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="E158" s="112" t="inlineStr">
         <is>
@@ -72074,14 +72074,14 @@
       </c>
       <c r="G158" s="78" t="inlineStr">
         <is>
-          <t>Compra do dia 15/10/2026 — Refil E3 R$ 80,00 + Refil Everest R$ 120,00.</t>
+          <t>Troca do dia 05/10/2026. Mesmo cliente tem pendência de 20/02/2026 (Mangueira, R$ 30,00).</t>
         </is>
       </c>
     </row>
     <row r="159" s="157">
       <c r="A159" s="78" t="inlineStr">
         <is>
-          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
+          <t>Rafael Landin Ribeiro</t>
         </is>
       </c>
       <c r="B159" s="78" t="inlineStr">
@@ -72090,7 +72090,7 @@
         </is>
       </c>
       <c r="C159" s="77" t="n">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="D159" s="79" t="n">
         <v>140</v>
@@ -72106,26 +72106,26 @@
       </c>
       <c r="G159" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 15/10/2026. Recebido via Pix em 16/10/2026 — lançado em "Out 2026".</t>
+          <t>Troca do dia 09/10/2026. Recebido via Pix em 09/10/2026.</t>
         </is>
       </c>
     </row>
     <row r="160" s="157">
       <c r="A160" s="78" t="inlineStr">
         <is>
-          <t>Colegio Oasis de Jacobina - Unopar</t>
+          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
         </is>
       </c>
       <c r="B160" s="78" t="inlineStr">
         <is>
-          <t>2x Refil Plissado + 2x Carcaça 9"</t>
+          <t>Refil Pro Life + Refil Universal (restante)</t>
         </is>
       </c>
       <c r="C160" s="77" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="D160" s="79" t="n">
-        <v>400</v>
+        <v>85</v>
       </c>
       <c r="E160" s="112" t="inlineStr">
         <is>
@@ -72138,26 +72138,26 @@
       </c>
       <c r="G160" s="78" t="inlineStr">
         <is>
-          <t>2x Refil Plissado R$ 80,00 cada + 2x Carcaça 9" R$ 120,00 cada. Cláudio assinou para pagar depois. Falta enviar a NF.</t>
+          <t>Venda de R$ 170,00 — R$ 85,00 pagos no débito em 09/10/2026; restante via Pix previsto para 16/10/2026.</t>
         </is>
       </c>
     </row>
     <row r="161" s="157">
       <c r="A161" s="78" t="inlineStr">
         <is>
-          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+          <t>Tropical Motos LTDA</t>
         </is>
       </c>
       <c r="B161" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Pré Filtro (restante)</t>
+          <t>Refil Pro Life</t>
         </is>
       </c>
       <c r="C161" s="77" t="n">
-        <v>46311</v>
+        <v>46304</v>
       </c>
       <c r="D161" s="79" t="n">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="E161" s="112" t="inlineStr">
         <is>
@@ -72170,26 +72170,26 @@
       </c>
       <c r="G161" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 16/10/2026 — bebedouro da recepção. Venda de R$ 200,00: R$ 140,00 pagos em dinheiro em 16/10/2026; falta R$ 60,00.</t>
+          <t>Troca do dia 09/10/2026 — purificador do andar de cima.</t>
         </is>
       </c>
     </row>
     <row r="162" s="157">
       <c r="A162" s="78" t="inlineStr">
         <is>
-          <t>Contabilidade Abreu</t>
+          <t>Casa do Construtor</t>
         </is>
       </c>
       <c r="B162" s="78" t="inlineStr">
         <is>
-          <t>Termostato</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C162" s="77" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="D162" s="79" t="n">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="E162" s="112" t="inlineStr">
         <is>
@@ -72202,52 +72202,207 @@
       </c>
       <c r="G162" s="78" t="inlineStr">
         <is>
+          <t>Troca do dia 15/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" s="157">
+      <c r="A163" s="78" t="inlineStr">
+        <is>
+          <t>Lapec</t>
+        </is>
+      </c>
+      <c r="B163" s="78" t="inlineStr">
+        <is>
+          <t>Refil E3 + Refil Everest</t>
+        </is>
+      </c>
+      <c r="C163" s="77" t="n">
+        <v>46310</v>
+      </c>
+      <c r="D163" s="79" t="n">
+        <v>200</v>
+      </c>
+      <c r="E163" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F163" s="112">
+        <f>IF(OR($E163="Recebido",$C163=""),"",MAX(0,TODAY()-$C163))</f>
+        <v/>
+      </c>
+      <c r="G163" s="78" t="inlineStr">
+        <is>
+          <t>Compra do dia 15/10/2026 — Refil E3 R$ 80,00 + Refil Everest R$ 120,00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" s="157">
+      <c r="A164" s="78" t="inlineStr">
+        <is>
+          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
+        </is>
+      </c>
+      <c r="B164" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="C164" s="77" t="n">
+        <v>46310</v>
+      </c>
+      <c r="D164" s="79" t="n">
+        <v>140</v>
+      </c>
+      <c r="E164" s="112" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
+      <c r="F164" s="112">
+        <f>IF(OR($E164="Recebido",$C164=""),"",MAX(0,TODAY()-$C164))</f>
+        <v/>
+      </c>
+      <c r="G164" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 15/10/2026. Recebido via Pix em 16/10/2026 — lançado em "Out 2026".</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" s="157">
+      <c r="A165" s="78" t="inlineStr">
+        <is>
+          <t>Colegio Oasis de Jacobina - Unopar</t>
+        </is>
+      </c>
+      <c r="B165" s="78" t="inlineStr">
+        <is>
+          <t>2x Refil Plissado + 2x Carcaça 9"</t>
+        </is>
+      </c>
+      <c r="C165" s="77" t="n">
+        <v>46305</v>
+      </c>
+      <c r="D165" s="79" t="n">
+        <v>400</v>
+      </c>
+      <c r="E165" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F165" s="112">
+        <f>IF(OR($E165="Recebido",$C165=""),"",MAX(0,TODAY()-$C165))</f>
+        <v/>
+      </c>
+      <c r="G165" s="78" t="inlineStr">
+        <is>
+          <t>2x Refil Plissado R$ 80,00 cada + 2x Carcaça 9" R$ 120,00 cada. Cláudio assinou para pagar depois. Falta enviar a NF.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" s="157">
+      <c r="A166" s="78" t="inlineStr">
+        <is>
+          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+        </is>
+      </c>
+      <c r="B166" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro (restante)</t>
+        </is>
+      </c>
+      <c r="C166" s="77" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D166" s="79" t="n">
+        <v>60</v>
+      </c>
+      <c r="E166" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F166" s="112">
+        <f>IF(OR($E166="Recebido",$C166=""),"",MAX(0,TODAY()-$C166))</f>
+        <v/>
+      </c>
+      <c r="G166" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 16/10/2026 — bebedouro da recepção. Venda de R$ 200,00: R$ 140,00 pagos em dinheiro em 16/10/2026; falta R$ 60,00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" s="157">
+      <c r="A167" s="78" t="inlineStr">
+        <is>
+          <t>Contabilidade Abreu</t>
+        </is>
+      </c>
+      <c r="B167" s="78" t="inlineStr">
+        <is>
+          <t>Termostato</t>
+        </is>
+      </c>
+      <c r="C167" s="77" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D167" s="79" t="n">
+        <v>170</v>
+      </c>
+      <c r="E167" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F167" s="112">
+        <f>IF(OR($E167="Recebido",$C167=""),"",MAX(0,TODAY()-$C167))</f>
+        <v/>
+      </c>
+      <c r="G167" s="78" t="inlineStr">
+        <is>
           <t>Troca de termostato do dia 16/10/2026.</t>
         </is>
       </c>
     </row>
-    <row r="163" s="157">
-      <c r="A163" s="86" t="inlineStr">
+    <row r="168" s="157">
+      <c r="A168" s="86" t="inlineStr">
         <is>
           <t>TOTAL EM ABERTO A RECEBER (detalhe)</t>
         </is>
       </c>
-      <c r="D163" s="115">
-        <f>SUMIF(E102:E162,"Pendente",D102:D162)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="164" s="157">
-      <c r="A164" s="202" t="inlineStr">
+      <c r="D168" s="115">
+        <f>SUMIF(E107:E167,"Pendente",D107:D167)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="169" s="157">
+      <c r="A169" s="202" t="inlineStr">
         <is>
           <t>CONFERÊNCIA COM AS ABAS DOS MESES</t>
         </is>
       </c>
-      <c r="B164" s="159" t="n"/>
-      <c r="C164" s="159" t="n"/>
-      <c r="D164" s="159" t="n"/>
-      <c r="E164" s="159" t="n"/>
-      <c r="F164" s="159" t="n"/>
-      <c r="G164" s="160" t="n"/>
-    </row>
-    <row r="165" s="157">
-      <c r="A165" s="203">
-        <f>IF(ROUND(D163-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D163-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="166" s="157">
-      <c r="A166" s="203" t="inlineStr">
+      <c r="B169" s="159" t="n"/>
+      <c r="C169" s="159" t="n"/>
+      <c r="D169" s="159" t="n"/>
+      <c r="E169" s="159" t="n"/>
+      <c r="F169" s="159" t="n"/>
+      <c r="G169" s="160" t="n"/>
+    </row>
+    <row r="170" s="157">
+      <c r="A170" s="203">
+        <f>IF(ROUND(D168-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D168-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="171" s="157">
+      <c r="A171" s="203" t="inlineStr">
         <is>
           <t>As contas a pagar do DigiSat (pendentes até 27/07/2026) foram todas quitadas — confirmado em 19/08/2026. A única dívida em aberto hoje é o Capital de Giro do Banco do Brasil. Lance aqui novos compromissos conforme surgirem.</t>
         </is>
       </c>
     </row>
-    <row r="167" s="157"/>
-    <row r="168" s="157"/>
-    <row r="169" s="157"/>
-    <row r="170" s="157"/>
-    <row r="171" s="157"/>
     <row r="172" s="157"/>
     <row r="173" s="157"/>
     <row r="174" s="157"/>
@@ -72281,27 +72436,32 @@
     <row r="202" s="157"/>
     <row r="203" s="157"/>
     <row r="204" s="157"/>
+    <row r="205" s="157"/>
+    <row r="206" s="157"/>
+    <row r="207" s="157"/>
+    <row r="208" s="157"/>
+    <row r="209" s="157"/>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A169:G169"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A100:G100"/>
+    <mergeCell ref="A105:G105"/>
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="A5:B6"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E5:F6"/>
-    <mergeCell ref="A165:G165"/>
-    <mergeCell ref="A99:G99"/>
-    <mergeCell ref="A164:G164"/>
+    <mergeCell ref="A104:G104"/>
+    <mergeCell ref="A170:G170"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E11:E94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E11:E99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Pago,Previsto"</formula1>
     </dataValidation>
-    <dataValidation sqref="E102:E162" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E107:E167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Recebido"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Atualizacao do painel - 21/10/2026 12:07
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -57662,38 +57662,99 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="17" t="n"/>
-      <c r="B149" s="18" t="n"/>
-      <c r="C149" s="18" t="n"/>
-      <c r="D149" s="27" t="n"/>
-      <c r="E149" s="18" t="n"/>
+      <c r="A149" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B149" s="18" t="inlineStr">
+        <is>
+          <t>Eliane Lisboa Silva</t>
+        </is>
+      </c>
+      <c r="C149" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D149" s="27" t="n">
+        <v>200</v>
+      </c>
+      <c r="E149" s="18" t="inlineStr">
+        <is>
+          <t>Dinheiro</t>
+        </is>
+      </c>
       <c r="F149" s="19" t="n"/>
       <c r="G149" s="19" t="n"/>
       <c r="H149" s="21" t="n"/>
       <c r="I149" s="18" t="n"/>
-      <c r="J149" s="18" t="n"/>
+      <c r="J149" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0908</t>
+        </is>
+      </c>
     </row>
     <row r="150">
-      <c r="A150" s="44" t="n"/>
-      <c r="B150" s="45" t="n"/>
-      <c r="C150" s="45" t="n"/>
-      <c r="D150" s="46" t="n"/>
-      <c r="E150" s="45" t="n"/>
+      <c r="A150" s="44" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B150" s="45" t="inlineStr">
+        <is>
+          <t>Studio Malena Lorrane</t>
+        </is>
+      </c>
+      <c r="C150" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="D150" s="46" t="n">
+        <v>150</v>
+      </c>
+      <c r="E150" s="45" t="inlineStr">
+        <is>
+          <t>Aguardando Pagamento</t>
+        </is>
+      </c>
       <c r="F150" s="47" t="n"/>
       <c r="G150" s="48" t="n"/>
       <c r="H150" s="49" t="n"/>
-      <c r="I150" s="45" t="n"/>
+      <c r="I150" s="45" t="inlineStr">
+        <is>
+          <t>Venda de R$ 190,00: Refil Everest R$ 130,00 + Pré Filtro R$ 60,00 (o pré-filtro antigo, de 2020, da saída de água foi trocado na hora). R$ 40,00 do refil foram pagos com serviço de sobrancelha feito para a Edilânia; ficou devendo R$ 150,00 (R$ 90,00 do refil + R$ 60,00 do pré-filtro).</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>EMP-0283</t>
+        </is>
+      </c>
     </row>
     <row r="151">
-      <c r="A151" s="17" t="n"/>
-      <c r="B151" s="18" t="n"/>
+      <c r="A151" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B151" s="18" t="inlineStr">
+        <is>
+          <t>Edivandro De Jesus Bispo</t>
+        </is>
+      </c>
       <c r="C151" s="18" t="n"/>
       <c r="D151" s="27" t="n"/>
       <c r="E151" s="18" t="n"/>
       <c r="F151" s="19" t="n"/>
-      <c r="G151" s="19" t="n"/>
-      <c r="H151" s="21" t="n"/>
-      <c r="I151" s="18" t="n"/>
+      <c r="G151" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="H151" s="21" t="inlineStr">
+        <is>
+          <t>Manutenção e Reparos</t>
+        </is>
+      </c>
+      <c r="I151" s="18" t="inlineStr">
+        <is>
+          <t>Colocação de piso vinílico na loja, na área perto do banheiro. Pix de R$ 200,00 em 21/10/2026 09:56 pelo Banco do Nordeste (ID E07237373202610211255VN1BQCN2DOB).</t>
+        </is>
+      </c>
       <c r="J151" s="18" t="n"/>
     </row>
     <row r="152">
@@ -67367,7 +67428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G171"/>
+  <dimension ref="A1:G181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="157" min="1" max="1"/>
@@ -72367,52 +72428,182 @@
       </c>
     </row>
     <row r="168" s="157">
-      <c r="A168" s="86" t="inlineStr">
+      <c r="A168" s="78" t="inlineStr">
+        <is>
+          <t>Studio Malena Lorrane</t>
+        </is>
+      </c>
+      <c r="B168" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro (restante)</t>
+        </is>
+      </c>
+      <c r="C168" s="77" t="n">
+        <v>46316</v>
+      </c>
+      <c r="D168" s="79" t="n">
+        <v>150</v>
+      </c>
+      <c r="E168" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F168" s="112">
+        <f>IF(OR($E168="Recebido",$C168=""),"",MAX(0,TODAY()-$C168))</f>
+        <v/>
+      </c>
+      <c r="G168" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 21/10/2026. Venda de R$ 190,00; R$ 40,00 pagos com serviço de sobrancelha para a Edilânia. Deve R$ 90,00 do refil + R$ 60,00 do pré-filtro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" s="157">
+      <c r="A169" s="78" t="n"/>
+      <c r="B169" s="78" t="n"/>
+      <c r="C169" s="77" t="n"/>
+      <c r="D169" s="79" t="n"/>
+      <c r="E169" s="112" t="n"/>
+      <c r="F169" s="112">
+        <f>IF(OR($E169="Recebido",$C169=""),"",MAX(0,TODAY()-$C169))</f>
+        <v/>
+      </c>
+      <c r="G169" s="78" t="n"/>
+    </row>
+    <row r="170" s="157">
+      <c r="A170" s="78" t="n"/>
+      <c r="B170" s="78" t="n"/>
+      <c r="C170" s="77" t="n"/>
+      <c r="D170" s="79" t="n"/>
+      <c r="E170" s="112" t="n"/>
+      <c r="F170" s="112">
+        <f>IF(OR($E170="Recebido",$C170=""),"",MAX(0,TODAY()-$C170))</f>
+        <v/>
+      </c>
+      <c r="G170" s="78" t="n"/>
+    </row>
+    <row r="171" s="157">
+      <c r="A171" s="78" t="n"/>
+      <c r="B171" s="78" t="n"/>
+      <c r="C171" s="77" t="n"/>
+      <c r="D171" s="79" t="n"/>
+      <c r="E171" s="112" t="n"/>
+      <c r="F171" s="112">
+        <f>IF(OR($E171="Recebido",$C171=""),"",MAX(0,TODAY()-$C171))</f>
+        <v/>
+      </c>
+      <c r="G171" s="78" t="n"/>
+    </row>
+    <row r="172" s="157">
+      <c r="A172" s="78" t="n"/>
+      <c r="B172" s="78" t="n"/>
+      <c r="C172" s="77" t="n"/>
+      <c r="D172" s="79" t="n"/>
+      <c r="E172" s="112" t="n"/>
+      <c r="F172" s="112">
+        <f>IF(OR($E172="Recebido",$C172=""),"",MAX(0,TODAY()-$C172))</f>
+        <v/>
+      </c>
+      <c r="G172" s="78" t="n"/>
+    </row>
+    <row r="173" s="157">
+      <c r="A173" s="78" t="n"/>
+      <c r="B173" s="78" t="n"/>
+      <c r="C173" s="77" t="n"/>
+      <c r="D173" s="79" t="n"/>
+      <c r="E173" s="112" t="n"/>
+      <c r="F173" s="112">
+        <f>IF(OR($E173="Recebido",$C173=""),"",MAX(0,TODAY()-$C173))</f>
+        <v/>
+      </c>
+      <c r="G173" s="78" t="n"/>
+    </row>
+    <row r="174" s="157">
+      <c r="A174" s="78" t="n"/>
+      <c r="B174" s="78" t="n"/>
+      <c r="C174" s="77" t="n"/>
+      <c r="D174" s="79" t="n"/>
+      <c r="E174" s="112" t="n"/>
+      <c r="F174" s="112">
+        <f>IF(OR($E174="Recebido",$C174=""),"",MAX(0,TODAY()-$C174))</f>
+        <v/>
+      </c>
+      <c r="G174" s="78" t="n"/>
+    </row>
+    <row r="175" s="157">
+      <c r="A175" s="78" t="n"/>
+      <c r="B175" s="78" t="n"/>
+      <c r="C175" s="77" t="n"/>
+      <c r="D175" s="79" t="n"/>
+      <c r="E175" s="112" t="n"/>
+      <c r="F175" s="112">
+        <f>IF(OR($E175="Recebido",$C175=""),"",MAX(0,TODAY()-$C175))</f>
+        <v/>
+      </c>
+      <c r="G175" s="78" t="n"/>
+    </row>
+    <row r="176" s="157">
+      <c r="A176" s="78" t="n"/>
+      <c r="B176" s="78" t="n"/>
+      <c r="C176" s="77" t="n"/>
+      <c r="D176" s="79" t="n"/>
+      <c r="E176" s="112" t="n"/>
+      <c r="F176" s="112">
+        <f>IF(OR($E176="Recebido",$C176=""),"",MAX(0,TODAY()-$C176))</f>
+        <v/>
+      </c>
+      <c r="G176" s="78" t="n"/>
+    </row>
+    <row r="177" s="157">
+      <c r="A177" s="78" t="n"/>
+      <c r="B177" s="78" t="n"/>
+      <c r="C177" s="77" t="n"/>
+      <c r="D177" s="79" t="n"/>
+      <c r="E177" s="112" t="n"/>
+      <c r="F177" s="112">
+        <f>IF(OR($E177="Recebido",$C177=""),"",MAX(0,TODAY()-$C177))</f>
+        <v/>
+      </c>
+      <c r="G177" s="78" t="n"/>
+    </row>
+    <row r="178" s="157">
+      <c r="A178" s="86" t="inlineStr">
         <is>
           <t>TOTAL EM ABERTO A RECEBER (detalhe)</t>
         </is>
       </c>
-      <c r="D168" s="115">
-        <f>SUMIF(E107:E167,"Pendente",D107:D167)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="169" s="157">
-      <c r="A169" s="202" t="inlineStr">
+      <c r="D178" s="115">
+        <f>SUMIF(E107:E177,"Pendente",D107:D177)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="179" s="157">
+      <c r="A179" s="202" t="inlineStr">
         <is>
           <t>CONFERÊNCIA COM AS ABAS DOS MESES</t>
         </is>
       </c>
-      <c r="B169" s="159" t="n"/>
-      <c r="C169" s="159" t="n"/>
-      <c r="D169" s="159" t="n"/>
-      <c r="E169" s="159" t="n"/>
-      <c r="F169" s="159" t="n"/>
-      <c r="G169" s="160" t="n"/>
-    </row>
-    <row r="170" s="157">
-      <c r="A170" s="203">
-        <f>IF(ROUND(D168-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D168-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="171" s="157">
-      <c r="A171" s="203" t="inlineStr">
+      <c r="B179" s="159" t="n"/>
+      <c r="C179" s="159" t="n"/>
+      <c r="D179" s="159" t="n"/>
+      <c r="E179" s="159" t="n"/>
+      <c r="F179" s="159" t="n"/>
+      <c r="G179" s="160" t="n"/>
+    </row>
+    <row r="180" s="157">
+      <c r="A180" s="203">
+        <f>IF(ROUND(D178-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D178-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="181" s="157">
+      <c r="A181" s="203" t="inlineStr">
         <is>
           <t>As contas a pagar do DigiSat (pendentes até 27/07/2026) foram todas quitadas — confirmado em 19/08/2026. A única dívida em aberto hoje é o Capital de Giro do Banco do Brasil. Lance aqui novos compromissos conforme surgirem.</t>
         </is>
       </c>
     </row>
-    <row r="172" s="157"/>
-    <row r="173" s="157"/>
-    <row r="174" s="157"/>
-    <row r="175" s="157"/>
-    <row r="176" s="157"/>
-    <row r="177" s="157"/>
-    <row r="178" s="157"/>
-    <row r="179" s="157"/>
-    <row r="180" s="157"/>
-    <row r="181" s="157"/>
     <row r="182" s="157"/>
     <row r="183" s="157"/>
     <row r="184" s="157"/>
@@ -72441,10 +72632,19 @@
     <row r="207" s="157"/>
     <row r="208" s="157"/>
     <row r="209" s="157"/>
+    <row r="210" s="157"/>
+    <row r="211" s="157"/>
+    <row r="212" s="157"/>
+    <row r="213" s="157"/>
+    <row r="214" s="157"/>
+    <row r="215" s="157"/>
+    <row r="216" s="157"/>
+    <row r="217" s="157"/>
+    <row r="218" s="157"/>
+    <row r="219" s="157"/>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A169:G169"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
@@ -72454,14 +72654,15 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E5:F6"/>
     <mergeCell ref="A104:G104"/>
-    <mergeCell ref="A170:G170"/>
+    <mergeCell ref="A179:G179"/>
+    <mergeCell ref="A180:G180"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="E11:E99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Pago,Previsto"</formula1>
     </dataValidation>
-    <dataValidation sqref="E107:E167" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E107:E177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Recebido"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Atualizacao do painel - 21/10/2026 14:35
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -57758,84 +57758,203 @@
       <c r="J151" s="18" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="44" t="n"/>
-      <c r="B152" s="45" t="n"/>
-      <c r="C152" s="45" t="n"/>
-      <c r="D152" s="46" t="n"/>
-      <c r="E152" s="45" t="n"/>
-      <c r="F152" s="47" t="n"/>
+      <c r="A152" s="44" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B152" s="45" t="inlineStr">
+        <is>
+          <t>Miralva Lopes da Silva</t>
+        </is>
+      </c>
+      <c r="C152" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D152" s="46" t="n">
+        <v>140</v>
+      </c>
+      <c r="E152" s="45" t="inlineStr">
+        <is>
+          <t>Débito</t>
+        </is>
+      </c>
+      <c r="F152" s="47" t="n">
+        <v>2.03</v>
+      </c>
       <c r="G152" s="48" t="n"/>
       <c r="H152" s="49" t="n"/>
       <c r="I152" s="45" t="n"/>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>CLI-0390</t>
+        </is>
+      </c>
     </row>
     <row r="153">
-      <c r="A153" s="17" t="n"/>
-      <c r="B153" s="18" t="n"/>
+      <c r="A153" s="17" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B153" s="18" t="inlineStr">
+        <is>
+          <t>Cezar Silva Atacado e Varejo (Iene Quedila Nunes Dourado)</t>
+        </is>
+      </c>
       <c r="C153" s="18" t="n"/>
       <c r="D153" s="27" t="n"/>
       <c r="E153" s="18" t="n"/>
       <c r="F153" s="19" t="n"/>
-      <c r="G153" s="19" t="n"/>
-      <c r="H153" s="21" t="n"/>
-      <c r="I153" s="18" t="n"/>
+      <c r="G153" s="19" t="n">
+        <v>40</v>
+      </c>
+      <c r="H153" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I153" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 16/10/2026.</t>
+        </is>
+      </c>
       <c r="J153" s="18" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="44" t="n"/>
-      <c r="B154" s="45" t="n"/>
+      <c r="A154" s="44" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B154" s="45" t="inlineStr">
+        <is>
+          <t>Thiago de Jesus Nascimento</t>
+        </is>
+      </c>
       <c r="C154" s="45" t="n"/>
       <c r="D154" s="46" t="n"/>
       <c r="E154" s="45" t="n"/>
       <c r="F154" s="47" t="n"/>
-      <c r="G154" s="48" t="n"/>
-      <c r="H154" s="49" t="n"/>
-      <c r="I154" s="45" t="n"/>
+      <c r="G154" s="48" t="n">
+        <v>28</v>
+      </c>
+      <c r="H154" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I154" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 19/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
-      <c r="A155" s="17" t="n"/>
-      <c r="B155" s="18" t="n"/>
+      <c r="A155" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B155" s="18" t="inlineStr">
+        <is>
+          <t>Japedido Software</t>
+        </is>
+      </c>
       <c r="C155" s="18" t="n"/>
       <c r="D155" s="27" t="n"/>
       <c r="E155" s="18" t="n"/>
       <c r="F155" s="19" t="n"/>
-      <c r="G155" s="19" t="n"/>
-      <c r="H155" s="21" t="n"/>
-      <c r="I155" s="18" t="n"/>
+      <c r="G155" s="19" t="n">
+        <v>38.99</v>
+      </c>
+      <c r="H155" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I155" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 20/10/2026.</t>
+        </is>
+      </c>
       <c r="J155" s="18" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="44" t="n"/>
-      <c r="B156" s="45" t="n"/>
+      <c r="A156" s="44" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B156" s="45" t="inlineStr">
+        <is>
+          <t>Maria Eva dos Santos</t>
+        </is>
+      </c>
       <c r="C156" s="45" t="n"/>
       <c r="D156" s="46" t="n"/>
       <c r="E156" s="45" t="n"/>
       <c r="F156" s="47" t="n"/>
-      <c r="G156" s="48" t="n"/>
-      <c r="H156" s="49" t="n"/>
-      <c r="I156" s="45" t="n"/>
+      <c r="G156" s="48" t="n">
+        <v>350</v>
+      </c>
+      <c r="H156" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I156" s="45" t="inlineStr">
+        <is>
+          <t>Extrato Stone — saída de 20/10/2026. Diarista — não é o mesmo pagamento da "Diarista Eva" de R$ 400,00 de 17/10.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
-      <c r="A157" s="17" t="n"/>
-      <c r="B157" s="18" t="n"/>
+      <c r="A157" s="17" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B157" s="18" t="inlineStr">
+        <is>
+          <t>Uellinton Silva de Jesus</t>
+        </is>
+      </c>
       <c r="C157" s="18" t="n"/>
       <c r="D157" s="27" t="n"/>
       <c r="E157" s="18" t="n"/>
       <c r="F157" s="19" t="n"/>
-      <c r="G157" s="19" t="n"/>
-      <c r="H157" s="21" t="n"/>
-      <c r="I157" s="18" t="n"/>
+      <c r="G157" s="19" t="n">
+        <v>80</v>
+      </c>
+      <c r="H157" s="21" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I157" s="18" t="inlineStr">
+        <is>
+          <t>Extrato Stone — Pix de 20/10/2026 18:58 (CNPJ 18.097.008/0001-83). Lançado como gasto pessoal — confirmar com a Edilânia.</t>
+        </is>
+      </c>
       <c r="J157" s="18" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="44" t="n"/>
-      <c r="B158" s="45" t="n"/>
+      <c r="A158" s="44" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B158" s="45" t="inlineStr">
+        <is>
+          <t>Fatura Claro TV (Embratel)</t>
+        </is>
+      </c>
       <c r="C158" s="45" t="n"/>
       <c r="D158" s="46" t="n"/>
       <c r="E158" s="45" t="n"/>
       <c r="F158" s="47" t="n"/>
-      <c r="G158" s="48" t="n"/>
-      <c r="H158" s="49" t="n"/>
-      <c r="I158" s="45" t="n"/>
+      <c r="G158" s="48" t="n">
+        <v>249.7</v>
+      </c>
+      <c r="H158" s="49" t="inlineStr">
+        <is>
+          <t>Pro Labore Edilânia</t>
+        </is>
+      </c>
+      <c r="I158" s="45" t="inlineStr">
+        <is>
+          <t>TV de casa — despesa pessoal. Pix de R$ 249,70 em 21/10/2026 14:26 pelo Banco do Nordeste para Embratel (ID E07237373202610211726RDWOGZX74RT).</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="17" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 21/10/2026 18:07
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -56926,7 +56926,7 @@
       </c>
       <c r="I125" s="18" t="inlineStr">
         <is>
-          <t>Pedido da Edilânia em 17/10/2026 — despesa pessoal.</t>
+          <t>Pedido da Edilânia em 17/10/2026 — despesa pessoal. Pago em dinheiro (confirmado em 21/10/2026: é diferente do Pix de R$ 350,00 de 20/10).</t>
         </is>
       </c>
       <c r="J125" s="18" t="n"/>
@@ -57897,7 +57897,7 @@
       </c>
       <c r="I156" s="45" t="inlineStr">
         <is>
-          <t>Extrato Stone — saída de 20/10/2026. Diarista — não é o mesmo pagamento da "Diarista Eva" de R$ 400,00 de 17/10.</t>
+          <t>Extrato Stone — Pix de 20/10/2026. Diarista — pagamento diferente do de 17/10 (R$ 400,00 em dinheiro); confirmado pela Edilânia em 21/10/2026.</t>
         </is>
       </c>
     </row>
@@ -57907,7 +57907,7 @@
       </c>
       <c r="B157" s="18" t="inlineStr">
         <is>
-          <t>Uellinton Silva de Jesus</t>
+          <t>Mensalidade Academia (Uellinton Silva de Jesus)</t>
         </is>
       </c>
       <c r="C157" s="18" t="n"/>
@@ -57924,7 +57924,7 @@
       </c>
       <c r="I157" s="18" t="inlineStr">
         <is>
-          <t>Extrato Stone — Pix de 20/10/2026 18:58 (CNPJ 18.097.008/0001-83). Lançado como gasto pessoal — confirmar com a Edilânia.</t>
+          <t>Extrato Stone — Pix de 20/10/2026 18:58 (CNPJ 18.097.008/0001-83). Mensalidade da academia — despesa pessoal (confirmado pela Edilânia em 21/10/2026).</t>
         </is>
       </c>
       <c r="J157" s="18" t="n"/>
@@ -57957,38 +57957,94 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="17" t="n"/>
-      <c r="B159" s="18" t="n"/>
-      <c r="C159" s="18" t="n"/>
-      <c r="D159" s="27" t="n"/>
-      <c r="E159" s="18" t="n"/>
+      <c r="A159" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B159" s="18" t="inlineStr">
+        <is>
+          <t>Marmoraria Pedra Bella LTDA</t>
+        </is>
+      </c>
+      <c r="C159" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D159" s="27" t="n">
+        <v>135</v>
+      </c>
+      <c r="E159" s="18" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F159" s="19" t="n"/>
       <c r="G159" s="19" t="n"/>
       <c r="H159" s="21" t="n"/>
-      <c r="I159" s="18" t="n"/>
-      <c r="J159" s="18" t="n"/>
+      <c r="I159" s="18" t="inlineStr">
+        <is>
+          <t>Cliente comprou o refil e fez a troca por conta própria em 19/10/2026 (sem serviço da loja).</t>
+        </is>
+      </c>
+      <c r="J159" s="18" t="inlineStr">
+        <is>
+          <t>EMP-0215</t>
+        </is>
+      </c>
     </row>
     <row r="160">
-      <c r="A160" s="44" t="n"/>
-      <c r="B160" s="45" t="n"/>
+      <c r="A160" s="44" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B160" s="45" t="inlineStr">
+        <is>
+          <t>Filtros Planeta Água</t>
+        </is>
+      </c>
       <c r="C160" s="45" t="n"/>
       <c r="D160" s="46" t="n"/>
       <c r="E160" s="45" t="n"/>
       <c r="F160" s="47" t="n"/>
-      <c r="G160" s="48" t="n"/>
-      <c r="H160" s="49" t="n"/>
-      <c r="I160" s="45" t="n"/>
+      <c r="G160" s="48" t="n">
+        <v>537.9299999999999</v>
+      </c>
+      <c r="H160" s="49" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I160" s="45" t="inlineStr">
+        <is>
+          <t>Comprado: 10x Refil Fit PP 9.3/4" + 5x Refil Universal Rosca Curta + 5x Refil Universal Rosca Longa + 5x Refil Universal Rosca Média + 5x Refil Top Color + 3x Refil Acquatec + 5x Refil CP500 + 30x Refil Carbon Tech 9" + 20x Refil Plissado 9.3/4" (Poli Flu) + 5x Refil E3 Compacto + Carcaça Fit 9.3/4" Branca (rosca 1/2") (NF-e 133138 de 12/08/2026, nota de R$ 2.263,62 em 4 boletos). Boleto doc. 133138/4 (emissão 12/08/2026) · parcela 4/4 (última) — venc. 21/10/2026. Pago em 21/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="161">
-      <c r="A161" s="17" t="n"/>
-      <c r="B161" s="18" t="n"/>
+      <c r="A161" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B161" s="18" t="inlineStr">
+        <is>
+          <t>Everest Refrigeração</t>
+        </is>
+      </c>
       <c r="C161" s="18" t="n"/>
       <c r="D161" s="27" t="n"/>
       <c r="E161" s="18" t="n"/>
       <c r="F161" s="19" t="n"/>
-      <c r="G161" s="19" t="n"/>
-      <c r="H161" s="21" t="n"/>
-      <c r="I161" s="18" t="n"/>
+      <c r="G161" s="19" t="n">
+        <v>613.12</v>
+      </c>
+      <c r="H161" s="21" t="inlineStr">
+        <is>
+          <t>Fornecedores / Mercadoria</t>
+        </is>
+      </c>
+      <c r="I161" s="18" t="inlineStr">
+        <is>
+          <t>Comprado: Purificador Everest Fit Prata + Purificador Everest Slim Preto + Purificador Everest Star Preto + Purificador Everest Plus Preto (NF-e 386838 de 23/09/2026, nota de R$ 3.065,60 em 5 boletos). Boleto doc. 386838 (emissão 23/09/2026) · parcela 1/5 — venc. 23/10/2026. Pago antecipado em 21/10/2026.</t>
+        </is>
+      </c>
       <c r="J161" s="18" t="n"/>
     </row>
     <row r="162">
@@ -69209,7 +69265,7 @@
       </c>
       <c r="E59" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F59" s="112">
@@ -69218,7 +69274,7 @@
       </c>
       <c r="G59" s="78" t="inlineStr">
         <is>
-          <t>Comprado: 10x Refil Fit PP 9.3/4" + 5x Refil Universal Rosca Curta + 5x Refil Universal Rosca Longa + 5x Refil Universal Rosca Média + 5x Refil Top Color + 3x Refil Acquatec + 5x Refil CP500 + 30x Refil Carbon Tech 9" + 20x Refil Plissado 9.3/4" (Poli Flu) + 5x Refil E3 Compacto + Carcaça Fit 9.3/4" Branca (rosca 1/2") (NF-e 133138 de 12/08/2026, nota de R$ 2.263,62 em 4 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109). Nosso número 109/00257852-2. Linha digitável 34191.09008 25785.221430 81531.550002 6 16060000053793. Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133138 (emissão 12/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.263,62 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 43260805097806000163550010001331381847671397.</t>
+          <t>Comprado: 10x Refil Fit PP 9.3/4" + 5x Refil Universal Rosca Curta + 5x Refil Universal Rosca Longa + 5x Refil Universal Rosca Média + 5x Refil Top Color + 3x Refil Acquatec + 5x Refil CP500 + 30x Refil Carbon Tech 9" + 20x Refil Plissado 9.3/4" (Poli Flu) + 5x Refil E3 Compacto + Carcaça Fit 9.3/4" Branca (rosca 1/2") (NF-e 133138 de 12/08/2026, nota de R$ 2.263,62 em 4 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7 (carteira 109). Nosso número 109/00257852-2. Linha digitável 34191.09008 25785.221430 81531.550002 6 16060000053793. Após o vencimento: multa de 1,9% + juros de 0,1% ao dia; protesto no 5º dia útil. | Conferido com o XML da NF-e nº 133138 (emissão 12/08/2026): FILTROS PLANETA AGUA INDUSTRIA E COMERCIO LTDA, CNPJ 05.097.806/0001-63, RUA FRANCISCO BALBINOT, 139, SAO ROQUE, FARROUPILHA/RS. Valor total da nota R$ 2.263,62 em 4 parcelas. Frete CIF (frete por conta do fornecedor), transportadora PATRUS TRANSPORTES URGENTES. Chave da NF-e 43260805097806000163550010001331381847671397. Pago em 21/10/2026 — lançado em "Out 2026" como "Filtros Planeta Água".</t>
         </is>
       </c>
     </row>
@@ -69721,7 +69777,7 @@
       </c>
       <c r="E75" s="113" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Pago</t>
         </is>
       </c>
       <c r="F75" s="113">
@@ -69730,7 +69786,7 @@
       </c>
       <c r="G75" s="82" t="inlineStr">
         <is>
-          <t>Comprado: Purificador Everest Fit Prata + Purificador Everest Slim Preto + Purificador Everest Star Preto + Purificador Everest Plus Preto (NF-e 386838 de 23/09/2026, nota de R$ 3.065,60 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910774. Linha digitável 34191.12366 91077.460300 52238.850003 1 16080000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210.</t>
+          <t>Comprado: Purificador Everest Fit Prata + Purificador Everest Slim Preto + Purificador Everest Star Preto + Purificador Everest Plus Preto (NF-e 386838 de 23/09/2026, nota de R$ 3.065,60 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/36910774. Linha digitável 34191.12366 91077.460300 52238.850003 1 16080000061312. Boleto recebido por e-mail em 23/09/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 386838". Após o vencimento: multa de 2% + juros de R$ 0,20 ao dia. | Conferido com o XML da NF-e nº 386838 (emissão 23/09/2026): EVEREST REFRIGERACAO INDUSTRIA E COMERCIO LTDA., CNPJ 33.079.641/0001-32, RUA CARDOSO QUINTAO, 914, TOMAS COELHO, RIO DE JANEIRO/RJ. Valor total da nota R$ 3.065,60 em 5 parcelas. Frete FOB (frete por conta da loja), transportadora PATRUS TRANSPORTES URGENTES LTDA. Chave da NF-e 33260933079641000132550020003868381733266210. Pago em 21/10/2026 — lançado em "Out 2026" como "Everest Refrigeração".</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao do painel - 21/10/2026 18:08
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -58048,11 +58048,27 @@
       <c r="J161" s="18" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="44" t="n"/>
-      <c r="B162" s="45" t="n"/>
-      <c r="C162" s="45" t="n"/>
-      <c r="D162" s="46" t="n"/>
-      <c r="E162" s="45" t="n"/>
+      <c r="A162" s="44" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B162" s="45" t="inlineStr">
+        <is>
+          <t>Consumidor Final</t>
+        </is>
+      </c>
+      <c r="C162" s="45" t="inlineStr">
+        <is>
+          <t>Conexão Reta Rosca</t>
+        </is>
+      </c>
+      <c r="D162" s="46" t="n">
+        <v>25</v>
+      </c>
+      <c r="E162" s="45" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F162" s="47" t="n"/>
       <c r="G162" s="48" t="n"/>
       <c r="H162" s="49" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 22/10/2026 18:16
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -56747,7 +56747,7 @@
       </c>
       <c r="B119" s="18" t="inlineStr">
         <is>
-          <t>Eduardo Santos da Silva</t>
+          <t>Tania Dourado - Eduardo Dourado</t>
         </is>
       </c>
       <c r="C119" s="18" t="inlineStr">
@@ -56769,7 +56769,7 @@
       <c r="I119" s="18" t="n"/>
       <c r="J119" s="18" t="inlineStr">
         <is>
-          <t>CLI-0408</t>
+          <t>CLI-0525</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao do painel - 23/10/2026 11:58
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -58118,27 +58118,70 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="44" t="n"/>
-      <c r="B164" s="45" t="n"/>
-      <c r="C164" s="45" t="n"/>
-      <c r="D164" s="46" t="n"/>
-      <c r="E164" s="45" t="n"/>
+      <c r="A164" s="44" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B164" s="45" t="inlineStr">
+        <is>
+          <t>Alessandra Carvalho Vieira - Paulo Sergio</t>
+        </is>
+      </c>
+      <c r="C164" s="45" t="inlineStr">
+        <is>
+          <t>Refil Everest + Mangueira</t>
+        </is>
+      </c>
+      <c r="D164" s="46" t="n">
+        <v>150</v>
+      </c>
+      <c r="E164" s="45" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F164" s="47" t="n"/>
       <c r="G164" s="48" t="n"/>
       <c r="H164" s="49" t="n"/>
       <c r="I164" s="45" t="n"/>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>CLI-0586</t>
+        </is>
+      </c>
     </row>
     <row r="165">
-      <c r="A165" s="17" t="n"/>
-      <c r="B165" s="18" t="n"/>
-      <c r="C165" s="18" t="n"/>
-      <c r="D165" s="27" t="n"/>
-      <c r="E165" s="18" t="n"/>
-      <c r="F165" s="19" t="n"/>
+      <c r="A165" s="17" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B165" s="18" t="inlineStr">
+        <is>
+          <t>Rita Mesquita</t>
+        </is>
+      </c>
+      <c r="C165" s="18" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="D165" s="27" t="n">
+        <v>140</v>
+      </c>
+      <c r="E165" s="18" t="inlineStr">
+        <is>
+          <t>Crédito à Vista</t>
+        </is>
+      </c>
+      <c r="F165" s="19" t="n">
+        <v>4.91</v>
+      </c>
       <c r="G165" s="19" t="n"/>
       <c r="H165" s="21" t="n"/>
       <c r="I165" s="18" t="n"/>
-      <c r="J165" s="18" t="n"/>
+      <c r="J165" s="18" t="inlineStr">
+        <is>
+          <t>CLI-0554</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="44" t="n"/>

</xml_diff>

<commit_message>
Atualizacao do painel - 23/10/2026 18:04
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -67693,7 +67693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G181"/>
+  <dimension ref="A1:G188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="157" min="1" max="1"/>
@@ -67744,7 +67744,7 @@
     </row>
     <row r="5">
       <c r="A5" s="189">
-        <f>D102</f>
+        <f>D109</f>
         <v/>
       </c>
       <c r="C5" s="204">
@@ -70649,1013 +70649,1013 @@
       </c>
     </row>
     <row r="100" s="157">
-      <c r="A100" s="86" t="inlineStr">
+      <c r="A100" s="82" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B100" s="82" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 389424 (emissão 22/10/2026) · parcela 1/5</t>
+        </is>
+      </c>
+      <c r="C100" s="81" t="n">
+        <v>46347</v>
+      </c>
+      <c r="D100" s="83" t="n">
+        <v>675.84</v>
+      </c>
+      <c r="E100" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F100" s="113">
+        <f>IF(OR($E100="Pago",$C100=""),"",MAX(0,TODAY()-$C100))</f>
+        <v/>
+      </c>
+      <c r="G100" s="82" t="inlineStr">
+        <is>
+          <t>Comprado: Purificador Everest Star Branco + Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Slim Preto + 4x Purificador Everest Baby Preto (NF-e 389424 de 22/10/2026, nota de R$ 3.379,19 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/40350414. Linha digitável 34191.12408 35041.480308 52238.850003 7 16370000067584. Boleto recebido por e-mail em 22/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 389424". Após o vencimento: multa de 2% + juros de R$ 0,23 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" s="157">
+      <c r="A101" s="82" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B101" s="82" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 389424 (emissão 22/10/2026) · parcela 2/5</t>
+        </is>
+      </c>
+      <c r="C101" s="81" t="n">
+        <v>46377</v>
+      </c>
+      <c r="D101" s="83" t="n">
+        <v>675.84</v>
+      </c>
+      <c r="E101" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F101" s="113">
+        <f>IF(OR($E101="Pago",$C101=""),"",MAX(0,TODAY()-$C101))</f>
+        <v/>
+      </c>
+      <c r="G101" s="82" t="inlineStr">
+        <is>
+          <t>Comprado: Purificador Everest Star Branco + Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Slim Preto + 4x Purificador Everest Baby Preto (NF-e 389424 de 22/10/2026, nota de R$ 3.379,19 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/40350342. Linha digitável 34191.12408 35034.210308 52238.850003 7 16670000067584. Boleto recebido por e-mail em 22/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 389424". Após o vencimento: multa de 2% + juros de R$ 0,23 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" s="157">
+      <c r="A102" s="82" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B102" s="82" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 389424 (emissão 22/10/2026) · parcela 3/5</t>
+        </is>
+      </c>
+      <c r="C102" s="81" t="n">
+        <v>46407</v>
+      </c>
+      <c r="D102" s="83" t="n">
+        <v>675.84</v>
+      </c>
+      <c r="E102" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F102" s="113">
+        <f>IF(OR($E102="Pago",$C102=""),"",MAX(0,TODAY()-$C102))</f>
+        <v/>
+      </c>
+      <c r="G102" s="82" t="inlineStr">
+        <is>
+          <t>Comprado: Purificador Everest Star Branco + Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Slim Preto + 4x Purificador Everest Baby Preto (NF-e 389424 de 22/10/2026, nota de R$ 3.379,19 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/40350264. Linha digitável 34191.12408 35026.470308 52238.850003 3 16970000067584. Boleto recebido por e-mail em 22/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 389424". Após o vencimento: multa de 2% + juros de R$ 0,23 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" s="157">
+      <c r="A103" s="82" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B103" s="82" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 389424 (emissão 22/10/2026) · parcela 4/5</t>
+        </is>
+      </c>
+      <c r="C103" s="81" t="n">
+        <v>46437</v>
+      </c>
+      <c r="D103" s="83" t="n">
+        <v>675.84</v>
+      </c>
+      <c r="E103" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F103" s="113">
+        <f>IF(OR($E103="Pago",$C103=""),"",MAX(0,TODAY()-$C103))</f>
+        <v/>
+      </c>
+      <c r="G103" s="82" t="inlineStr">
+        <is>
+          <t>Comprado: Purificador Everest Star Branco + Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Slim Preto + 4x Purificador Everest Baby Preto (NF-e 389424 de 22/10/2026, nota de R$ 3.379,19 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/40350393. Linha digitável 34191.12408 35039.340308 52238.850003 5 17270000067584. Boleto recebido por e-mail em 22/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 389424". Após o vencimento: multa de 2% + juros de R$ 0,23 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" s="157">
+      <c r="A104" s="82" t="inlineStr">
+        <is>
+          <t>Everest Refrigeracao e Industria</t>
+        </is>
+      </c>
+      <c r="B104" s="82" t="inlineStr">
+        <is>
+          <t>Mercadoria — doc. 389424 (emissão 22/10/2026) · parcela 5/5 (última)</t>
+        </is>
+      </c>
+      <c r="C104" s="81" t="n">
+        <v>46467</v>
+      </c>
+      <c r="D104" s="83" t="n">
+        <v>675.83</v>
+      </c>
+      <c r="E104" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F104" s="113">
+        <f>IF(OR($E104="Pago",$C104=""),"",MAX(0,TODAY()-$C104))</f>
+        <v/>
+      </c>
+      <c r="G104" s="82" t="inlineStr">
+        <is>
+          <t>Comprado: Purificador Everest Star Branco + Purificador Everest Fit Branco + Purificador Everest Slim Branco + Purificador Everest Slim Preto + 4x Purificador Everest Baby Preto (NF-e 389424 de 22/10/2026, nota de R$ 3.379,19 em 5 boletos). Categoria quando pagar: Fornecedores / Mercadoria. Boleto Itaú 341-7. Nosso número 112/40350359. Linha digitável 34191.12408 35035.950308 52238.850003 4 17570000067583. Boleto recebido por e-mail em 22/10/2026; PDF salvo em "03 - Despesas e Contas a Pagar/Boletos Everest NF 389424". Após o vencimento: multa de 2% + juros de R$ 0,23 ao dia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" s="157">
+      <c r="A105" s="82" t="inlineStr">
+        <is>
+          <t>SEFAZ-BA — DAE ICMS Antecipação Parcial</t>
+        </is>
+      </c>
+      <c r="B105" s="82" t="inlineStr">
+        <is>
+          <t>ICMS Antecipação Parcial — referência 09/2026 (cód. receita 2175, nº 1971838234)</t>
+        </is>
+      </c>
+      <c r="C105" s="81" t="n">
+        <v>46320</v>
+      </c>
+      <c r="D105" s="83" t="n">
+        <v>983.48</v>
+      </c>
+      <c r="E105" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F105" s="113">
+        <f>IF(OR($E105="Pago",$C105=""),"",MAX(0,TODAY()-$C105))</f>
+        <v/>
+      </c>
+      <c r="G105" s="82" t="inlineStr">
+        <is>
+          <t>Categoria quando pagar: Impostos e Taxas. Inscrição Estadual 066.200.856 — Planeta Agua Ltda, CNPJ 07.341.784/0001-60. Notas fiscais da guia (4): 386188 // 134720 // 386838 // 387488. Código de barras 85820000009 0 83480005202 7 61026197183 8 82342175193 2. Pode pagar por código de barras ou Pix (QR Code). Guia emitida em 19/10/2026; vale para pagamento até 26/10/2026 — depois disso precisa emitir outro DAE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" s="157">
+      <c r="A106" s="82" t="inlineStr">
+        <is>
+          <t>Empresa Baiana de Aguas e Saneamento SA (Embasa)</t>
+        </is>
+      </c>
+      <c r="B106" s="82" t="inlineStr">
+        <is>
+          <t>Conta de água — despesa pessoal do dono (não é da loja) — ref. 11/2026</t>
+        </is>
+      </c>
+      <c r="C106" s="81" t="n">
+        <v>46327</v>
+      </c>
+      <c r="D106" s="83" t="n">
+        <v>51.85</v>
+      </c>
+      <c r="E106" s="113" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F106" s="113">
+        <f>IF(OR($E106="Pago",$C106=""),"",MAX(0,TODAY()-$C106))</f>
+        <v/>
+      </c>
+      <c r="G106" s="82" t="inlineStr">
+        <is>
+          <t>Categoria quando pagar: Pro Labore Edilânia (despesa pessoal do dono). Conta em nome de Adriano Silva Fontes, matrícula 0531718-70, consumo 10 m³. Código de barras 82600000000-8 51850047820-2 53171870112-5 60000000000-7. Pode pagar por Pix (QR Code da conta).</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" s="157">
+      <c r="A107" s="86" t="inlineStr">
         <is>
           <t>TOTAL A PAGAR — COM BOLETO EM MÃOS</t>
         </is>
       </c>
-      <c r="B100" s="86" t="n"/>
-      <c r="C100" s="114" t="n"/>
-      <c r="D100" s="115">
-        <f>SUMIF(E11:E99,"Pendente",D11:D99)</f>
-        <v/>
-      </c>
-      <c r="E100" s="116" t="n"/>
-      <c r="F100" s="116" t="n"/>
-      <c r="G100" s="86" t="n"/>
-    </row>
-    <row r="101" s="157">
-      <c r="A101" s="144" t="inlineStr">
+      <c r="B107" s="86" t="n"/>
+      <c r="C107" s="114" t="n"/>
+      <c r="D107" s="115">
+        <f>SUMIF(E11:E106,"Pendente",D11:D106)</f>
+        <v/>
+      </c>
+      <c r="E107" s="116" t="n"/>
+      <c r="F107" s="116" t="n"/>
+      <c r="G107" s="86" t="n"/>
+    </row>
+    <row r="108" s="157">
+      <c r="A108" s="144" t="inlineStr">
         <is>
           <t>PREVISTO — compromisso certo que ainda não está documentado</t>
         </is>
       </c>
-      <c r="B101" s="144" t="n"/>
-      <c r="C101" s="145" t="n"/>
-      <c r="D101" s="146">
-        <f>SUMIF(E11:E99,"Previsto",D11:D99)</f>
-        <v/>
-      </c>
-      <c r="E101" s="142" t="n"/>
-      <c r="F101" s="142" t="n"/>
-      <c r="G101" s="144" t="n"/>
-    </row>
-    <row r="102" s="157">
-      <c r="A102" s="86" t="inlineStr">
+      <c r="B108" s="144" t="n"/>
+      <c r="C108" s="145" t="n"/>
+      <c r="D108" s="146">
+        <f>SUMIF(E11:E106,"Previsto",D11:D106)</f>
+        <v/>
+      </c>
+      <c r="E108" s="142" t="n"/>
+      <c r="F108" s="142" t="n"/>
+      <c r="G108" s="144" t="n"/>
+    </row>
+    <row r="109" s="157">
+      <c r="A109" s="86" t="inlineStr">
         <is>
           <t>TOTAL GERAL A PAGAR (boletos + previsão)</t>
         </is>
       </c>
-      <c r="B102" s="86" t="n"/>
-      <c r="C102" s="114" t="n"/>
-      <c r="D102" s="115">
-        <f>D100+D101</f>
-        <v/>
-      </c>
-      <c r="E102" s="116" t="n"/>
-      <c r="F102" s="116" t="n"/>
-      <c r="G102" s="86" t="n"/>
-    </row>
-    <row r="103" ht="15.75" customHeight="1" s="157"/>
-    <row r="104" ht="15.75" customHeight="1" s="157">
-      <c r="A104" s="200" t="inlineStr">
+      <c r="B109" s="86" t="n"/>
+      <c r="C109" s="114" t="n"/>
+      <c r="D109" s="115">
+        <f>D107+D108</f>
+        <v/>
+      </c>
+      <c r="E109" s="116" t="n"/>
+      <c r="F109" s="116" t="n"/>
+      <c r="G109" s="86" t="n"/>
+    </row>
+    <row r="110" ht="15.75" customHeight="1" s="157"/>
+    <row r="111" ht="15.75" customHeight="1" s="157">
+      <c r="A111" s="200" t="inlineStr">
         <is>
           <t>CONTAS A RECEBER  —  vendas feitas e ainda não pagas</t>
         </is>
       </c>
     </row>
-    <row r="105" s="157">
-      <c r="A105" s="194" t="inlineStr">
+    <row r="112" s="157">
+      <c r="A112" s="194" t="inlineStr">
         <is>
           <t>Espelho das vendas marcadas como "Aguardando Pagamento" nas abas dos meses. Ao receber, mude a Forma de Pagamento na aba do mês E o Status aqui. A linha de conferência avisa se os dois deixarem de bater.</t>
         </is>
       </c>
     </row>
-    <row r="106" s="157">
-      <c r="A106" s="111" t="inlineStr">
+    <row r="113" s="157">
+      <c r="A113" s="111" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="B106" s="111" t="inlineStr">
+      <c r="B113" s="111" t="inlineStr">
         <is>
           <t>Produto / Referência</t>
         </is>
       </c>
-      <c r="C106" s="111" t="inlineStr">
+      <c r="C113" s="111" t="inlineStr">
         <is>
           <t>Data da Venda</t>
         </is>
       </c>
-      <c r="D106" s="111" t="inlineStr">
+      <c r="D113" s="111" t="inlineStr">
         <is>
           <t>Valor (R$)</t>
         </is>
       </c>
-      <c r="E106" s="111" t="inlineStr">
+      <c r="E113" s="111" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F106" s="111" t="inlineStr">
+      <c r="F113" s="111" t="inlineStr">
         <is>
           <t>Dias em Atraso</t>
         </is>
       </c>
-      <c r="G106" s="111" t="inlineStr">
+      <c r="G113" s="111" t="inlineStr">
         <is>
           <t>Observações</t>
         </is>
       </c>
     </row>
-    <row r="107" s="157">
-      <c r="A107" s="78" t="inlineStr">
+    <row r="114" s="157">
+      <c r="A114" s="78" t="inlineStr">
         <is>
           <t>Centro de Especialidades Odontomédicas</t>
         </is>
       </c>
-      <c r="B107" s="78" t="inlineStr">
+      <c r="B114" s="78" t="inlineStr">
         <is>
           <t>Refil Everest</t>
         </is>
       </c>
-      <c r="C107" s="77" t="n">
+      <c r="C114" s="77" t="n">
         <v>46239</v>
       </c>
-      <c r="D107" s="79" t="n">
+      <c r="D114" s="79" t="n">
         <v>140</v>
       </c>
-      <c r="E107" s="112" t="inlineStr">
+      <c r="E114" s="112" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
-      <c r="F107" s="112">
-        <f>IF(OR($E107="Recebido",$C107=""),"",MAX(0,TODAY()-$C107))</f>
-        <v/>
-      </c>
-      <c r="G107" s="78" t="n"/>
-    </row>
-    <row r="108" s="157">
-      <c r="A108" s="82" t="inlineStr">
+      <c r="F114" s="112">
+        <f>IF(OR($E114="Recebido",$C114=""),"",MAX(0,TODAY()-$C114))</f>
+        <v/>
+      </c>
+      <c r="G114" s="78" t="n"/>
+    </row>
+    <row r="115" s="157">
+      <c r="A115" s="82" t="inlineStr">
         <is>
           <t>Supermercado Brasil</t>
         </is>
       </c>
-      <c r="B108" s="82" t="inlineStr">
+      <c r="B115" s="82" t="inlineStr">
         <is>
           <t>2x Refil Pro Life</t>
         </is>
       </c>
-      <c r="C108" s="81" t="n">
+      <c r="C115" s="81" t="n">
         <v>46239</v>
       </c>
-      <c r="D108" s="83" t="n">
+      <c r="D115" s="83" t="n">
         <v>280</v>
       </c>
-      <c r="E108" s="113" t="inlineStr">
+      <c r="E115" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F108" s="113">
-        <f>IF(OR($E108="Recebido",$C108=""),"",MAX(0,TODAY()-$C108))</f>
-        <v/>
-      </c>
-      <c r="G108" s="82" t="inlineStr">
+      <c r="F115" s="113">
+        <f>IF(OR($E115="Recebido",$C115=""),"",MAX(0,TODAY()-$C115))</f>
+        <v/>
+      </c>
+      <c r="G115" s="82" t="inlineStr">
         <is>
           <t>Recebido via Pix em 22/10/2026 — lançado em "Out 2026".</t>
         </is>
       </c>
     </row>
-    <row r="109" s="157">
-      <c r="A109" s="78" t="inlineStr">
+    <row r="116" s="157">
+      <c r="A116" s="78" t="inlineStr">
         <is>
           <t>Tropical Motos LTDA</t>
         </is>
       </c>
-      <c r="B109" s="78" t="inlineStr">
+      <c r="B116" s="78" t="inlineStr">
         <is>
           <t>3x Refil Everest + Refil Pro Life + 3x Pré Filtro + Válvula Reguladora de Pressão</t>
         </is>
       </c>
-      <c r="C109" s="77" t="n">
+      <c r="C116" s="77" t="n">
         <v>46245</v>
       </c>
-      <c r="D109" s="79" t="n">
+      <c r="D116" s="79" t="n">
         <v>820</v>
       </c>
-      <c r="E109" s="112" t="inlineStr">
+      <c r="E116" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F109" s="112">
-        <f>IF(OR($E109="Recebido",$C109=""),"",MAX(0,TODAY()-$C109))</f>
-        <v/>
-      </c>
-      <c r="G109" s="78" t="inlineStr">
+      <c r="F116" s="112">
+        <f>IF(OR($E116="Recebido",$C116=""),"",MAX(0,TODAY()-$C116))</f>
+        <v/>
+      </c>
+      <c r="G116" s="78" t="inlineStr">
         <is>
           <t>Recebido via TED em 25/08/2026. NF conferida: valor correto é R$820 (faltava a válvula no lançamento original de R$740).</t>
         </is>
       </c>
     </row>
-    <row r="110" s="157">
-      <c r="A110" s="82" t="inlineStr">
+    <row r="117" s="157">
+      <c r="A117" s="82" t="inlineStr">
         <is>
           <t>Free Way</t>
         </is>
       </c>
-      <c r="B110" s="82" t="inlineStr">
+      <c r="B117" s="82" t="inlineStr">
         <is>
           <t>5x Refil Everest</t>
         </is>
       </c>
-      <c r="C110" s="81" t="n">
+      <c r="C117" s="81" t="n">
         <v>46251</v>
       </c>
-      <c r="D110" s="83" t="n">
+      <c r="D117" s="83" t="n">
         <v>700</v>
       </c>
-      <c r="E110" s="113" t="inlineStr">
+      <c r="E117" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F110" s="113">
-        <f>IF(OR($E110="Recebido",$C110=""),"",MAX(0,TODAY()-$C110))</f>
-        <v/>
-      </c>
-      <c r="G110" s="82" t="inlineStr">
+      <c r="F117" s="113">
+        <f>IF(OR($E117="Recebido",$C117=""),"",MAX(0,TODAY()-$C117))</f>
+        <v/>
+      </c>
+      <c r="G117" s="82" t="inlineStr">
         <is>
           <t>Recebido via TED em 02/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="111" s="157">
-      <c r="A111" s="78" t="inlineStr">
+    <row r="118" s="157">
+      <c r="A118" s="78" t="inlineStr">
         <is>
           <t>Neli Sena Rego</t>
         </is>
       </c>
-      <c r="B111" s="78" t="inlineStr">
+      <c r="B118" s="78" t="inlineStr">
         <is>
           <t>Refil Pro Life</t>
         </is>
       </c>
-      <c r="C111" s="77" t="n">
+      <c r="C118" s="77" t="n">
         <v>46254</v>
       </c>
-      <c r="D111" s="79" t="n">
+      <c r="D118" s="79" t="n">
         <v>140</v>
       </c>
-      <c r="E111" s="112" t="inlineStr">
+      <c r="E118" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F111" s="112">
-        <f>IF(OR($E111="Recebido",$C111=""),"",MAX(0,TODAY()-$C111))</f>
-        <v/>
-      </c>
-      <c r="G111" s="78" t="inlineStr">
+      <c r="F118" s="112">
+        <f>IF(OR($E118="Recebido",$C118=""),"",MAX(0,TODAY()-$C118))</f>
+        <v/>
+      </c>
+      <c r="G118" s="78" t="inlineStr">
         <is>
           <t>Recebido em dinheiro em 01/09/2026 (R$ 170,00 pelas duas vendas)</t>
         </is>
       </c>
     </row>
-    <row r="112" s="157">
-      <c r="A112" s="82" t="inlineStr">
+    <row r="119" s="157">
+      <c r="A119" s="82" t="inlineStr">
         <is>
           <t>Neli Sena Rego</t>
         </is>
       </c>
-      <c r="B112" s="82" t="inlineStr">
+      <c r="B119" s="82" t="inlineStr">
         <is>
           <t>Conexão + Mangueira</t>
         </is>
       </c>
-      <c r="C112" s="81" t="n">
+      <c r="C119" s="81" t="n">
         <v>46255</v>
       </c>
-      <c r="D112" s="83" t="n">
+      <c r="D119" s="83" t="n">
         <v>40</v>
       </c>
-      <c r="E112" s="113" t="inlineStr">
+      <c r="E119" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F112" s="113">
-        <f>IF(OR($E112="Recebido",$C112=""),"",MAX(0,TODAY()-$C112))</f>
-        <v/>
-      </c>
-      <c r="G112" s="82" t="inlineStr">
+      <c r="F119" s="113">
+        <f>IF(OR($E119="Recebido",$C119=""),"",MAX(0,TODAY()-$C119))</f>
+        <v/>
+      </c>
+      <c r="G119" s="82" t="inlineStr">
         <is>
           <t>Recebido em dinheiro em 01/09/2026 (R$ 170,00 pelas duas vendas)</t>
         </is>
       </c>
     </row>
-    <row r="113" s="157">
-      <c r="A113" s="78" t="inlineStr">
+    <row r="120" s="157">
+      <c r="A120" s="78" t="inlineStr">
         <is>
           <t>Lapec</t>
         </is>
       </c>
-      <c r="B113" s="78" t="inlineStr">
+      <c r="B120" s="78" t="inlineStr">
         <is>
           <t>4x Refil Everest</t>
         </is>
       </c>
-      <c r="C113" s="77" t="n">
+      <c r="C120" s="77" t="n">
         <v>46258</v>
       </c>
-      <c r="D113" s="79" t="n">
+      <c r="D120" s="79" t="n">
         <v>480</v>
       </c>
-      <c r="E113" s="112" t="inlineStr">
+      <c r="E120" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F113" s="112">
-        <f>IF(OR($E113="Recebido",$C113=""),"",MAX(0,TODAY()-$C113))</f>
-        <v/>
-      </c>
-      <c r="G113" s="78" t="inlineStr">
+      <c r="F120" s="112">
+        <f>IF(OR($E120="Recebido",$C120=""),"",MAX(0,TODAY()-$C120))</f>
+        <v/>
+      </c>
+      <c r="G120" s="78" t="inlineStr">
         <is>
           <t>Recebido em dinheiro em 08/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
-    <row r="114" s="157">
-      <c r="A114" s="82" t="inlineStr">
+    <row r="121" s="157">
+      <c r="A121" s="82" t="inlineStr">
         <is>
           <t>Cícero Lima</t>
         </is>
       </c>
-      <c r="B114" s="82" t="inlineStr">
+      <c r="B121" s="82" t="inlineStr">
         <is>
           <t>Refil Everest</t>
         </is>
       </c>
-      <c r="C114" s="81" t="n">
+      <c r="C121" s="81" t="n">
         <v>46261</v>
       </c>
-      <c r="D114" s="83" t="n">
+      <c r="D121" s="83" t="n">
         <v>140</v>
       </c>
-      <c r="E114" s="113" t="inlineStr">
+      <c r="E121" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F114" s="113">
-        <f>IF(OR($E114="Recebido",$C114=""),"",MAX(0,TODAY()-$C114))</f>
-        <v/>
-      </c>
-      <c r="G114" s="82" t="inlineStr">
+      <c r="F121" s="113">
+        <f>IF(OR($E121="Recebido",$C121=""),"",MAX(0,TODAY()-$C121))</f>
+        <v/>
+      </c>
+      <c r="G121" s="82" t="inlineStr">
         <is>
           <t>Recebido via Pix em 27/08/2026</t>
         </is>
       </c>
     </row>
-    <row r="115" s="157">
-      <c r="A115" s="78" t="inlineStr">
+    <row r="122" s="157">
+      <c r="A122" s="78" t="inlineStr">
         <is>
           <t>Promotoria Regional de Jacobina</t>
         </is>
       </c>
-      <c r="B115" s="78" t="inlineStr">
+      <c r="B122" s="78" t="inlineStr">
         <is>
           <t>2x Carcaça 9" + 2x Refil Plissado 9" + Conexão Reta Rosca</t>
         </is>
       </c>
-      <c r="C115" s="77" t="n">
+      <c r="C122" s="77" t="n">
         <v>46261</v>
       </c>
-      <c r="D115" s="79" t="n">
+      <c r="D122" s="79" t="n">
         <v>470</v>
       </c>
-      <c r="E115" s="112" t="inlineStr">
+      <c r="E122" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F115" s="112">
-        <f>IF(OR($E115="Recebido",$C115=""),"",MAX(0,TODAY()-$C115))</f>
-        <v/>
-      </c>
-      <c r="G115" s="78" t="inlineStr">
+      <c r="F122" s="112">
+        <f>IF(OR($E122="Recebido",$C122=""),"",MAX(0,TODAY()-$C122))</f>
+        <v/>
+      </c>
+      <c r="G122" s="78" t="inlineStr">
         <is>
           <t>Pago em 28/08/2026 em duas formas: R$ 270,00 Pix + R$ 200,00 crédito 2x</t>
         </is>
       </c>
     </row>
-    <row r="116" s="157">
-      <c r="A116" s="82" t="inlineStr">
+    <row r="123" s="157">
+      <c r="A123" s="82" t="inlineStr">
         <is>
           <t>Lucas Souza</t>
         </is>
       </c>
-      <c r="B116" s="82" t="inlineStr">
+      <c r="B123" s="82" t="inlineStr">
         <is>
           <t>Refil Everest + Pré Filtro</t>
         </is>
       </c>
-      <c r="C116" s="81" t="n">
+      <c r="C123" s="81" t="n">
         <v>46261</v>
       </c>
-      <c r="D116" s="83" t="n">
+      <c r="D123" s="83" t="n">
         <v>200</v>
       </c>
-      <c r="E116" s="113" t="inlineStr">
+      <c r="E123" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F116" s="113">
-        <f>IF(OR($E116="Recebido",$C116=""),"",MAX(0,TODAY()-$C116))</f>
-        <v/>
-      </c>
-      <c r="G116" s="82" t="inlineStr">
+      <c r="F123" s="113">
+        <f>IF(OR($E123="Recebido",$C123=""),"",MAX(0,TODAY()-$C123))</f>
+        <v/>
+      </c>
+      <c r="G123" s="82" t="inlineStr">
         <is>
           <t>Recebido em dinheiro em 03/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
-    <row r="117" s="157">
-      <c r="A117" s="78" t="inlineStr">
+    <row r="124" s="157">
+      <c r="A124" s="78" t="inlineStr">
         <is>
           <t>FG Boa Vista (Recife/PE)</t>
         </is>
       </c>
-      <c r="B117" s="78" t="inlineStr">
+      <c r="B124" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C117" s="77" t="n">
+      <c r="C124" s="77" t="n">
         <v>46261</v>
       </c>
-      <c r="D117" s="79" t="n">
+      <c r="D124" s="79" t="n">
         <v>1008.8</v>
       </c>
-      <c r="E117" s="112" t="inlineStr">
+      <c r="E124" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F117" s="112">
-        <f>IF(OR($E117="Recebido",$C117=""),"",MAX(0,TODAY()-$C117))</f>
-        <v/>
-      </c>
-      <c r="G117" s="78" t="inlineStr">
+      <c r="F124" s="112">
+        <f>IF(OR($E124="Recebido",$C124=""),"",MAX(0,TODAY()-$C124))</f>
+        <v/>
+      </c>
+      <c r="G124" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.280 · recebido em 30/08/2026 (Nota Paga no portal V360)</t>
         </is>
       </c>
     </row>
-    <row r="118" s="157">
-      <c r="A118" s="82" t="inlineStr">
+    <row r="125" s="157">
+      <c r="A125" s="82" t="inlineStr">
         <is>
           <t>UNIFG Guanambi (Guanambi/BA)</t>
         </is>
       </c>
-      <c r="B118" s="82" t="inlineStr">
+      <c r="B125" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C118" s="81" t="n">
+      <c r="C125" s="81" t="n">
         <v>46261</v>
       </c>
-      <c r="D118" s="83" t="n">
+      <c r="D125" s="83" t="n">
         <v>4534.75</v>
       </c>
-      <c r="E118" s="113" t="inlineStr">
+      <c r="E125" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F118" s="113">
-        <f>IF(OR($E118="Recebido",$C118=""),"",MAX(0,TODAY()-$C118))</f>
-        <v/>
-      </c>
-      <c r="G118" s="82" t="inlineStr">
+      <c r="F125" s="113">
+        <f>IF(OR($E125="Recebido",$C125=""),"",MAX(0,TODAY()-$C125))</f>
+        <v/>
+      </c>
+      <c r="G125" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.281 · recebido em 30/08/2026 (Nota Paga no portal V360)</t>
         </is>
       </c>
     </row>
-    <row r="119" s="157">
-      <c r="A119" s="78" t="inlineStr">
+    <row r="126" s="157">
+      <c r="A126" s="78" t="inlineStr">
         <is>
           <t>UNP Zona Norte (Natal/RN)</t>
         </is>
       </c>
-      <c r="B119" s="78" t="inlineStr">
+      <c r="B126" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C119" s="77" t="n">
+      <c r="C126" s="77" t="n">
         <v>46261</v>
       </c>
-      <c r="D119" s="79" t="n">
+      <c r="D126" s="79" t="n">
         <v>870</v>
       </c>
-      <c r="E119" s="112" t="inlineStr">
+      <c r="E126" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F119" s="112">
-        <f>IF(OR($E119="Recebido",$C119=""),"",MAX(0,TODAY()-$C119))</f>
-        <v/>
-      </c>
-      <c r="G119" s="78" t="inlineStr">
+      <c r="F126" s="112">
+        <f>IF(OR($E126="Recebido",$C126=""),"",MAX(0,TODAY()-$C126))</f>
+        <v/>
+      </c>
+      <c r="G126" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.282 · recebido em 30/08/2026 (Nota Paga no portal V360)</t>
         </is>
       </c>
     </row>
-    <row r="120" s="157">
-      <c r="A120" s="82" t="inlineStr">
+    <row r="127" s="157">
+      <c r="A127" s="82" t="inlineStr">
         <is>
           <t>UNP Caicó (Caicó/RN)</t>
         </is>
       </c>
-      <c r="B120" s="82" t="inlineStr">
+      <c r="B127" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C120" s="81" t="n">
+      <c r="C127" s="81" t="n">
         <v>46261</v>
       </c>
-      <c r="D120" s="83" t="n">
+      <c r="D127" s="83" t="n">
         <v>440</v>
       </c>
-      <c r="E120" s="113" t="inlineStr">
+      <c r="E127" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F120" s="113">
-        <f>IF(OR($E120="Recebido",$C120=""),"",MAX(0,TODAY()-$C120))</f>
-        <v/>
-      </c>
-      <c r="G120" s="82" t="inlineStr">
+      <c r="F127" s="113">
+        <f>IF(OR($E127="Recebido",$C127=""),"",MAX(0,TODAY()-$C127))</f>
+        <v/>
+      </c>
+      <c r="G127" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.283 · recebido via Pix em 27/08/2026</t>
         </is>
       </c>
     </row>
-    <row r="121" s="157">
-      <c r="A121" s="78" t="inlineStr">
+    <row r="128" s="157">
+      <c r="A128" s="78" t="inlineStr">
         <is>
           <t>AGES Irecê (Irecê/BA)</t>
         </is>
       </c>
-      <c r="B121" s="78" t="inlineStr">
+      <c r="B128" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C121" s="77" t="n">
+      <c r="C128" s="77" t="n">
         <v>46269</v>
       </c>
-      <c r="D121" s="79" t="n">
+      <c r="D128" s="79" t="n">
         <v>1338.6</v>
       </c>
-      <c r="E121" s="112" t="inlineStr">
+      <c r="E128" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F121" s="112">
-        <f>IF(OR($E121="Recebido",$C121=""),"",MAX(0,TODAY()-$C121))</f>
-        <v/>
-      </c>
-      <c r="G121" s="78" t="inlineStr">
+      <c r="F128" s="112">
+        <f>IF(OR($E128="Recebido",$C128=""),"",MAX(0,TODAY()-$C128))</f>
+        <v/>
+      </c>
+      <c r="G128" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.294 · recebido via Pix em 04/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="122" s="157">
-      <c r="A122" s="82" t="inlineStr">
+    <row r="129" s="157">
+      <c r="A129" s="82" t="inlineStr">
         <is>
           <t>CIS Irecê (Irecê/BA)</t>
         </is>
       </c>
-      <c r="B122" s="82" t="inlineStr">
+      <c r="B129" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C122" s="81" t="n">
+      <c r="C129" s="81" t="n">
         <v>46269</v>
       </c>
-      <c r="D122" s="83" t="n">
+      <c r="D129" s="83" t="n">
         <v>1358</v>
       </c>
-      <c r="E122" s="113" t="inlineStr">
+      <c r="E129" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F122" s="113">
-        <f>IF(OR($E122="Recebido",$C122=""),"",MAX(0,TODAY()-$C122))</f>
-        <v/>
-      </c>
-      <c r="G122" s="82" t="inlineStr">
+      <c r="F129" s="113">
+        <f>IF(OR($E129="Recebido",$C129=""),"",MAX(0,TODAY()-$C129))</f>
+        <v/>
+      </c>
+      <c r="G129" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.295 · recebido via Pix em 04/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="123" s="157">
-      <c r="A123" s="78" t="inlineStr">
+    <row r="130" s="157">
+      <c r="A130" s="78" t="inlineStr">
         <is>
           <t>AGES Senhor do Bonfim (S. do Bonfim/BA)</t>
         </is>
       </c>
-      <c r="B123" s="78" t="inlineStr">
+      <c r="B130" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C123" s="77" t="n">
+      <c r="C130" s="77" t="n">
         <v>46270</v>
       </c>
-      <c r="D123" s="79" t="n">
+      <c r="D130" s="79" t="n">
         <v>649.9</v>
       </c>
-      <c r="E123" s="112" t="inlineStr">
+      <c r="E130" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F123" s="112">
-        <f>IF(OR($E123="Recebido",$C123=""),"",MAX(0,TODAY()-$C123))</f>
-        <v/>
-      </c>
-      <c r="G123" s="78" t="inlineStr">
+      <c r="F130" s="112">
+        <f>IF(OR($E130="Recebido",$C130=""),"",MAX(0,TODAY()-$C130))</f>
+        <v/>
+      </c>
+      <c r="G130" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.298 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="124" s="157">
-      <c r="A124" s="82" t="inlineStr">
+    <row r="131" s="157">
+      <c r="A131" s="82" t="inlineStr">
         <is>
           <t>CIS Senhor do Bonfim (S. do Bonfim/BA)</t>
         </is>
       </c>
-      <c r="B124" s="82" t="inlineStr">
+      <c r="B131" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C124" s="81" t="n">
+      <c r="C131" s="81" t="n">
         <v>46270</v>
       </c>
-      <c r="D124" s="83" t="n">
+      <c r="D131" s="83" t="n">
         <v>562.6</v>
       </c>
-      <c r="E124" s="113" t="inlineStr">
+      <c r="E131" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F124" s="113">
-        <f>IF(OR($E124="Recebido",$C124=""),"",MAX(0,TODAY()-$C124))</f>
-        <v/>
-      </c>
-      <c r="G124" s="82" t="inlineStr">
+      <c r="F131" s="113">
+        <f>IF(OR($E131="Recebido",$C131=""),"",MAX(0,TODAY()-$C131))</f>
+        <v/>
+      </c>
+      <c r="G131" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.299 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="125" s="157">
-      <c r="A125" s="78" t="inlineStr">
+    <row r="132" s="157">
+      <c r="A132" s="78" t="inlineStr">
         <is>
           <t>AGES Paripiranga (Paripiranga/BA)</t>
         </is>
       </c>
-      <c r="B125" s="78" t="inlineStr">
+      <c r="B132" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C125" s="77" t="n">
+      <c r="C132" s="77" t="n">
         <v>46270</v>
       </c>
-      <c r="D125" s="79" t="n">
+      <c r="D132" s="79" t="n">
         <v>1086.4</v>
       </c>
-      <c r="E125" s="112" t="inlineStr">
+      <c r="E132" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F125" s="112">
-        <f>IF(OR($E125="Recebido",$C125=""),"",MAX(0,TODAY()-$C125))</f>
-        <v/>
-      </c>
-      <c r="G125" s="78" t="inlineStr">
+      <c r="F132" s="112">
+        <f>IF(OR($E132="Recebido",$C132=""),"",MAX(0,TODAY()-$C132))</f>
+        <v/>
+      </c>
+      <c r="G132" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.300 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="126" s="157">
-      <c r="A126" s="82" t="inlineStr">
+    <row r="133" s="157">
+      <c r="A133" s="82" t="inlineStr">
         <is>
           <t>Clínica Veterinária Paripiranga (Paripiranga/BA)</t>
         </is>
       </c>
-      <c r="B126" s="82" t="inlineStr">
+      <c r="B133" s="82" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C126" s="81" t="n">
+      <c r="C133" s="81" t="n">
         <v>46270</v>
       </c>
-      <c r="D126" s="83" t="n">
+      <c r="D133" s="83" t="n">
         <v>1265.85</v>
       </c>
-      <c r="E126" s="113" t="inlineStr">
+      <c r="E133" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F126" s="113">
-        <f>IF(OR($E126="Recebido",$C126=""),"",MAX(0,TODAY()-$C126))</f>
-        <v/>
-      </c>
-      <c r="G126" s="82" t="inlineStr">
+      <c r="F133" s="113">
+        <f>IF(OR($E133="Recebido",$C133=""),"",MAX(0,TODAY()-$C133))</f>
+        <v/>
+      </c>
+      <c r="G133" s="82" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.301 · recebido via Pix em 08/09/2026.</t>
         </is>
       </c>
     </row>
-    <row r="127" s="157">
-      <c r="A127" s="78" t="inlineStr">
+    <row r="134" s="157">
+      <c r="A134" s="78" t="inlineStr">
         <is>
           <t>UNP Mossoró (Mossoró/RN)</t>
         </is>
       </c>
-      <c r="B127" s="78" t="inlineStr">
+      <c r="B134" s="78" t="inlineStr">
         <is>
           <t>Refis — troca de julho/2026</t>
         </is>
       </c>
-      <c r="C127" s="77" t="n">
+      <c r="C134" s="77" t="n">
         <v>46270</v>
       </c>
-      <c r="D127" s="79" t="n">
+      <c r="D134" s="79" t="n">
         <v>1867.25</v>
       </c>
-      <c r="E127" s="112" t="inlineStr">
+      <c r="E134" s="112" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F127" s="112">
-        <f>IF(OR($E127="Recebido",$C127=""),"",MAX(0,TODAY()-$C127))</f>
-        <v/>
-      </c>
-      <c r="G127" s="78" t="inlineStr">
+      <c r="F134" s="112">
+        <f>IF(OR($E134="Recebido",$C134=""),"",MAX(0,TODAY()-$C134))</f>
+        <v/>
+      </c>
+      <c r="G134" s="78" t="inlineStr">
         <is>
           <t>Grupo Ânima — NF 000.004.302 · recebido via Pix em 08/09/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" s="157">
-      <c r="A128" s="82" t="inlineStr">
-        <is>
-          <t>CIS Jacobina (Jacobina/BA)</t>
-        </is>
-      </c>
-      <c r="B128" s="82" t="inlineStr">
-        <is>
-          <t>Refis — troca de julho/2026</t>
-        </is>
-      </c>
-      <c r="C128" s="81" t="n">
-        <v>46290</v>
-      </c>
-      <c r="D128" s="83" t="n">
-        <v>2095.2</v>
-      </c>
-      <c r="E128" s="113" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F128" s="113">
-        <f>IF(OR($E128="Recebido",$C128=""),"",MAX(0,TODAY()-$C128))</f>
-        <v/>
-      </c>
-      <c r="G128" s="82" t="inlineStr">
-        <is>
-          <t>Grupo Ânima — NF 000.004.333 de 26/08/2026 · OC AEMPPO00004452 · 30 dias · recebido via Pix em 25/09/2026 (Nota Paga no portal V360).</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" s="157">
-      <c r="A129" s="78" t="inlineStr">
-        <is>
-          <t>AGES Jacobina (Jacobina/BA)</t>
-        </is>
-      </c>
-      <c r="B129" s="78" t="inlineStr">
-        <is>
-          <t>Refis — troca de julho/2026</t>
-        </is>
-      </c>
-      <c r="C129" s="77" t="n">
-        <v>46305</v>
-      </c>
-      <c r="D129" s="79" t="n">
-        <v>1188.25</v>
-      </c>
-      <c r="E129" s="112" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F129" s="112">
-        <f>IF(OR($E129="Recebido",$C129=""),"",MAX(0,TODAY()-$C129))</f>
-        <v/>
-      </c>
-      <c r="G129" s="78" t="inlineStr">
-        <is>
-          <t>Grupo Ânima — NF 000.004.332 de 26/08/2026 · OC AEMPPO00004453 · 45 dias · Recebido em 13/10/2026 no BNB (Nota Paga no portal V360).</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" s="157">
-      <c r="A130" s="82" t="inlineStr">
-        <is>
-          <t>Instituto Paulo Leão</t>
-        </is>
-      </c>
-      <c r="B130" s="82" t="inlineStr">
-        <is>
-          <t>Refil E3 + Pré Filtro</t>
-        </is>
-      </c>
-      <c r="C130" s="81" t="n">
-        <v>46265</v>
-      </c>
-      <c r="D130" s="83" t="n">
-        <v>160</v>
-      </c>
-      <c r="E130" s="113" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F130" s="113">
-        <f>IF(OR($E130="Recebido",$C130=""),"",MAX(0,TODAY()-$C130))</f>
-        <v/>
-      </c>
-      <c r="G130" s="82" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 08/09/2026 — lançado em "Set 2026".</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" s="157">
-      <c r="A131" s="78" t="inlineStr">
-        <is>
-          <t>Eletronic Segurança Eletronica</t>
-        </is>
-      </c>
-      <c r="B131" s="78" t="inlineStr">
-        <is>
-          <t>Pré Filtro</t>
-        </is>
-      </c>
-      <c r="C131" s="77" t="n">
-        <v>46265</v>
-      </c>
-      <c r="D131" s="79" t="n">
-        <v>60</v>
-      </c>
-      <c r="E131" s="112" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F131" s="112">
-        <f>IF(OR($E131="Recebido",$C131=""),"",MAX(0,TODAY()-$C131))</f>
-        <v/>
-      </c>
-      <c r="G131" s="78" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 03/09/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" s="157">
-      <c r="A132" s="82" t="inlineStr">
-        <is>
-          <t>Clube dos Mineiros</t>
-        </is>
-      </c>
-      <c r="B132" s="82" t="inlineStr">
-        <is>
-          <t>Refil Pro Life</t>
-        </is>
-      </c>
-      <c r="C132" s="81" t="n">
-        <v>46265</v>
-      </c>
-      <c r="D132" s="83" t="n">
-        <v>150</v>
-      </c>
-      <c r="E132" s="113" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F132" s="113">
-        <f>IF(OR($E132="Recebido",$C132=""),"",MAX(0,TODAY()-$C132))</f>
-        <v/>
-      </c>
-      <c r="G132" s="82" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 01/09/2026 (pagador: Sindicato dos Mineiros de Jacobina).</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" s="157">
-      <c r="A133" s="78" t="inlineStr">
-        <is>
-          <t>Armazem Cecilio Mota</t>
-        </is>
-      </c>
-      <c r="B133" s="78" t="inlineStr">
-        <is>
-          <t>Refil Everest + Refil Carbon 9"</t>
-        </is>
-      </c>
-      <c r="C133" s="77" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D133" s="79" t="n">
-        <v>225</v>
-      </c>
-      <c r="E133" s="112" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F133" s="112">
-        <f>IF(OR($E133="Recebido",$C133=""),"",MAX(0,TODAY()-$C133))</f>
-        <v/>
-      </c>
-      <c r="G133" s="78" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" s="157">
-      <c r="A134" s="82" t="inlineStr">
-        <is>
-          <t>Clebson Dantas Da Silva</t>
-        </is>
-      </c>
-      <c r="B134" s="82" t="inlineStr">
-        <is>
-          <t>Refil Everest</t>
-        </is>
-      </c>
-      <c r="C134" s="81" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D134" s="83" t="n">
-        <v>140</v>
-      </c>
-      <c r="E134" s="113" t="inlineStr">
-        <is>
-          <t>Recebido</t>
-        </is>
-      </c>
-      <c r="F134" s="113">
-        <f>IF(OR($E134="Recebido",$C134=""),"",MAX(0,TODAY()-$C134))</f>
-        <v/>
-      </c>
-      <c r="G134" s="82" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 02/09/2026</t>
         </is>
       </c>
     </row>
     <row r="135" s="157">
       <c r="A135" s="82" t="inlineStr">
         <is>
-          <t>Tesla Imagem Medicina Diagnostica Ltda</t>
+          <t>CIS Jacobina (Jacobina/BA)</t>
         </is>
       </c>
       <c r="B135" s="82" t="inlineStr">
         <is>
-          <t>3x Refil Everest + 2x Pré Filtro</t>
+          <t>Refis — troca de julho/2026</t>
         </is>
       </c>
       <c r="C135" s="81" t="n">
-        <v>46267</v>
+        <v>46290</v>
       </c>
       <c r="D135" s="83" t="n">
-        <v>540</v>
+        <v>2095.2</v>
       </c>
       <c r="E135" s="113" t="inlineStr">
         <is>
@@ -71668,26 +71668,26 @@
       </c>
       <c r="G135" s="82" t="inlineStr">
         <is>
-          <t>Troca do dia 02/09/2026 — 1º Andar, Térreo e Copa. Recebido via Pix em 08/09/2026 — lançado em "Set 2026".</t>
+          <t>Grupo Ânima — NF 000.004.333 de 26/08/2026 · OC AEMPPO00004452 · 30 dias · recebido via Pix em 25/09/2026 (Nota Paga no portal V360).</t>
         </is>
       </c>
     </row>
     <row r="136" s="157">
       <c r="A136" s="78" t="inlineStr">
         <is>
-          <t>Cecilio Mota Junior</t>
+          <t>AGES Jacobina (Jacobina/BA)</t>
         </is>
       </c>
       <c r="B136" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Refis — troca de julho/2026</t>
         </is>
       </c>
       <c r="C136" s="77" t="n">
-        <v>46267</v>
+        <v>46305</v>
       </c>
       <c r="D136" s="79" t="n">
-        <v>140</v>
+        <v>1188.25</v>
       </c>
       <c r="E136" s="112" t="inlineStr">
         <is>
@@ -71700,58 +71700,58 @@
       </c>
       <c r="G136" s="78" t="inlineStr">
         <is>
-          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
+          <t>Grupo Ânima — NF 000.004.332 de 26/08/2026 · OC AEMPPO00004453 · 45 dias · Recebido em 13/10/2026 no BNB (Nota Paga no portal V360).</t>
         </is>
       </c>
     </row>
     <row r="137" s="157">
-      <c r="A137" s="78" t="inlineStr">
-        <is>
-          <t>Tereza Cristina Aquino Martins - Luiz Augusto</t>
-        </is>
-      </c>
-      <c r="B137" s="78" t="inlineStr">
-        <is>
-          <t>Refil Everest + Pré Filtro</t>
-        </is>
-      </c>
-      <c r="C137" s="77" t="n">
-        <v>46268</v>
-      </c>
-      <c r="D137" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="E137" s="112" t="inlineStr">
+      <c r="A137" s="82" t="inlineStr">
+        <is>
+          <t>Instituto Paulo Leão</t>
+        </is>
+      </c>
+      <c r="B137" s="82" t="inlineStr">
+        <is>
+          <t>Refil E3 + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="C137" s="81" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D137" s="83" t="n">
+        <v>160</v>
+      </c>
+      <c r="E137" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F137" s="112">
+      <c r="F137" s="113">
         <f>IF(OR($E137="Recebido",$C137=""),"",MAX(0,TODAY()-$C137))</f>
         <v/>
       </c>
-      <c r="G137" s="78" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 04/09/2026.</t>
+      <c r="G137" s="82" t="inlineStr">
+        <is>
+          <t>Recebido via Pix em 08/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="138" s="157">
       <c r="A138" s="78" t="inlineStr">
         <is>
-          <t>Samille Fiscina Lima Lordello - Tiago (Cartório)</t>
+          <t>Eletronic Segurança Eletronica</t>
         </is>
       </c>
       <c r="B138" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life</t>
+          <t>Pré Filtro</t>
         </is>
       </c>
       <c r="C138" s="77" t="n">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="D138" s="79" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="E138" s="112" t="inlineStr">
         <is>
@@ -71764,58 +71764,58 @@
       </c>
       <c r="G138" s="78" t="inlineStr">
         <is>
-          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
+          <t>Recebido via Pix em 03/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="139" s="157">
-      <c r="A139" s="78" t="inlineStr">
-        <is>
-          <t>Bomboniere Doce Mania - Veronildo Basilio</t>
-        </is>
-      </c>
-      <c r="B139" s="78" t="inlineStr">
-        <is>
-          <t>Refil Plissado + Refil BAG</t>
-        </is>
-      </c>
-      <c r="C139" s="77" t="n">
-        <v>46274</v>
-      </c>
-      <c r="D139" s="79" t="n">
+      <c r="A139" s="82" t="inlineStr">
+        <is>
+          <t>Clube dos Mineiros</t>
+        </is>
+      </c>
+      <c r="B139" s="82" t="inlineStr">
+        <is>
+          <t>Refil Pro Life</t>
+        </is>
+      </c>
+      <c r="C139" s="81" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D139" s="83" t="n">
         <v>150</v>
       </c>
-      <c r="E139" s="112" t="inlineStr">
+      <c r="E139" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F139" s="112">
+      <c r="F139" s="113">
         <f>IF(OR($E139="Recebido",$C139=""),"",MAX(0,TODAY()-$C139))</f>
         <v/>
       </c>
-      <c r="G139" s="78" t="inlineStr">
-        <is>
-          <t>Recebido em dinheiro em 16/09/2026 — lançado em "Set 2026".</t>
+      <c r="G139" s="82" t="inlineStr">
+        <is>
+          <t>Recebido via Pix em 01/09/2026 (pagador: Sindicato dos Mineiros de Jacobina).</t>
         </is>
       </c>
     </row>
     <row r="140" s="157">
       <c r="A140" s="78" t="inlineStr">
         <is>
-          <t>Adriadne (Hotel Jovem Jota)</t>
+          <t>Armazem Cecilio Mota</t>
         </is>
       </c>
       <c r="B140" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Refil Everest + Refil Carbon 9"</t>
         </is>
       </c>
       <c r="C140" s="77" t="n">
-        <v>46275</v>
+        <v>46266</v>
       </c>
       <c r="D140" s="79" t="n">
-        <v>140</v>
+        <v>225</v>
       </c>
       <c r="E140" s="112" t="inlineStr">
         <is>
@@ -71828,78 +71828,78 @@
       </c>
       <c r="G140" s="78" t="inlineStr">
         <is>
-          <t>Recebido via Pix em 11/09/2026 — lançado em "Set 2026".</t>
+          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="141" s="157">
-      <c r="A141" s="78" t="inlineStr">
-        <is>
-          <t>Pousada Triunfo Ltda (Hotel Triunfo)</t>
-        </is>
-      </c>
-      <c r="B141" s="78" t="inlineStr">
-        <is>
-          <t>Refil Everest + Pré Filtro</t>
-        </is>
-      </c>
-      <c r="C141" s="77" t="n">
-        <v>46275</v>
-      </c>
-      <c r="D141" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="E141" s="112" t="inlineStr">
+      <c r="A141" s="82" t="inlineStr">
+        <is>
+          <t>Clebson Dantas Da Silva</t>
+        </is>
+      </c>
+      <c r="B141" s="82" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="C141" s="81" t="n">
+        <v>46266</v>
+      </c>
+      <c r="D141" s="83" t="n">
+        <v>140</v>
+      </c>
+      <c r="E141" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F141" s="112">
+      <c r="F141" s="113">
         <f>IF(OR($E141="Recebido",$C141=""),"",MAX(0,TODAY()-$C141))</f>
         <v/>
       </c>
-      <c r="G141" s="78" t="inlineStr">
-        <is>
-          <t>Recebido via Pix em 11/09/2026 — lançado em "Set 2026".</t>
+      <c r="G141" s="82" t="inlineStr">
+        <is>
+          <t>Recebido via Pix em 02/09/2026</t>
         </is>
       </c>
     </row>
     <row r="142" s="157">
-      <c r="A142" s="78" t="inlineStr">
-        <is>
-          <t>Topvel Tropical Veiculos e Pecas</t>
-        </is>
-      </c>
-      <c r="B142" s="78" t="inlineStr">
-        <is>
-          <t>2x Refil Everest + 2x Pré Filtro</t>
-        </is>
-      </c>
-      <c r="C142" s="77" t="n">
-        <v>46276</v>
-      </c>
-      <c r="D142" s="79" t="n">
-        <v>370</v>
-      </c>
-      <c r="E142" s="112" t="inlineStr">
+      <c r="A142" s="82" t="inlineStr">
+        <is>
+          <t>Tesla Imagem Medicina Diagnostica Ltda</t>
+        </is>
+      </c>
+      <c r="B142" s="82" t="inlineStr">
+        <is>
+          <t>3x Refil Everest + 2x Pré Filtro</t>
+        </is>
+      </c>
+      <c r="C142" s="81" t="n">
+        <v>46267</v>
+      </c>
+      <c r="D142" s="83" t="n">
+        <v>540</v>
+      </c>
+      <c r="E142" s="113" t="inlineStr">
         <is>
           <t>Recebido</t>
         </is>
       </c>
-      <c r="F142" s="112">
+      <c r="F142" s="113">
         <f>IF(OR($E142="Recebido",$C142=""),"",MAX(0,TODAY()-$C142))</f>
         <v/>
       </c>
-      <c r="G142" s="78" t="inlineStr">
-        <is>
-          <t>Troca do dia 11/09/2026 — dois purificadores. Recebido via TED no BNB em 05/10/2026 — lançado em "Out 2026".</t>
+      <c r="G142" s="82" t="inlineStr">
+        <is>
+          <t>Troca do dia 02/09/2026 — 1º Andar, Térreo e Copa. Recebido via Pix em 08/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="143" s="157">
       <c r="A143" s="78" t="inlineStr">
         <is>
-          <t>J Diesel Motores e Reparos - Gilmara</t>
+          <t>Cecilio Mota Junior</t>
         </is>
       </c>
       <c r="B143" s="78" t="inlineStr">
@@ -71908,7 +71908,7 @@
         </is>
       </c>
       <c r="C143" s="77" t="n">
-        <v>46276</v>
+        <v>46267</v>
       </c>
       <c r="D143" s="79" t="n">
         <v>140</v>
@@ -71924,14 +71924,14 @@
       </c>
       <c r="G143" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 11/09/2026.</t>
+          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="144" s="157">
       <c r="A144" s="78" t="inlineStr">
         <is>
-          <t>IOB</t>
+          <t>Tereza Cristina Aquino Martins - Luiz Augusto</t>
         </is>
       </c>
       <c r="B144" s="78" t="inlineStr">
@@ -71940,7 +71940,7 @@
         </is>
       </c>
       <c r="C144" s="77" t="n">
-        <v>46279</v>
+        <v>46268</v>
       </c>
       <c r="D144" s="79" t="n">
         <v>200</v>
@@ -71956,26 +71956,26 @@
       </c>
       <c r="G144" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 14/09/2026.</t>
+          <t>Recebido via Pix em 04/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="145" s="157">
       <c r="A145" s="78" t="inlineStr">
         <is>
-          <t>Clínica Santa Cecília</t>
+          <t>Samille Fiscina Lima Lordello - Tiago (Cartório)</t>
         </is>
       </c>
       <c r="B145" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Termostato</t>
+          <t>Refil Pro Life</t>
         </is>
       </c>
       <c r="C145" s="77" t="n">
-        <v>46281</v>
+        <v>46269</v>
       </c>
       <c r="D145" s="79" t="n">
-        <v>310</v>
+        <v>140</v>
       </c>
       <c r="E145" s="112" t="inlineStr">
         <is>
@@ -71988,26 +71988,26 @@
       </c>
       <c r="G145" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 16/09/2026 — refil + troca de termostato. Recebido via Pix em 29/09/2026.</t>
+          <t>Recebido via Pix em 10/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="146" s="157">
       <c r="A146" s="78" t="inlineStr">
         <is>
-          <t>Marilda Macedo / José Luciano Costa</t>
+          <t>Bomboniere Doce Mania - Veronildo Basilio</t>
         </is>
       </c>
       <c r="B146" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Pré Filtro</t>
+          <t>Refil Plissado + Refil BAG</t>
         </is>
       </c>
       <c r="C146" s="77" t="n">
-        <v>46283</v>
+        <v>46274</v>
       </c>
       <c r="D146" s="79" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="E146" s="112" t="inlineStr">
         <is>
@@ -72020,14 +72020,14 @@
       </c>
       <c r="G146" s="78" t="inlineStr">
         <is>
-          <t>Recebido via Pix em 19/09/2026 — lançado em "Set 2026".</t>
+          <t>Recebido em dinheiro em 16/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="147" s="157">
       <c r="A147" s="78" t="inlineStr">
         <is>
-          <t>Tatiana Rocha</t>
+          <t>Adriadne (Hotel Jovem Jota)</t>
         </is>
       </c>
       <c r="B147" s="78" t="inlineStr">
@@ -72036,7 +72036,7 @@
         </is>
       </c>
       <c r="C147" s="77" t="n">
-        <v>46286</v>
+        <v>46275</v>
       </c>
       <c r="D147" s="79" t="n">
         <v>140</v>
@@ -72052,26 +72052,26 @@
       </c>
       <c r="G147" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 21/09/2026. Recebido via Pix em 22/09/2026 — lançado em "Set 2026".</t>
+          <t>Recebido via Pix em 11/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="148" s="157">
       <c r="A148" s="78" t="inlineStr">
         <is>
-          <t>Cleone Gomes de Andrade</t>
+          <t>Pousada Triunfo Ltda (Hotel Triunfo)</t>
         </is>
       </c>
       <c r="B148" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Refil Everest + Pré Filtro</t>
         </is>
       </c>
       <c r="C148" s="77" t="n">
-        <v>46286</v>
+        <v>46275</v>
       </c>
       <c r="D148" s="79" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="E148" s="112" t="inlineStr">
         <is>
@@ -72084,30 +72084,30 @@
       </c>
       <c r="G148" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 21/09/2026. Recebido via Pix em 21/09/2026.</t>
+          <t>Recebido via Pix em 11/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="149" s="157">
       <c r="A149" s="78" t="inlineStr">
         <is>
-          <t>Centro de Especialidades Odontomédicas</t>
+          <t>Topvel Tropical Veiculos e Pecas</t>
         </is>
       </c>
       <c r="B149" s="78" t="inlineStr">
         <is>
-          <t>2x Refil Everest</t>
+          <t>2x Refil Everest + 2x Pré Filtro</t>
         </is>
       </c>
       <c r="C149" s="77" t="n">
-        <v>46044</v>
+        <v>46276</v>
       </c>
       <c r="D149" s="79" t="n">
-        <v>280</v>
+        <v>370</v>
       </c>
       <c r="E149" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F149" s="112">
@@ -72116,30 +72116,30 @@
       </c>
       <c r="G149" s="78" t="inlineStr">
         <is>
-          <t>NF-e 4039 de 22/01/2026 (CNPJ 54.747.945/0001-09). Venda anterior ao controle manual (aba Jan 2026 vem do Livro Caixa). Conferido no DigiSat em 28/09/2026: não recebido. Mesmo cliente tem outra pendência de 05/08/2026 (R$ 140,00).</t>
+          <t>Troca do dia 11/09/2026 — dois purificadores. Recebido via TED no BNB em 05/10/2026 — lançado em "Out 2026".</t>
         </is>
       </c>
     </row>
     <row r="150" s="157">
       <c r="A150" s="78" t="inlineStr">
         <is>
-          <t>Igreja Messiânica Mundial do Brasil</t>
+          <t>J Diesel Motores e Reparos - Gilmara</t>
         </is>
       </c>
       <c r="B150" s="78" t="inlineStr">
         <is>
-          <t>Mangueira</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C150" s="77" t="n">
-        <v>46073</v>
+        <v>46276</v>
       </c>
       <c r="D150" s="79" t="n">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="E150" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F150" s="112">
@@ -72148,30 +72148,30 @@
       </c>
       <c r="G150" s="78" t="inlineStr">
         <is>
-          <t>NF-e 4075 de 20/02/2026 (CNPJ 62.647.383/0063-44). Conferido no DigiSat em 28/09/2026: não recebido.</t>
+          <t>Troca do dia 11/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="151" s="157">
       <c r="A151" s="78" t="inlineStr">
         <is>
-          <t>Centro Médico de Jacobina</t>
+          <t>IOB</t>
         </is>
       </c>
       <c r="B151" s="78" t="inlineStr">
         <is>
-          <t>2x Botão Completo</t>
+          <t>Refil Everest + Pré Filtro</t>
         </is>
       </c>
       <c r="C151" s="77" t="n">
-        <v>46203</v>
+        <v>46279</v>
       </c>
       <c r="D151" s="79" t="n">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="E151" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F151" s="112">
@@ -72180,26 +72180,26 @@
       </c>
       <c r="G151" s="78" t="inlineStr">
         <is>
-          <t>NF-e 4242 de 30/06/2026 (CNPJ 13.228.432/0001-04). Conferido no DigiSat em 28/09/2026: não recebido.</t>
+          <t>Troca do dia 14/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="152" s="157">
       <c r="A152" s="78" t="inlineStr">
         <is>
-          <t>Vivencie Turismo Agencia de Viagens - Aneildes Rios</t>
+          <t>Clínica Santa Cecília</t>
         </is>
       </c>
       <c r="B152" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Refil Everest + Termostato</t>
         </is>
       </c>
       <c r="C152" s="77" t="n">
-        <v>46294</v>
+        <v>46281</v>
       </c>
       <c r="D152" s="79" t="n">
-        <v>140</v>
+        <v>310</v>
       </c>
       <c r="E152" s="112" t="inlineStr">
         <is>
@@ -72212,26 +72212,26 @@
       </c>
       <c r="G152" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 29/09/2026. Recebido via Pix em 05/10/2026 — R$ 135,00 (Pix único de R$ 270,00 com as duas trocas; R$ 10,00 de desconto dividido).</t>
+          <t>Troca do dia 16/09/2026 — refil + troca de termostato. Recebido via Pix em 29/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="153" s="157">
       <c r="A153" s="78" t="inlineStr">
         <is>
-          <t>Lapec</t>
+          <t>Marilda Macedo / José Luciano Costa</t>
         </is>
       </c>
       <c r="B153" s="78" t="inlineStr">
         <is>
-          <t>Refil C+3</t>
+          <t>Refil Everest + Pré Filtro</t>
         </is>
       </c>
       <c r="C153" s="77" t="n">
-        <v>46294</v>
+        <v>46283</v>
       </c>
       <c r="D153" s="79" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E153" s="112" t="inlineStr">
         <is>
@@ -72244,14 +72244,14 @@
       </c>
       <c r="G153" s="78" t="inlineStr">
         <is>
-          <t>Pagamento previsto para 30/09/2026. Recebido em dinheiro em 14/10/2026 — lançado em "Set 2026".</t>
+          <t>Recebido via Pix em 19/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="154" s="157">
       <c r="A154" s="78" t="inlineStr">
         <is>
-          <t>PC Jacobina Administradora de Cartões LTDA - Cartão de Todos</t>
+          <t>Tatiana Rocha</t>
         </is>
       </c>
       <c r="B154" s="78" t="inlineStr">
@@ -72260,7 +72260,7 @@
         </is>
       </c>
       <c r="C154" s="77" t="n">
-        <v>46295</v>
+        <v>46286</v>
       </c>
       <c r="D154" s="79" t="n">
         <v>140</v>
@@ -72276,14 +72276,14 @@
       </c>
       <c r="G154" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 30/09/2026. Recebido via Pix em 01/10/2026 (comprovante enviado em 06/10/2026) — lançado em "Out 2026".</t>
+          <t>Troca do dia 21/09/2026. Recebido via Pix em 22/09/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="155" s="157">
       <c r="A155" s="78" t="inlineStr">
         <is>
-          <t>Aneilde Rios de Oliveira</t>
+          <t>Cleone Gomes de Andrade</t>
         </is>
       </c>
       <c r="B155" s="78" t="inlineStr">
@@ -72292,7 +72292,7 @@
         </is>
       </c>
       <c r="C155" s="77" t="n">
-        <v>46296</v>
+        <v>46286</v>
       </c>
       <c r="D155" s="79" t="n">
         <v>140</v>
@@ -72308,30 +72308,30 @@
       </c>
       <c r="G155" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 01/10/2026 (casa, Caeira). Recebido via Pix em 05/10/2026 — R$ 135,00 (Pix único de R$ 270,00 com as duas trocas; R$ 10,00 de desconto dividido).</t>
+          <t>Troca do dia 21/09/2026. Recebido via Pix em 21/09/2026.</t>
         </is>
       </c>
     </row>
     <row r="156" s="157">
       <c r="A156" s="78" t="inlineStr">
         <is>
-          <t>Centro Medico da Chapada Diamantina LTDA</t>
+          <t>Centro de Especialidades Odontomédicas</t>
         </is>
       </c>
       <c r="B156" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life + 2x Botão Completo</t>
+          <t>2x Refil Everest</t>
         </is>
       </c>
       <c r="C156" s="77" t="n">
-        <v>46296</v>
+        <v>46044</v>
       </c>
       <c r="D156" s="79" t="n">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="E156" s="112" t="inlineStr">
         <is>
-          <t>Recebido</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="F156" s="112">
@@ -72340,30 +72340,30 @@
       </c>
       <c r="G156" s="78" t="inlineStr">
         <is>
-          <t>Subsolo — troca do dia 01/10/2026 (refil + 2 botões). Recebido em 05/10/2026 no crédito em 3x (pagamento único de R$ 400,00 pelas duas trocas).</t>
+          <t>NF-e 4039 de 22/01/2026 (CNPJ 54.747.945/0001-09). Venda anterior ao controle manual (aba Jan 2026 vem do Livro Caixa). Conferido no DigiSat em 28/09/2026: não recebido. Mesmo cliente tem outra pendência de 05/08/2026 (R$ 140,00).</t>
         </is>
       </c>
     </row>
     <row r="157" s="157">
       <c r="A157" s="78" t="inlineStr">
         <is>
-          <t>Centro Medico da Chapada Diamantina LTDA</t>
+          <t>Igreja Messiânica Mundial do Brasil</t>
         </is>
       </c>
       <c r="B157" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life + 2x Botão Completo</t>
+          <t>Mangueira</t>
         </is>
       </c>
       <c r="C157" s="77" t="n">
-        <v>46297</v>
+        <v>46073</v>
       </c>
       <c r="D157" s="79" t="n">
-        <v>200</v>
+        <v>30</v>
       </c>
       <c r="E157" s="112" t="inlineStr">
         <is>
-          <t>Recebido</t>
+          <t>Pendente</t>
         </is>
       </c>
       <c r="F157" s="112">
@@ -72372,26 +72372,26 @@
       </c>
       <c r="G157" s="78" t="inlineStr">
         <is>
-          <t>1º Andar — troca do dia 02/10/2026 (refil + 2 botões). Recebido em 05/10/2026 no crédito em 3x (pagamento único de R$ 400,00 pelas duas trocas).</t>
+          <t>NF-e 4075 de 20/02/2026 (CNPJ 62.647.383/0063-44). Conferido no DigiSat em 28/09/2026: não recebido.</t>
         </is>
       </c>
     </row>
     <row r="158" s="157">
       <c r="A158" s="78" t="inlineStr">
         <is>
-          <t>Igreja Messiânica Mundial do Brasil</t>
+          <t>Centro Médico de Jacobina</t>
         </is>
       </c>
       <c r="B158" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>2x Botão Completo</t>
         </is>
       </c>
       <c r="C158" s="77" t="n">
-        <v>46300</v>
+        <v>46203</v>
       </c>
       <c r="D158" s="79" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="E158" s="112" t="inlineStr">
         <is>
@@ -72404,14 +72404,14 @@
       </c>
       <c r="G158" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 05/10/2026. Mesmo cliente tem pendência de 20/02/2026 (Mangueira, R$ 30,00).</t>
+          <t>NF-e 4242 de 30/06/2026 (CNPJ 13.228.432/0001-04). Conferido no DigiSat em 28/09/2026: não recebido.</t>
         </is>
       </c>
     </row>
     <row r="159" s="157">
       <c r="A159" s="78" t="inlineStr">
         <is>
-          <t>Rafael Landin Ribeiro</t>
+          <t>Vivencie Turismo Agencia de Viagens - Aneildes Rios</t>
         </is>
       </c>
       <c r="B159" s="78" t="inlineStr">
@@ -72420,7 +72420,7 @@
         </is>
       </c>
       <c r="C159" s="77" t="n">
-        <v>46304</v>
+        <v>46294</v>
       </c>
       <c r="D159" s="79" t="n">
         <v>140</v>
@@ -72436,30 +72436,30 @@
       </c>
       <c r="G159" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 09/10/2026. Recebido via Pix em 09/10/2026.</t>
+          <t>Troca do dia 29/09/2026. Recebido via Pix em 05/10/2026 — R$ 135,00 (Pix único de R$ 270,00 com as duas trocas; R$ 10,00 de desconto dividido).</t>
         </is>
       </c>
     </row>
     <row r="160" s="157">
       <c r="A160" s="78" t="inlineStr">
         <is>
-          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
+          <t>Lapec</t>
         </is>
       </c>
       <c r="B160" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life + Refil Universal (restante)</t>
+          <t>Refil C+3</t>
         </is>
       </c>
       <c r="C160" s="77" t="n">
-        <v>46304</v>
+        <v>46294</v>
       </c>
       <c r="D160" s="79" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="E160" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F160" s="112">
@@ -72468,30 +72468,30 @@
       </c>
       <c r="G160" s="78" t="inlineStr">
         <is>
-          <t>Venda de R$ 170,00 — R$ 85,00 pagos no débito em 09/10/2026; restante via Pix previsto para 16/10/2026.</t>
+          <t>Pagamento previsto para 30/09/2026. Recebido em dinheiro em 14/10/2026 — lançado em "Set 2026".</t>
         </is>
       </c>
     </row>
     <row r="161" s="157">
       <c r="A161" s="78" t="inlineStr">
         <is>
-          <t>Tropical Motos LTDA</t>
+          <t>PC Jacobina Administradora de Cartões LTDA - Cartão de Todos</t>
         </is>
       </c>
       <c r="B161" s="78" t="inlineStr">
         <is>
-          <t>Refil Pro Life</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C161" s="77" t="n">
-        <v>46304</v>
+        <v>46295</v>
       </c>
       <c r="D161" s="79" t="n">
         <v>140</v>
       </c>
       <c r="E161" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F161" s="112">
@@ -72500,14 +72500,14 @@
       </c>
       <c r="G161" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 09/10/2026 — purificador do andar de cima.</t>
+          <t>Troca do dia 30/09/2026. Recebido via Pix em 01/10/2026 (comprovante enviado em 06/10/2026) — lançado em "Out 2026".</t>
         </is>
       </c>
     </row>
     <row r="162" s="157">
       <c r="A162" s="78" t="inlineStr">
         <is>
-          <t>Casa do Construtor</t>
+          <t>Aneilde Rios de Oliveira</t>
         </is>
       </c>
       <c r="B162" s="78" t="inlineStr">
@@ -72516,7 +72516,7 @@
         </is>
       </c>
       <c r="C162" s="77" t="n">
-        <v>46310</v>
+        <v>46296</v>
       </c>
       <c r="D162" s="79" t="n">
         <v>140</v>
@@ -72532,30 +72532,30 @@
       </c>
       <c r="G162" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 15/10/2026. Recebido via Pix em 21/10/2026.</t>
+          <t>Troca do dia 01/10/2026 (casa, Caeira). Recebido via Pix em 05/10/2026 — R$ 135,00 (Pix único de R$ 270,00 com as duas trocas; R$ 10,00 de desconto dividido).</t>
         </is>
       </c>
     </row>
     <row r="163" s="157">
       <c r="A163" s="78" t="inlineStr">
         <is>
-          <t>Lapec</t>
+          <t>Centro Medico da Chapada Diamantina LTDA</t>
         </is>
       </c>
       <c r="B163" s="78" t="inlineStr">
         <is>
-          <t>Refil E3 + Refil Everest</t>
+          <t>Refil Pro Life + 2x Botão Completo</t>
         </is>
       </c>
       <c r="C163" s="77" t="n">
-        <v>46310</v>
+        <v>46296</v>
       </c>
       <c r="D163" s="79" t="n">
         <v>200</v>
       </c>
       <c r="E163" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F163" s="112">
@@ -72564,26 +72564,26 @@
       </c>
       <c r="G163" s="78" t="inlineStr">
         <is>
-          <t>Compra do dia 15/10/2026 — Refil E3 R$ 80,00 + Refil Everest R$ 120,00.</t>
+          <t>Subsolo — troca do dia 01/10/2026 (refil + 2 botões). Recebido em 05/10/2026 no crédito em 3x (pagamento único de R$ 400,00 pelas duas trocas).</t>
         </is>
       </c>
     </row>
     <row r="164" s="157">
       <c r="A164" s="78" t="inlineStr">
         <is>
-          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
+          <t>Centro Medico da Chapada Diamantina LTDA</t>
         </is>
       </c>
       <c r="B164" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest</t>
+          <t>Refil Pro Life + 2x Botão Completo</t>
         </is>
       </c>
       <c r="C164" s="77" t="n">
-        <v>46310</v>
+        <v>46297</v>
       </c>
       <c r="D164" s="79" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="E164" s="112" t="inlineStr">
         <is>
@@ -72596,26 +72596,26 @@
       </c>
       <c r="G164" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 15/10/2026. Recebido via Pix em 16/10/2026 — lançado em "Out 2026".</t>
+          <t>1º Andar — troca do dia 02/10/2026 (refil + 2 botões). Recebido em 05/10/2026 no crédito em 3x (pagamento único de R$ 400,00 pelas duas trocas).</t>
         </is>
       </c>
     </row>
     <row r="165" s="157">
       <c r="A165" s="78" t="inlineStr">
         <is>
-          <t>Colegio Oasis de Jacobina - Unopar</t>
+          <t>Igreja Messiânica Mundial do Brasil</t>
         </is>
       </c>
       <c r="B165" s="78" t="inlineStr">
         <is>
-          <t>2x Refil Plissado + 2x Carcaça 9"</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C165" s="77" t="n">
-        <v>46305</v>
+        <v>46300</v>
       </c>
       <c r="D165" s="79" t="n">
-        <v>400</v>
+        <v>140</v>
       </c>
       <c r="E165" s="112" t="inlineStr">
         <is>
@@ -72628,26 +72628,26 @@
       </c>
       <c r="G165" s="78" t="inlineStr">
         <is>
-          <t>2x Refil Plissado R$ 80,00 cada + 2x Carcaça 9" R$ 120,00 cada. Cláudio assinou para pagar depois. Falta enviar a NF.</t>
+          <t>Troca do dia 05/10/2026. Mesmo cliente tem pendência de 20/02/2026 (Mangueira, R$ 30,00).</t>
         </is>
       </c>
     </row>
     <row r="166" s="157">
       <c r="A166" s="78" t="inlineStr">
         <is>
-          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+          <t>Rafael Landin Ribeiro</t>
         </is>
       </c>
       <c r="B166" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Pré Filtro (restante)</t>
+          <t>Refil Everest</t>
         </is>
       </c>
       <c r="C166" s="77" t="n">
-        <v>46311</v>
+        <v>46304</v>
       </c>
       <c r="D166" s="79" t="n">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="E166" s="112" t="inlineStr">
         <is>
@@ -72660,26 +72660,26 @@
       </c>
       <c r="G166" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 16/10/2026 — bebedouro da recepção. Venda de R$ 200,00: R$ 140,00 pagos em dinheiro em 16/10/2026; falta R$ 60,00. Recebido em dinheiro em 20/10/2026.</t>
+          <t>Troca do dia 09/10/2026. Recebido via Pix em 09/10/2026.</t>
         </is>
       </c>
     </row>
     <row r="167" s="157">
       <c r="A167" s="78" t="inlineStr">
         <is>
-          <t>Contabilidade Abreu</t>
+          <t>Restaurante Bonzão Bode - Aloisio Queiroz</t>
         </is>
       </c>
       <c r="B167" s="78" t="inlineStr">
         <is>
-          <t>Termostato</t>
+          <t>Refil Pro Life + Refil Universal (restante)</t>
         </is>
       </c>
       <c r="C167" s="77" t="n">
-        <v>46311</v>
+        <v>46304</v>
       </c>
       <c r="D167" s="79" t="n">
-        <v>170</v>
+        <v>85</v>
       </c>
       <c r="E167" s="112" t="inlineStr">
         <is>
@@ -72692,26 +72692,26 @@
       </c>
       <c r="G167" s="78" t="inlineStr">
         <is>
-          <t>Troca de termostato do dia 16/10/2026.</t>
+          <t>Venda de R$ 170,00 — R$ 85,00 pagos no débito em 09/10/2026; restante via Pix previsto para 16/10/2026.</t>
         </is>
       </c>
     </row>
     <row r="168" s="157">
       <c r="A168" s="78" t="inlineStr">
         <is>
-          <t>Studio Malena Lorrane</t>
+          <t>Tropical Motos LTDA</t>
         </is>
       </c>
       <c r="B168" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Pré Filtro (restante)</t>
+          <t>Refil Pro Life</t>
         </is>
       </c>
       <c r="C168" s="77" t="n">
-        <v>46316</v>
+        <v>46304</v>
       </c>
       <c r="D168" s="79" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E168" s="112" t="inlineStr">
         <is>
@@ -72724,14 +72724,14 @@
       </c>
       <c r="G168" s="78" t="inlineStr">
         <is>
-          <t>Troca do dia 21/10/2026. Venda de R$ 190,00; R$ 40,00 pagos com serviço de sobrancelha para a Edilânia. Deve R$ 90,00 do refil + R$ 60,00 do pré-filtro.</t>
+          <t>Troca do dia 09/10/2026 — purificador do andar de cima.</t>
         </is>
       </c>
     </row>
     <row r="169" s="157">
       <c r="A169" s="78" t="inlineStr">
         <is>
-          <t>Marsilia Marmores e Granitos Erelli</t>
+          <t>Casa do Construtor</t>
         </is>
       </c>
       <c r="B169" s="78" t="inlineStr">
@@ -72740,14 +72740,14 @@
         </is>
       </c>
       <c r="C169" s="77" t="n">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="D169" s="79" t="n">
         <v>140</v>
       </c>
       <c r="E169" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F169" s="112">
@@ -72756,23 +72756,23 @@
       </c>
       <c r="G169" s="78" t="inlineStr">
         <is>
-          <t>Venda de 19/10/2026.</t>
+          <t>Troca do dia 15/10/2026. Recebido via Pix em 21/10/2026.</t>
         </is>
       </c>
     </row>
     <row r="170" s="157">
       <c r="A170" s="78" t="inlineStr">
         <is>
-          <t>Banco do Nordeste do Brasil</t>
+          <t>Lapec</t>
         </is>
       </c>
       <c r="B170" s="78" t="inlineStr">
         <is>
-          <t>Refil Everest + Pré Filtro</t>
+          <t>Refil E3 + Refil Everest</t>
         </is>
       </c>
       <c r="C170" s="77" t="n">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="D170" s="79" t="n">
         <v>200</v>
@@ -72788,14 +72788,14 @@
       </c>
       <c r="G170" s="78" t="inlineStr">
         <is>
-          <t>Venda de 20/10/2026.</t>
+          <t>Compra do dia 15/10/2026 — Refil E3 R$ 80,00 + Refil Everest R$ 120,00.</t>
         </is>
       </c>
     </row>
     <row r="171" s="157">
       <c r="A171" s="78" t="inlineStr">
         <is>
-          <t>Magna dos Santos Carneiro Goncalves - Mirna</t>
+          <t>Primeiro Tabelionato de Notas - Tatiana Miranda Siqueira</t>
         </is>
       </c>
       <c r="B171" s="78" t="inlineStr">
@@ -72804,14 +72804,14 @@
         </is>
       </c>
       <c r="C171" s="77" t="n">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="D171" s="79" t="n">
         <v>140</v>
       </c>
       <c r="E171" s="112" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>Recebido</t>
         </is>
       </c>
       <c r="F171" s="112">
@@ -72820,26 +72820,26 @@
       </c>
       <c r="G171" s="78" t="inlineStr">
         <is>
-          <t>Venda de 20/10/2026.</t>
+          <t>Troca do dia 15/10/2026. Recebido via Pix em 16/10/2026 — lançado em "Out 2026".</t>
         </is>
       </c>
     </row>
     <row r="172" s="157">
       <c r="A172" s="78" t="inlineStr">
         <is>
-          <t>Loja da Claro</t>
+          <t>Colegio Oasis de Jacobina - Unopar</t>
         </is>
       </c>
       <c r="B172" s="78" t="inlineStr">
         <is>
-          <t>Refil Lacqua</t>
+          <t>2x Refil Plissado + 2x Carcaça 9"</t>
         </is>
       </c>
       <c r="C172" s="77" t="n">
-        <v>46315</v>
+        <v>46305</v>
       </c>
       <c r="D172" s="79" t="n">
-        <v>80</v>
+        <v>400</v>
       </c>
       <c r="E172" s="112" t="inlineStr">
         <is>
@@ -72852,114 +72852,331 @@
       </c>
       <c r="G172" s="78" t="inlineStr">
         <is>
-          <t>Venda de 20/10/2026.</t>
+          <t>2x Refil Plissado R$ 80,00 cada + 2x Carcaça 9" R$ 120,00 cada. Cláudio assinou para pagar depois. Falta enviar a NF.</t>
         </is>
       </c>
     </row>
     <row r="173" s="157">
-      <c r="A173" s="78" t="n"/>
-      <c r="B173" s="78" t="n"/>
-      <c r="C173" s="77" t="n"/>
-      <c r="D173" s="79" t="n"/>
-      <c r="E173" s="112" t="n"/>
+      <c r="A173" s="78" t="inlineStr">
+        <is>
+          <t>DFLL Serviços Medicos Ltda - ImCardio - Instituto Materno Cardiologico</t>
+        </is>
+      </c>
+      <c r="B173" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro (restante)</t>
+        </is>
+      </c>
+      <c r="C173" s="77" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D173" s="79" t="n">
+        <v>60</v>
+      </c>
+      <c r="E173" s="112" t="inlineStr">
+        <is>
+          <t>Recebido</t>
+        </is>
+      </c>
       <c r="F173" s="112">
         <f>IF(OR($E173="Recebido",$C173=""),"",MAX(0,TODAY()-$C173))</f>
         <v/>
       </c>
-      <c r="G173" s="78" t="n"/>
+      <c r="G173" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 16/10/2026 — bebedouro da recepção. Venda de R$ 200,00: R$ 140,00 pagos em dinheiro em 16/10/2026; falta R$ 60,00. Recebido em dinheiro em 20/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="174" s="157">
-      <c r="A174" s="78" t="n"/>
-      <c r="B174" s="78" t="n"/>
-      <c r="C174" s="77" t="n"/>
-      <c r="D174" s="79" t="n"/>
-      <c r="E174" s="112" t="n"/>
+      <c r="A174" s="78" t="inlineStr">
+        <is>
+          <t>Contabilidade Abreu</t>
+        </is>
+      </c>
+      <c r="B174" s="78" t="inlineStr">
+        <is>
+          <t>Termostato</t>
+        </is>
+      </c>
+      <c r="C174" s="77" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D174" s="79" t="n">
+        <v>170</v>
+      </c>
+      <c r="E174" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
       <c r="F174" s="112">
         <f>IF(OR($E174="Recebido",$C174=""),"",MAX(0,TODAY()-$C174))</f>
         <v/>
       </c>
-      <c r="G174" s="78" t="n"/>
+      <c r="G174" s="78" t="inlineStr">
+        <is>
+          <t>Troca de termostato do dia 16/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="175" s="157">
-      <c r="A175" s="78" t="n"/>
-      <c r="B175" s="78" t="n"/>
-      <c r="C175" s="77" t="n"/>
-      <c r="D175" s="79" t="n"/>
-      <c r="E175" s="112" t="n"/>
+      <c r="A175" s="78" t="inlineStr">
+        <is>
+          <t>Studio Malena Lorrane</t>
+        </is>
+      </c>
+      <c r="B175" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro (restante)</t>
+        </is>
+      </c>
+      <c r="C175" s="77" t="n">
+        <v>46316</v>
+      </c>
+      <c r="D175" s="79" t="n">
+        <v>150</v>
+      </c>
+      <c r="E175" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
       <c r="F175" s="112">
         <f>IF(OR($E175="Recebido",$C175=""),"",MAX(0,TODAY()-$C175))</f>
         <v/>
       </c>
-      <c r="G175" s="78" t="n"/>
+      <c r="G175" s="78" t="inlineStr">
+        <is>
+          <t>Troca do dia 21/10/2026. Venda de R$ 190,00; R$ 40,00 pagos com serviço de sobrancelha para a Edilânia. Deve R$ 90,00 do refil + R$ 60,00 do pré-filtro.</t>
+        </is>
+      </c>
     </row>
     <row r="176" s="157">
-      <c r="A176" s="78" t="n"/>
-      <c r="B176" s="78" t="n"/>
-      <c r="C176" s="77" t="n"/>
-      <c r="D176" s="79" t="n"/>
-      <c r="E176" s="112" t="n"/>
+      <c r="A176" s="78" t="inlineStr">
+        <is>
+          <t>Marsilia Marmores e Granitos Erelli</t>
+        </is>
+      </c>
+      <c r="B176" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="C176" s="77" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D176" s="79" t="n">
+        <v>140</v>
+      </c>
+      <c r="E176" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
       <c r="F176" s="112">
         <f>IF(OR($E176="Recebido",$C176=""),"",MAX(0,TODAY()-$C176))</f>
         <v/>
       </c>
-      <c r="G176" s="78" t="n"/>
+      <c r="G176" s="78" t="inlineStr">
+        <is>
+          <t>Venda de 19/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="177" s="157">
-      <c r="A177" s="78" t="n"/>
-      <c r="B177" s="78" t="n"/>
-      <c r="C177" s="77" t="n"/>
-      <c r="D177" s="79" t="n"/>
-      <c r="E177" s="112" t="n"/>
+      <c r="A177" s="78" t="inlineStr">
+        <is>
+          <t>Banco do Nordeste do Brasil</t>
+        </is>
+      </c>
+      <c r="B177" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest + Pré Filtro</t>
+        </is>
+      </c>
+      <c r="C177" s="77" t="n">
+        <v>46315</v>
+      </c>
+      <c r="D177" s="79" t="n">
+        <v>200</v>
+      </c>
+      <c r="E177" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
       <c r="F177" s="112">
         <f>IF(OR($E177="Recebido",$C177=""),"",MAX(0,TODAY()-$C177))</f>
         <v/>
       </c>
-      <c r="G177" s="78" t="n"/>
+      <c r="G177" s="78" t="inlineStr">
+        <is>
+          <t>Venda de 20/10/2026.</t>
+        </is>
+      </c>
     </row>
     <row r="178" s="157">
-      <c r="A178" s="86" t="inlineStr">
+      <c r="A178" s="78" t="inlineStr">
+        <is>
+          <t>Magna dos Santos Carneiro Goncalves - Mirna</t>
+        </is>
+      </c>
+      <c r="B178" s="78" t="inlineStr">
+        <is>
+          <t>Refil Everest</t>
+        </is>
+      </c>
+      <c r="C178" s="77" t="n">
+        <v>46315</v>
+      </c>
+      <c r="D178" s="79" t="n">
+        <v>140</v>
+      </c>
+      <c r="E178" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F178" s="112">
+        <f>IF(OR($E178="Recebido",$C178=""),"",MAX(0,TODAY()-$C178))</f>
+        <v/>
+      </c>
+      <c r="G178" s="78" t="inlineStr">
+        <is>
+          <t>Venda de 20/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" s="157">
+      <c r="A179" s="78" t="inlineStr">
+        <is>
+          <t>Loja da Claro</t>
+        </is>
+      </c>
+      <c r="B179" s="78" t="inlineStr">
+        <is>
+          <t>Refil Lacqua</t>
+        </is>
+      </c>
+      <c r="C179" s="77" t="n">
+        <v>46315</v>
+      </c>
+      <c r="D179" s="79" t="n">
+        <v>80</v>
+      </c>
+      <c r="E179" s="112" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="F179" s="112">
+        <f>IF(OR($E179="Recebido",$C179=""),"",MAX(0,TODAY()-$C179))</f>
+        <v/>
+      </c>
+      <c r="G179" s="78" t="inlineStr">
+        <is>
+          <t>Venda de 20/10/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" s="157">
+      <c r="A180" s="78" t="n"/>
+      <c r="B180" s="78" t="n"/>
+      <c r="C180" s="77" t="n"/>
+      <c r="D180" s="79" t="n"/>
+      <c r="E180" s="112" t="n"/>
+      <c r="F180" s="112">
+        <f>IF(OR($E180="Recebido",$C180=""),"",MAX(0,TODAY()-$C180))</f>
+        <v/>
+      </c>
+      <c r="G180" s="78" t="n"/>
+    </row>
+    <row r="181" s="157">
+      <c r="A181" s="78" t="n"/>
+      <c r="B181" s="78" t="n"/>
+      <c r="C181" s="77" t="n"/>
+      <c r="D181" s="79" t="n"/>
+      <c r="E181" s="112" t="n"/>
+      <c r="F181" s="112">
+        <f>IF(OR($E181="Recebido",$C181=""),"",MAX(0,TODAY()-$C181))</f>
+        <v/>
+      </c>
+      <c r="G181" s="78" t="n"/>
+    </row>
+    <row r="182" s="157">
+      <c r="A182" s="78" t="n"/>
+      <c r="B182" s="78" t="n"/>
+      <c r="C182" s="77" t="n"/>
+      <c r="D182" s="79" t="n"/>
+      <c r="E182" s="112" t="n"/>
+      <c r="F182" s="112">
+        <f>IF(OR($E182="Recebido",$C182=""),"",MAX(0,TODAY()-$C182))</f>
+        <v/>
+      </c>
+      <c r="G182" s="78" t="n"/>
+    </row>
+    <row r="183" s="157">
+      <c r="A183" s="78" t="n"/>
+      <c r="B183" s="78" t="n"/>
+      <c r="C183" s="77" t="n"/>
+      <c r="D183" s="79" t="n"/>
+      <c r="E183" s="112" t="n"/>
+      <c r="F183" s="112">
+        <f>IF(OR($E183="Recebido",$C183=""),"",MAX(0,TODAY()-$C183))</f>
+        <v/>
+      </c>
+      <c r="G183" s="78" t="n"/>
+    </row>
+    <row r="184" s="157">
+      <c r="A184" s="78" t="n"/>
+      <c r="B184" s="78" t="n"/>
+      <c r="C184" s="77" t="n"/>
+      <c r="D184" s="79" t="n"/>
+      <c r="E184" s="112" t="n"/>
+      <c r="F184" s="112">
+        <f>IF(OR($E184="Recebido",$C184=""),"",MAX(0,TODAY()-$C184))</f>
+        <v/>
+      </c>
+      <c r="G184" s="78" t="n"/>
+    </row>
+    <row r="185" s="157">
+      <c r="A185" s="86" t="inlineStr">
         <is>
           <t>TOTAL EM ABERTO A RECEBER (detalhe)</t>
         </is>
       </c>
-      <c r="D178" s="115">
-        <f>SUMIF(E107:E177,"Pendente",D107:D177)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="179" s="157">
-      <c r="A179" s="202" t="inlineStr">
+      <c r="D185" s="115">
+        <f>SUMIF(E114:E184,"Pendente",D114:D184)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="186" s="157">
+      <c r="A186" s="202" t="inlineStr">
         <is>
           <t>CONFERÊNCIA COM AS ABAS DOS MESES</t>
         </is>
       </c>
-      <c r="B179" s="159" t="n"/>
-      <c r="C179" s="159" t="n"/>
-      <c r="D179" s="159" t="n"/>
-      <c r="E179" s="159" t="n"/>
-      <c r="F179" s="159" t="n"/>
-      <c r="G179" s="160" t="n"/>
-    </row>
-    <row r="180" s="157">
-      <c r="A180" s="203">
-        <f>IF(ROUND(D178-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D178-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="181" s="157">
-      <c r="A181" s="203" t="inlineStr">
+      <c r="B186" s="159" t="n"/>
+      <c r="C186" s="159" t="n"/>
+      <c r="D186" s="159" t="n"/>
+      <c r="E186" s="159" t="n"/>
+      <c r="F186" s="159" t="n"/>
+      <c r="G186" s="160" t="n"/>
+    </row>
+    <row r="187" s="157">
+      <c r="A187" s="203">
+        <f>IF(ROUND(D185-C5,2)=0,"OK — o detalhe acima bate com as vendas marcadas como Aguardando Pagamento nas abas dos meses.","ATENÇÃO: diferença de R$ "&amp;TEXT(ABS(D185-C5),"#,##0.00")&amp;" entre este detalhe e as abas dos meses — alguma venda mudou de status em um lado só.")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="188" s="157">
+      <c r="A188" s="203" t="inlineStr">
         <is>
           <t>As contas a pagar do DigiSat (pendentes até 27/07/2026) foram todas quitadas — confirmado em 19/08/2026. A única dívida em aberto hoje é o Capital de Giro do Banco do Brasil. Lance aqui novos compromissos conforme surgirem.</t>
         </is>
       </c>
     </row>
-    <row r="182" s="157"/>
-    <row r="183" s="157"/>
-    <row r="184" s="157"/>
-    <row r="185" s="157"/>
-    <row r="186" s="157"/>
-    <row r="187" s="157"/>
-    <row r="188" s="157"/>
     <row r="189" s="157"/>
     <row r="190" s="157"/>
     <row r="191" s="157"/>
@@ -72994,24 +73211,24 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A111:G111"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A105:G105"/>
+    <mergeCell ref="A186:G186"/>
     <mergeCell ref="C5:D6"/>
     <mergeCell ref="A5:B6"/>
+    <mergeCell ref="A187:G187"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E5:F6"/>
-    <mergeCell ref="A104:G104"/>
-    <mergeCell ref="A179:G179"/>
-    <mergeCell ref="A180:G180"/>
+    <mergeCell ref="A112:G112"/>
     <mergeCell ref="C4:D4"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E11:E99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E11:E106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Pago,Previsto"</formula1>
     </dataValidation>
-    <dataValidation sqref="E107:E177" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E114:E184" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendente,Recebido"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Atualizacao do painel - 24/10/2026 09:37
</commit_message>
<xml_diff>
--- a/Relatorio_Financeiro_2026.xlsx
+++ b/Relatorio_Financeiro_2026.xlsx
@@ -58184,15 +58184,40 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="44" t="n"/>
-      <c r="B166" s="45" t="n"/>
-      <c r="C166" s="45" t="n"/>
-      <c r="D166" s="46" t="n"/>
-      <c r="E166" s="45" t="n"/>
+      <c r="A166" s="44" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B166" s="45" t="inlineStr">
+        <is>
+          <t>Condominio Ilha do Ouro</t>
+        </is>
+      </c>
+      <c r="C166" s="45" t="inlineStr">
+        <is>
+          <t>2x Refil Everest</t>
+        </is>
+      </c>
+      <c r="D166" s="46" t="n">
+        <v>280</v>
+      </c>
+      <c r="E166" s="45" t="inlineStr">
+        <is>
+          <t>Pix</t>
+        </is>
+      </c>
       <c r="F166" s="47" t="n"/>
       <c r="G166" s="48" t="n"/>
       <c r="H166" s="49" t="n"/>
-      <c r="I166" s="45" t="n"/>
+      <c r="I166" s="45" t="inlineStr">
+        <is>
+          <t>Só compra dos refis — sem troca de refil</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>EMP-0085</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="17" t="n"/>

</xml_diff>